<commit_message>
Add ranking data for 2026-03-02
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -43,6 +43,7 @@
     <sheet name="2026-02-09" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="2026-02-16" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="2026-02-23" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="2026-03-02" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -30567,22 +30568,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>ワンパンマン</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>221撃目</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>異種族レビュアーズ</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>天原(原作) masha(作画)</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第90話</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第36話：クソガキ③</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第７４話『半球停止』③</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第７４話　黒板アートの戦いが始まった（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第38話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>いとこのこ</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>いぬちく(著者)</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第46話</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第83話その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第6話</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>このヒーラー、めんどくさい</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>丹念に発酵(著者)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第94話：審査</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第19話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第５７話　和解する器用貧乏（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第90話　初体験(はじめて)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第14話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>不純な彼女達は懺悔しない</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>ポロロッカ(著者)</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第35話</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第139話　イリスVS.フレイ・前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第133話　王都に戻ってみるⅡ（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第317話</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第29話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>まんきつしたい常連さん</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>しんみりん(著者)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第53話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第36話</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>重大告知！</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第42話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第２７食　コカトリスのフライドチキン、パクパクですわ！（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第78話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第37話 独身貴族は新しい喫茶店に呼ばれる（2）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第3話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>モリタ Ｕ４ nima</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第15話（２）　お嬢様と宰相と、とびきりの滋養食（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第61話②　期間限定イベントに参加してみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>勇者の元仲間夫婦は田舎でのんびり幸せに暮らす</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>薊マスラオ(漫画) 相野仁(原作) nima(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>骸骨騎士様、只今異世界へお出掛け中</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>サワノアキラ（漫画） 秤猿鬼（原作） KeG（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第66話　エルフ族の決断Ⅴ</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>拷問171</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>聖者無双</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第96話　戦闘準備・消えた魔物の死体②</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第148話 よくわからないけれど海難事故が起こったようです（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 林たかあき</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第64話 十字傷</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>お気楽領主の楽しい領地防衛 ～生産系魔術で名もなき村を最強の城塞都市に～</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>青色まろ（漫画） 赤池宗（原作） 転（原作イラスト）</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第37話　初めての戦争（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>KAKERU</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第73話「弓王2」（後半）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>小林さんちのメイドラゴン</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>クール教信者</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第160話</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第４５話　エリーゼ、死す（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第85話その4</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>アイドル辞めるけど結婚してくれますか!?</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>三吉汐美(著者)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第21話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>六志麻あさ 業務用餅 kisui</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第８１話</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第81話 テレビドラマ、撮影再開!!</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>遊び人な少女たちは今日も放課後ヤっている</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>逢上おかき(著者)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>EP.24②</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第39話</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第6話-2：聖務のお手伝い</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>ライブダンジョン！</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第94話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>漫画/すたひろ 原作/Y.A</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>chapter80【42話①】</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>空野進 sorani ファルまろ</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第17話　最弱貴族、魔王を住まわせる（２）</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ワンパンマン</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>原作/ＯＮＥ 作画/村田雄介</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>221撃目</t>
+          <t>第132話</t>
         </is>
       </c>
     </row>
@@ -30592,17 +31629,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>異種族レビュアーズ</t>
+          <t>異世界おじさん</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>天原(原作) masha(作画)</t>
+          <t>殆ど死んでいる(著者)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第90話</t>
+          <t>第75話</t>
         </is>
       </c>
     </row>
@@ -30612,17 +31649,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>zunta(作画) はらわたさいぞう(原作)</t>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第36話：クソガキ③</t>
+          <t>第76話 前編</t>
         </is>
       </c>
     </row>
@@ -30632,17 +31669,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>魔術師クノンは見えている</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第７４話『半球停止』③</t>
+          <t>第45話①</t>
         </is>
       </c>
     </row>
@@ -30652,17 +31689,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第７４話　黒板アートの戦いが始まった（１）</t>
+          <t>第７４話『半球停止』④</t>
         </is>
       </c>
     </row>
@@ -30672,17 +31709,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第38話②</t>
+          <t>第21話-1「乙女心」</t>
         </is>
       </c>
     </row>
@@ -30692,17 +31729,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>いとこのこ</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>いぬちく(著者)</t>
+          <t>むちまろ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第46話</t>
+          <t>第146話	ザクザクヘアカット！</t>
         </is>
       </c>
     </row>
@@ -30712,17 +31749,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第83話その2</t>
+          <t>第７４話　黒板アートの戦いが始まった（２）</t>
         </is>
       </c>
     </row>
@@ -30732,17 +31769,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+          <t>クセ強彼女は床にいざなう</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+          <t>須河篤志(著者)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第6話</t>
+          <t>第19話後半</t>
         </is>
       </c>
     </row>
@@ -30752,17 +31789,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>このヒーラー、めんどくさい</t>
+          <t>異世界居酒屋「のぶ」</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>丹念に発酵(著者)</t>
+          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第94話：審査</t>
+          <t>第130話</t>
         </is>
       </c>
     </row>
@@ -30772,17 +31809,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第19話後半</t>
+          <t>第16話-2</t>
         </is>
       </c>
     </row>
@@ -30802,7 +31839,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第５７話　和解する器用貧乏（３）</t>
+          <t>第５７話　和解する器用貧乏（４）</t>
         </is>
       </c>
     </row>
@@ -30812,17 +31849,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+          <t>ダークサモナーとデキている</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>板垣恵介 猪原賽 陸井栄史</t>
+          <t>車王(著者)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第90話　初体験(はじめて)</t>
+          <t>第85話</t>
         </is>
       </c>
     </row>
@@ -30832,17 +31869,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第14話-2</t>
+          <t>おまけ70</t>
         </is>
       </c>
     </row>
@@ -30852,17 +31889,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>不純な彼女達は懺悔しない</t>
+          <t>「おかえり、パパ」</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ポロロッカ(著者)</t>
+          <t>蝉丸</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第35話</t>
+          <t>第33話　対面</t>
         </is>
       </c>
     </row>
@@ -30872,17 +31909,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>食い詰め傭兵の幻想奇譚</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>原作／まいん キャラクター原案／peroshi 漫画／池宮アレア</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第139話　イリスVS.フレイ・前編</t>
+          <t>第29話 前編</t>
         </is>
       </c>
     </row>
@@ -30892,17 +31929,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第133話　王都に戻ってみるⅡ（後編）</t>
+          <t>第4話後編：大聖堂からの来訪者</t>
         </is>
       </c>
     </row>
@@ -30912,17 +31949,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>異世界のんびり農家</t>
+          <t>物語の黒幕に転生して</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第317話</t>
+          <t>第39話</t>
         </is>
       </c>
     </row>
@@ -30932,17 +31969,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>女友達は頼めば意外とヤらせてくれる</t>
+          <t>異世界のんびり農家</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ろくろ(漫画) 鏡遊(原作)</t>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第29話②</t>
+          <t>第318話</t>
         </is>
       </c>
     </row>
@@ -30952,17 +31989,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>まんきつしたい常連さん</t>
+          <t>淫獄団地</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>しんみりん(著者)</t>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第53話後編</t>
+          <t>第55話（前編）</t>
         </is>
       </c>
     </row>
@@ -30972,17 +32009,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第36話</t>
+          <t>第7話-1</t>
         </is>
       </c>
     </row>
@@ -30992,17 +32029,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ダークサモナーとデキている</t>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>車王(著者)</t>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>重大告知！</t>
+          <t>第37話 独身貴族は新しい喫茶店に呼ばれる（3）</t>
         </is>
       </c>
     </row>
@@ -31012,17 +32049,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第42話-2</t>
+          <t>第1話 奇跡のトワ</t>
         </is>
       </c>
     </row>
@@ -31032,17 +32069,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+          <t>剥かせて！竜ケ崎さん</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>島知宏 音速炒飯 有都あらゆる</t>
+          <t>一智和智</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第２７食　コカトリスのフライドチキン、パクパクですわ！（３）</t>
+          <t>大学生編 第18話</t>
         </is>
       </c>
     </row>
@@ -31052,17 +32089,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>アザミヤコを好きになる</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第78話①</t>
+          <t>第14話前編</t>
         </is>
       </c>
     </row>
@@ -31072,17 +32109,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+          <t>貞操逆転世界の童貞辺境領主騎士</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+          <t>柳瀬こたつ（漫画） 道造（原作） めろん２２（キャラクター原案）</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第37話 独身貴族は新しい喫茶店に呼ばれる（2）</t>
+          <t>第12話前半　神の館</t>
         </is>
       </c>
     </row>
@@ -31102,7 +32139,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第3話②</t>
+          <t>第3話③</t>
         </is>
       </c>
     </row>
@@ -31112,17 +32149,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+          <t>美人女上司滝沢さん</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>モリタ Ｕ４ nima</t>
+          <t>やんBARU(著者)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第15話（２）　お嬢様と宰相と、とびきりの滋養食（２）</t>
+          <t>第214話</t>
         </is>
       </c>
     </row>
@@ -31132,17 +32169,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第61話②　期間限定イベントに参加してみた</t>
+          <t>第51話 手紙の山と商会員①</t>
         </is>
       </c>
     </row>
@@ -31152,17 +32189,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>勇者の元仲間夫婦は田舎でのんびり幸せに暮らす</t>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>薊マスラオ(漫画) 相野仁(原作) nima(キャラクター原案)</t>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>5周年の休載イラスト＋懐かしい話</t>
         </is>
       </c>
     </row>
@@ -31172,17 +32209,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>骸骨騎士様、只今異世界へお出掛け中</t>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>サワノアキラ（漫画） 秤猿鬼（原作） KeG（キャラクター原案）</t>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第66話　エルフ族の決断Ⅴ</t>
+          <t>第12話-1：行き止まりの先</t>
         </is>
       </c>
     </row>
@@ -31192,17 +32229,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>拷問171</t>
+          <t>第7話後編</t>
         </is>
       </c>
     </row>
@@ -31212,17 +32249,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>聖者無双</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第96話　戦闘準備・消えた魔物の死体②</t>
+          <t>第62話①　故郷につれ出してみた</t>
         </is>
       </c>
     </row>
@@ -31232,17 +32269,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第148話 よくわからないけれど海難事故が起こったようです（２）</t>
+          <t>第29話</t>
         </is>
       </c>
     </row>
@@ -31252,17 +32289,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>板垣恵介 林たかあき</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第64話 十字傷</t>
+          <t>第149話 よくわからないけれど救助するみたいです（１）</t>
         </is>
       </c>
     </row>
@@ -31272,17 +32309,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>お気楽領主の楽しい領地防衛 ～生産系魔術で名もなき村を最強の城塞都市に～</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>青色まろ（漫画） 赤池宗（原作） 転（原作イラスト）</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第37話　初めての戦争（後編）</t>
+          <t>第４５話　エリーゼ、死す（４）</t>
         </is>
       </c>
     </row>
@@ -31292,17 +32329,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+          <t>英雄王、武を極めるため転生す ～そして、世界最強の見習い騎士♀～</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>KAKERU</t>
+          <t>漫画‥くろむら基人 原作‥ハヤケン キャラクター原案‥Nagu</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第73話「弓王2」（後半）</t>
+          <t>第33話 前編</t>
         </is>
       </c>
     </row>
@@ -31312,17 +32349,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>小林さんちのメイドラゴン</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>クール教信者</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第160話</t>
+          <t>第86話(前編)その1</t>
         </is>
       </c>
     </row>
@@ -31332,17 +32369,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>バーサス</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第４５話　エリーゼ、死す（３）</t>
+          <t>第31話　小粒との対話（2）</t>
         </is>
       </c>
     </row>
@@ -31352,17 +32389,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第85話その4</t>
+          <t>拷問172</t>
         </is>
       </c>
     </row>
@@ -31372,17 +32409,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>アイドル辞めるけど結婚してくれますか!?</t>
+          <t>くらいあの子としたいこと</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>三吉汐美(著者)</t>
+          <t>碇マナツ(著者)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第21話前半</t>
+          <t>第92話</t>
         </is>
       </c>
     </row>
@@ -31392,17 +32429,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>六志麻あさ 業務用餅 kisui</t>
+          <t>原作:剃り残し 漫画:大窪太一</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第８１話</t>
+          <t>第3話</t>
         </is>
       </c>
     </row>
@@ -31412,17 +32449,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+          <t>はぐはぐ(著者)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第81話 テレビドラマ、撮影再開!!</t>
+          <t>第94話</t>
         </is>
       </c>
     </row>
@@ -31432,17 +32469,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>遊び人な少女たちは今日も放課後ヤっている</t>
+          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>逢上おかき(著者)</t>
+          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>第8話②「1st ハイスクール・イベント」</t>
         </is>
       </c>
     </row>
@@ -31452,17 +32489,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>EP.24②</t>
+          <t>第22話④</t>
         </is>
       </c>
     </row>
@@ -31472,17 +32509,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
+          <t>魔王になったので、ダンジョン造って人外娘とほのぼのする</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
+          <t>遠野ノオト(作画) 流優(原作) だぶ竜(キャラクター原案)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第39話</t>
+          <t>第87話後半</t>
         </is>
       </c>
     </row>
@@ -31492,17 +32529,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+          <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第6話-2：聖務のお手伝い</t>
+          <t>第17話　最弱貴族、魔王を住まわせる（３）</t>
         </is>
       </c>
     </row>
@@ -31512,17 +32549,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ライブダンジョン！</t>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+          <t>セレビィ量産型(著者)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第94話前半</t>
+          <t>第25話後半</t>
         </is>
       </c>
     </row>
@@ -31532,17 +32569,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+          <t>異世界でも無難に生きたい症候群</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>漫画/すたひろ 原作/Y.A</t>
+          <t>原作：安泰（一二三書房刊） 漫画：笹峰コウ キャラクター原案：ひたきゆう</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>chapter80【42話①】</t>
+          <t>第34話②</t>
         </is>
       </c>
     </row>
@@ -31552,17 +32589,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+          <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>空野進 sorani ファルまろ</t>
+          <t>岡沢六十四 るれくちぇ sage・ジョー</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第17話　最弱貴族、魔王を住まわせる（２）</t>
+          <t>第78話(前編) 最強の親子</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-03-09
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -44,6 +44,7 @@
     <sheet name="2026-02-16" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="2026-02-23" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="2026-03-02" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="2026-03-09" sheetId="39" state="visible" r:id="rId39"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -31604,22 +31605,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第132話</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>異世界おじさん</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>殆ど死んでいる(著者)</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第75話</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第76話 前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第45話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第７４話『半球停止』④</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第21話-1「乙女心」</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第146話	ザクザクヘアカット！</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第７４話　黒板アートの戦いが始まった（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第19話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>異世界居酒屋「のぶ」</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第130話</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第16話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第５７話　和解する器用貧乏（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第85話</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>おまけ70</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>「おかえり、パパ」</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>蝉丸</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第33話　対面</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>食い詰め傭兵の幻想奇譚</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>原作／まいん キャラクター原案／peroshi 漫画／池宮アレア</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第29話 前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第4話後編：大聖堂からの来訪者</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>物語の黒幕に転生して</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第39話</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第318話</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>淫獄団地</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第55話（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第7話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第37話 独身貴族は新しい喫茶店に呼ばれる（3）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第1話 奇跡のトワ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>剥かせて！竜ケ崎さん</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>一智和智</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>大学生編 第18話</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>アザミヤコを好きになる</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第14話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界の童貞辺境領主騎士</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>柳瀬こたつ（漫画） 道造（原作） めろん２２（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第12話前半　神の館</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第3話③</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>美人女上司滝沢さん</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>やんBARU(著者)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第214話</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第51話 手紙の山と商会員①</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>5周年の休載イラスト＋懐かしい話</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第12話-1：行き止まりの先</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第7話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第62話①　故郷につれ出してみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第29話</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第149話 よくわからないけれど救助するみたいです（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第４５話　エリーゼ、死す（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>英雄王、武を極めるため転生す ～そして、世界最強の見習い騎士♀～</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>漫画‥くろむら基人 原作‥ハヤケン キャラクター原案‥Nagu</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第33話 前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第86話(前編)その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>バーサス</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第31話　小粒との対話（2）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>拷問172</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第92話</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>原作:剃り残し 漫画:大窪太一</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第3話</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>はぐはぐ(著者)</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第94話</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第8話②「1st ハイスクール・イベント」</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第22話④</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>魔王になったので、ダンジョン造って人外娘とほのぼのする</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>遠野ノオト(作画) 流優(原作) だぶ竜(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第87話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>空野進 sorani ファルまろ</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第17話　最弱貴族、魔王を住まわせる（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第25話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>異世界でも無難に生きたい症候群</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>原作：安泰（一二三書房刊） 漫画：笹峰コウ キャラクター原案：ひたきゆう</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第34話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>岡沢六十四 るれくちぇ sage・ジョー</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第78話(前編) 最強の親子</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>宇崎ちゃんは遊びたい！</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>丈(著者)</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第132話</t>
+          <t>222撃目</t>
         </is>
       </c>
     </row>
@@ -31629,17 +32666,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>異世界おじさん</t>
+          <t>王子様の友達</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>殆ど死んでいる(著者)</t>
+          <t>すけろく(著者)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第75話</t>
+          <t>第35話</t>
         </is>
       </c>
     </row>
@@ -31649,17 +32686,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+          <t>寿司ガキ</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+          <t>ichika(著者)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第76話 前編</t>
+          <t>第10話</t>
         </is>
       </c>
     </row>
@@ -31669,17 +32706,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>魔術師クノンは見えている</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第45話①</t>
+          <t>第７５話『黒兎停止』</t>
         </is>
       </c>
     </row>
@@ -31689,17 +32726,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第７４話『半球停止』④</t>
+          <t>第７５話　密室ホラーな戦いが始まった（１）</t>
         </is>
       </c>
     </row>
@@ -31709,17 +32746,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第21話-1「乙女心」</t>
+          <t>第84話その1</t>
         </is>
       </c>
     </row>
@@ -31729,17 +32766,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>いとこのこ</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>いぬちく(著者)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第146話	ザクザクヘアカット！</t>
+          <t>特別編7（かーうち先生、しゅる版先生、大川ぶくぶ先生、肉丸先生、肉村Q先生、ぎんもく先生）</t>
         </is>
       </c>
     </row>
@@ -31749,17 +32786,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>帰ってください！ 阿久津さん</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>長岡太一(著者)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第７４話　黒板アートの戦いが始まった（２）</t>
+          <t>第202話</t>
         </is>
       </c>
     </row>
@@ -31769,17 +32806,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第19話後半</t>
+          <t>特別編</t>
         </is>
       </c>
     </row>
@@ -31789,17 +32826,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>異世界居酒屋「のぶ」</t>
+          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
+          <t>久遠まこと(著者) 石のやっさん(原作)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第130話</t>
+          <t>第35話</t>
         </is>
       </c>
     </row>
@@ -31809,17 +32846,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第16話-2</t>
+          <t>第20話前半</t>
         </is>
       </c>
     </row>
@@ -31829,17 +32866,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第５７話　和解する器用貧乏（４）</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -31849,17 +32886,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ダークサモナーとデキている</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>車王(著者)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第85話</t>
+          <t>第５８話　真相を知った器用貧乏（１）</t>
         </is>
       </c>
     </row>
@@ -31879,7 +32916,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>おまけ70</t>
+          <t>第139話　イリスVS.フレイ・後編</t>
         </is>
       </c>
     </row>
@@ -31889,17 +32926,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>「おかえり、パパ」</t>
+          <t>このヒーラー、めんどくさい</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>蝉丸</t>
+          <t>丹念に発酵(著者)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第33話　対面</t>
+          <t>第95話：演技</t>
         </is>
       </c>
     </row>
@@ -31909,17 +32946,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>食い詰め傭兵の幻想奇譚</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>原作／まいん キャラクター原案／peroshi 漫画／池宮アレア</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第29話 前編</t>
+          <t>第134話　王都炎上Ⅰ（前編）</t>
         </is>
       </c>
     </row>
@@ -31929,17 +32966,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第4話後編：大聖堂からの来訪者</t>
+          <t>第91話　大地を揺らす者</t>
         </is>
       </c>
     </row>
@@ -31949,17 +32986,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>物語の黒幕に転生して</t>
+          <t>まんきつしたい常連さん</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
+          <t>しんみりん(著者)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第39話</t>
+          <t>第54話前編</t>
         </is>
       </c>
     </row>
@@ -31969,17 +33006,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>異世界のんびり農家</t>
+          <t>田舎で恋は難しい!?</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+          <t>ねこうめ(著者)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第318話</t>
+          <t>第5話</t>
         </is>
       </c>
     </row>
@@ -31989,17 +33026,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>淫獄団地</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第55話（前編）</t>
+          <t>第78話➁</t>
         </is>
       </c>
     </row>
@@ -32009,17 +33046,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>三部べべ(漫画) ねうしとら(原作)</t>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第7話-1</t>
+          <t>第37話 独身貴族は新しい喫茶店に呼ばれる（4）</t>
         </is>
       </c>
     </row>
@@ -32029,17 +33066,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+          <t>モリタ Ｕ４ nima</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第37話 独身貴族は新しい喫茶店に呼ばれる（3）</t>
+          <t>第15話（３）　お嬢様と宰相と、とびきりの滋養食（３）</t>
         </is>
       </c>
     </row>
@@ -32049,17 +33086,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第1話 奇跡のトワ</t>
+          <t>第62話②　故郷につれ出してみた</t>
         </is>
       </c>
     </row>
@@ -32069,17 +33106,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>剥かせて！竜ケ崎さん</t>
+          <t>濁る瞳で何を願う ハイセルク戦記</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>一智和智</t>
+          <t>トルトネン 創-taro 斎藤八呑</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>大学生編 第18話</t>
+          <t>第38話 泥濘にて泳ぐ</t>
         </is>
       </c>
     </row>
@@ -32089,17 +33126,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>アザミヤコを好きになる</t>
+          <t>異世界食堂　洋食のねこや</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第14話前編</t>
+          <t>第45話➁</t>
         </is>
       </c>
     </row>
@@ -32109,17 +33146,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>貞操逆転世界の童貞辺境領主騎士</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>柳瀬こたつ（漫画） 道造（原作） めろん２２（キャラクター原案）</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第12話前半　神の館</t>
+          <t>第149話 よくわからないけれど救助するみたいです（２）</t>
         </is>
       </c>
     </row>
@@ -32129,17 +33166,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>板垣恵介 林たかあき</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第3話③</t>
+          <t>第65話 返り咲き</t>
         </is>
       </c>
     </row>
@@ -32149,17 +33186,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>美人女上司滝沢さん</t>
+          <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>やんBARU(著者)</t>
+          <t>クール教信者</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第214話</t>
+          <t>第161話</t>
         </is>
       </c>
     </row>
@@ -32169,17 +33206,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第51話 手紙の山と商会員①</t>
+          <t>第30話①</t>
         </is>
       </c>
     </row>
@@ -32189,17 +33226,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+          <t>ダークサモナーとデキている</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+          <t>車王(著者)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>5周年の休載イラスト＋懐かしい話</t>
+          <t>コミックス告知</t>
         </is>
       </c>
     </row>
@@ -32209,17 +33246,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第12話-1：行き止まりの先</t>
+          <t>第４５話　エリーゼ、死す（５）</t>
         </is>
       </c>
     </row>
@@ -32229,17 +33266,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第7話後編</t>
+          <t>第86話(前編)その2</t>
         </is>
       </c>
     </row>
@@ -32249,17 +33286,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第62話①　故郷につれ出してみた</t>
+          <t>拷問173</t>
         </is>
       </c>
     </row>
@@ -32269,17 +33306,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
+          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
+          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第29話</t>
+          <t>第44話-2</t>
         </is>
       </c>
     </row>
@@ -32289,17 +33326,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>アイドル辞めるけど結婚してくれますか!?</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>三吉汐美(著者)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第149話 よくわからないけれど救助するみたいです（１）</t>
+          <t>第21話後半</t>
         </is>
       </c>
     </row>
@@ -32309,17 +33346,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>六志麻あさ 業務用餅 kisui</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第４５話　エリーゼ、死す（４）</t>
+          <t>第８２話</t>
         </is>
       </c>
     </row>
@@ -32329,17 +33366,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>英雄王、武を極めるため転生す ～そして、世界最強の見習い騎士♀～</t>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>漫画‥くろむら基人 原作‥ハヤケン キャラクター原案‥Nagu</t>
+          <t>KAKERU</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第33話 前編</t>
+          <t>第74話「弓王3」（前半）</t>
         </is>
       </c>
     </row>
@@ -32349,17 +33386,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第86話(前編)その1</t>
+          <t>第62話　潰</t>
         </is>
       </c>
     </row>
@@ -32369,17 +33406,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>バーサス</t>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第31話　小粒との対話（2）</t>
+          <t>第82話 ラオウとトキ、意外な関係!!</t>
         </is>
       </c>
     </row>
@@ -32389,17 +33426,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>おせっかい女子、恋をする</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>音竹 ひかる(著者)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>拷問172</t>
+          <t>第6話</t>
         </is>
       </c>
     </row>
@@ -32409,17 +33446,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>遊び人な少女たちは今日も放課後ヤっている</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>逢上おかき(著者)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第92話</t>
+          <t>第2話</t>
         </is>
       </c>
     </row>
@@ -32429,17 +33466,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+          <t>陰キャの俺が席替えでS級美少女に囲まれたら秘密の関係が始まった。</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>原作:剃り残し 漫画:大窪太一</t>
+          <t>星野 星野(原作) バラマツヒトミ(漫画) 黒兎 ゆう(キャラクター原案)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第3話</t>
+          <t>第11話</t>
         </is>
       </c>
     </row>
@@ -32449,17 +33486,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>サーシャちゃんとクラスメイトオタクくん</t>
+          <t>回復術士のやり直し</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>はぐはぐ(著者)</t>
+          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第94話</t>
+          <t>第76話-2</t>
         </is>
       </c>
     </row>
@@ -32469,17 +33506,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第8話②「1st ハイスクール・イベント」</t>
+          <t>第7話-1：暗躍する者たち</t>
         </is>
       </c>
     </row>
@@ -32489,17 +33526,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+          <t>天獄で悪魔がボクを魅惑する</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+          <t>銀河味めてお(著者)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第22話④</t>
+          <t>第39話</t>
         </is>
       </c>
     </row>
@@ -32509,17 +33546,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>魔王になったので、ダンジョン造って人外娘とほのぼのする</t>
+          <t>ライブダンジョン！</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>遠野ノオト(作画) 流優(原作) だぶ竜(キャラクター原案)</t>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第87話後半</t>
+          <t>第94話後半</t>
         </is>
       </c>
     </row>
@@ -32529,17 +33566,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+          <t>お前がヤったんだろ！</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>空野進 sorani ファルまろ</t>
+          <t>クシザキ</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第17話　最弱貴族、魔王を住まわせる（３）</t>
+          <t>第5話	佐倉モモカの昼食</t>
         </is>
       </c>
     </row>
@@ -32549,17 +33586,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>三枝さんはメガネ先輩と恋を描く</t>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>セレビィ量産型(著者)</t>
+          <t>漫画/すたひろ 原作/Y.A</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第25話後半</t>
+          <t>chapter81【42話②】</t>
         </is>
       </c>
     </row>
@@ -32569,17 +33606,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>異世界でも無難に生きたい症候群</t>
+          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>原作：安泰（一二三書房刊） 漫画：笹峰コウ キャラクター原案：ひたきゆう</t>
+          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第34話②</t>
+          <t>第40話</t>
         </is>
       </c>
     </row>
@@ -32589,17 +33626,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>岡沢六十四 るれくちぇ sage・ジョー</t>
+          <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第78話(前編) 最強の親子</t>
+          <t>第18話　最弱貴族、奔走する（１）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-03-16
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -45,6 +45,7 @@
     <sheet name="2026-02-23" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="2026-03-02" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="2026-03-09" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="2026-03-16" sheetId="40" state="visible" r:id="rId40"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -32641,1000 +32642,1000 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>ワンパンマン</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>222撃目</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>王子様の友達</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>すけろく(著者)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>第35話</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>寿司ガキ</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>ichika(著者)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>第10話</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>光永康則</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>第７５話『黒兎停止』</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>マツモトケンゴ</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>第７５話　密室ホラーな戦いが始まった（１）</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="0" t="inlineStr">
         <is>
           <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>第84話その1</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
         <is>
           <t>いとこのこ</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>いぬちく(著者)</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>特別編7（かーうち先生、しゅる版先生、大川ぶくぶ先生、肉丸先生、肉村Q先生、ぎんもく先生）</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>帰ってください！ 阿久津さん</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>長岡太一(著者)</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>第202話</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="0" t="inlineStr">
         <is>
           <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>特別編</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="0" t="inlineStr">
         <is>
           <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>久遠まこと(著者) 石のやっさん(原作)</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>第35話</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>第20話前半</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>第1話</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>第５８話　真相を知った器用貧乏（１）</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>実は俺、最強でした？</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>第139話　イリスVS.フレイ・後編</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>このヒーラー、めんどくさい</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>丹念に発酵(著者)</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>第95話：演技</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>第134話　王都炎上Ⅰ（前編）</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="0" t="inlineStr">
         <is>
           <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>板垣恵介 猪原賽 陸井栄史</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>第91話　大地を揺らす者</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="0" t="inlineStr">
         <is>
           <t>まんきつしたい常連さん</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
         <is>
           <t>しんみりん(著者)</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>第54話前編</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="0" t="inlineStr">
         <is>
           <t>田舎で恋は難しい!?</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="0" t="inlineStr">
         <is>
           <t>ねこうめ(著者)</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>第5話</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="0" t="inlineStr">
         <is>
           <t>リビルドワールド</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>第78話➁</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="0" t="inlineStr">
         <is>
           <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>第37話 独身貴族は新しい喫茶店に呼ばれる（4）</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="0" t="inlineStr">
         <is>
           <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>モリタ Ｕ４ nima</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>第15話（３）　お嬢様と宰相と、とびきりの滋養食（３）</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
+      <c r="A24" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="0" t="inlineStr">
         <is>
           <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>第62話②　故郷につれ出してみた</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
+      <c r="A25" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="0" t="inlineStr">
         <is>
           <t>濁る瞳で何を願う ハイセルク戦記</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>トルトネン 創-taro 斎藤八呑</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>第38話 泥濘にて泳ぐ</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
+      <c r="A26" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="0" t="inlineStr">
         <is>
           <t>異世界食堂　洋食のねこや</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>第45話➁</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="n">
+      <c r="A27" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="0" t="inlineStr">
         <is>
           <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>内々けやき あし カオミン</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>第149話 よくわからないけれど救助するみたいです（２）</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
+      <c r="A28" s="0" t="n">
         <v>27</v>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="0" t="inlineStr">
         <is>
           <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr">
         <is>
           <t>板垣恵介 林たかあき</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t>第65話 返り咲き</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="0" t="inlineStr">
         <is>
           <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>クール教信者</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>第161話</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="n">
+      <c r="A30" s="0" t="n">
         <v>29</v>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="0" t="inlineStr">
         <is>
           <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="0" t="inlineStr">
         <is>
           <t>第30話①</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="0" t="inlineStr">
         <is>
           <t>ダークサモナーとデキている</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>車王(著者)</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>コミックス告知</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="n">
+      <c r="A32" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="0" t="inlineStr">
         <is>
           <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="0" t="inlineStr">
         <is>
           <t>第４５話　エリーゼ、死す（５）</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="n">
+      <c r="A33" s="0" t="n">
         <v>32</v>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="0" t="inlineStr">
         <is>
           <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t>第86話(前編)その2</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
+      <c r="A34" s="0" t="n">
         <v>33</v>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="0" t="inlineStr">
         <is>
           <t>姫様“拷問”の時間です</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="0" t="inlineStr">
         <is>
           <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="0" t="inlineStr">
         <is>
           <t>拷問173</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="n">
+      <c r="A35" s="0" t="n">
         <v>34</v>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="0" t="inlineStr">
         <is>
           <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="0" t="inlineStr">
         <is>
           <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="0" t="inlineStr">
         <is>
           <t>第44話-2</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="n">
+      <c r="A36" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="0" t="inlineStr">
         <is>
           <t>アイドル辞めるけど結婚してくれますか!?</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr">
         <is>
           <t>三吉汐美(著者)</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="0" t="inlineStr">
         <is>
           <t>第21話後半</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="n">
+      <c r="A37" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="0" t="inlineStr">
         <is>
           <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr">
         <is>
           <t>六志麻あさ 業務用餅 kisui</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="0" t="inlineStr">
         <is>
           <t>第８２話</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="n">
+      <c r="A38" s="0" t="n">
         <v>37</v>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="0" t="inlineStr">
         <is>
           <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="0" t="inlineStr">
         <is>
           <t>KAKERU</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="0" t="inlineStr">
         <is>
           <t>第74話「弓王3」（前半）</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="0" t="inlineStr">
         <is>
           <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="0" t="inlineStr">
         <is>
           <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="0" t="inlineStr">
         <is>
           <t>第62話　潰</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
+      <c r="A40" s="0" t="n">
         <v>39</v>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="0" t="inlineStr">
         <is>
           <t>北斗の拳 世紀末ドラマ撮影伝</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="0" t="inlineStr">
         <is>
           <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="0" t="inlineStr">
         <is>
           <t>第82話 ラオウとトキ、意外な関係!!</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="n">
+      <c r="A41" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="0" t="inlineStr">
         <is>
           <t>おせっかい女子、恋をする</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="0" t="inlineStr">
         <is>
           <t>音竹 ひかる(著者)</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="0" t="inlineStr">
         <is>
           <t>第6話</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="n">
+      <c r="A42" s="0" t="n">
         <v>41</v>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="0" t="inlineStr">
         <is>
           <t>遊び人な少女たちは今日も放課後ヤっている</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="0" t="inlineStr">
         <is>
           <t>逢上おかき(著者)</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="0" t="inlineStr">
         <is>
           <t>第2話</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="0" t="inlineStr">
         <is>
           <t>陰キャの俺が席替えでS級美少女に囲まれたら秘密の関係が始まった。</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="0" t="inlineStr">
         <is>
           <t>星野 星野(原作) バラマツヒトミ(漫画) 黒兎 ゆう(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="0" t="inlineStr">
         <is>
           <t>第11話</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="n">
+      <c r="A44" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="0" t="inlineStr">
         <is>
           <t>回復術士のやり直し</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="0" t="inlineStr">
         <is>
           <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="0" t="inlineStr">
         <is>
           <t>第76話-2</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="0" t="inlineStr">
         <is>
           <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="0" t="inlineStr">
         <is>
           <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="0" t="inlineStr">
         <is>
           <t>第7話-1：暗躍する者たち</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
+      <c r="A46" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="0" t="inlineStr">
         <is>
           <t>天獄で悪魔がボクを魅惑する</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
         <is>
           <t>銀河味めてお(著者)</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="0" t="inlineStr">
         <is>
           <t>第39話</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="n">
+      <c r="A47" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="0" t="inlineStr">
         <is>
           <t>ライブダンジョン！</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="0" t="inlineStr">
         <is>
           <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="0" t="inlineStr">
         <is>
           <t>第94話後半</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="n">
+      <c r="A48" s="0" t="n">
         <v>47</v>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="0" t="inlineStr">
         <is>
           <t>お前がヤったんだろ！</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="0" t="inlineStr">
         <is>
           <t>クシザキ</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="0" t="inlineStr">
         <is>
           <t>第5話	佐倉モモカの昼食</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="n">
+      <c r="A49" s="0" t="n">
         <v>48</v>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="0" t="inlineStr">
         <is>
           <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="0" t="inlineStr">
         <is>
           <t>漫画/すたひろ 原作/Y.A</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="0" t="inlineStr">
         <is>
           <t>chapter81【42話②】</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="n">
+      <c r="A50" s="0" t="n">
         <v>49</v>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="0" t="inlineStr">
         <is>
           <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="0" t="inlineStr">
         <is>
           <t>昼行燈（原作） しいたけ元帥（漫画）</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="0" t="inlineStr">
         <is>
           <t>第40話</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="n">
+      <c r="A51" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="0" t="inlineStr">
         <is>
           <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="0" t="inlineStr">
         <is>
           <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="0" t="inlineStr">
         <is>
           <t>第18話　最弱貴族、奔走する（１）</t>
         </is>
@@ -34681,6 +34682,1042 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>第76話 後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>第45話➁</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>不徳のギルド</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>河添太一</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>第１０４話：dskb大作戦</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>第77話</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>第７５話　密室ホラーな戦いが始まった（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>第７５話『黒兎停止』②</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>第147話	着ぐるみありすの災難</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>いとこのこ</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>いぬちく(著者)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>特別編7（かーうち先生、しゅる版先生、大川ぶくぶ先生、肉丸先生、肉村Q先生、ぎんもく先生）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>第8話 前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>第39話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ダンジョンの幼なじみ</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>久真やすひさ(著者)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>第62話</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>第17話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>第20話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>第５８話　真相を知った器用貧乏（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>第140話　ティアの誘い</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>第86話</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>第134話　王都炎上Ⅰ（中編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>魔のものたちは企てる</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>加藤拓弐(原作) ガしガし(作画)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>第35話</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>第15話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>第5話前編：未練</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>不純な彼女達は懺悔しない</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ポロロッカ(著者)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>第36話</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>第7話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>淫獄団地</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>第55話（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>第46話　奴は再会する（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>夜州 nini 藻</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>第73話(前編)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>美人女上司滝沢さん</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>やんBARU(著者)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>第215話</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>第2話 ネトル（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>第４６話　勇者、ラファエルとのRAPバトルでドープな韻のパンチライン＆ディープなリリックはアゲアゲで会場を沸かす（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>【お知らせ】コミックス第9巻、本日発売！</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>第12話-2：行き止まりの先</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>第3話④</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>アザミヤコを好きになる</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>第14話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>理想のヒモ生活</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>第105話　その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>第150話 よくわからないけれど侵略しにきたみたいでゲソ（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>第86話(前編)その3</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>悪友の俺がポンコツ騎士を見てられないんだが、どう世話を焼きゃいい？ ～まどめ外伝～</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>原作：手島史詞 漫画：双葉もも キャラクター原案：COMTA 構成：板垣ハコ</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>第20話</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>第6話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>拷問174</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>第25.5話</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>はぐはぐ(著者)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>第95話</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>コミックス５巻ついに発売!!!</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>原作:剃り残し 漫画:大窪太一</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>第4話</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>第3話(2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>バーサス</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>第32話　蜷局山と…（1）</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>第93話</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>最果てのパラディン</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>奥橋睦（漫画） 柳野かなた（原作） 輪くすさが（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>第70話　無敵の巨人Ⅲ</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>インフィニット・デンドログラム</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>第76話</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>第7話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>異世界でも無難に生きたい症候群</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>原作：安泰（一二三書房刊） 漫画：笹峰コウ キャラクター原案：ひたきゆう</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>【お知らせ】コミックス第7巻、本日発売！</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ディーふらぐ！</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>春野友矢(著者)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>第177話</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add ranking data for 2026-03-23
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -46,6 +46,7 @@
     <sheet name="2026-03-02" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="2026-03-09" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="2026-03-16" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="2026-03-23" sheetId="41" state="visible" r:id="rId41"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -34714,22 +34715,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第76話 後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第45話➁</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>不徳のギルド</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>河添太一</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第１０４話：dskb大作戦</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第77話</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第７５話　密室ホラーな戦いが始まった（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第７５話『黒兎停止』②</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第147話	着ぐるみありすの災難</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>いとこのこ</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>いぬちく(著者)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>特別編7（かーうち先生、しゅる版先生、大川ぶくぶ先生、肉丸先生、肉村Q先生、ぎんもく先生）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第8話 前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第39話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>ダンジョンの幼なじみ</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>久真やすひさ(著者)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第62話</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第17話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第20話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第５８話　真相を知った器用貧乏（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第140話　ティアの誘い</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第86話</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第134話　王都炎上Ⅰ（中編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>魔のものたちは企てる</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>加藤拓弐(原作) ガしガし(作画)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第35話</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第15話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第5話前編：未練</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>不純な彼女達は懺悔しない</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>ポロロッカ(著者)</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第36話</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第7話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>淫獄団地</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第55話（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第46話　奴は再会する（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>夜州 nini 藻</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第73話(前編)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>美人女上司滝沢さん</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>やんBARU(著者)</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第215話</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第2話 ネトル（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第４６話　勇者、ラファエルとのRAPバトルでドープな韻のパンチライン＆ディープなリリックはアゲアゲで会場を沸かす（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>【お知らせ】コミックス第9巻、本日発売！</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第12話-2：行き止まりの先</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第3話④</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>アザミヤコを好きになる</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第14話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>理想のヒモ生活</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第105話　その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第150話 よくわからないけれど侵略しにきたみたいでゲソ（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第86話(前編)その3</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>悪友の俺がポンコツ騎士を見てられないんだが、どう世話を焼きゃいい？ ～まどめ外伝～</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>原作：手島史詞 漫画：双葉もも キャラクター原案：COMTA 構成：板垣ハコ</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第20話</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第6話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>拷問174</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第25.5話</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>はぐはぐ(著者)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第95話</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>コミックス５巻ついに発売!!!</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>原作:剃り残し 漫画:大窪太一</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第4話</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第3話(2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>バーサス</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第32話　蜷局山と…（1）</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第93話</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>最果てのパラディン</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>奥橋睦（漫画） 柳野かなた（原作） 輪くすさが（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第70話　無敵の巨人Ⅲ</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>インフィニット・デンドログラム</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第76話</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第7話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>異世界でも無難に生きたい症候群</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>原作：安泰（一二三書房刊） 漫画：笹峰コウ キャラクター原案：ひたきゆう</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>【お知らせ】コミックス第7巻、本日発売！</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>ディーふらぐ！</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>春野友矢(著者)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第177話</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第76話 後編</t>
+          <t>第133話</t>
         </is>
       </c>
     </row>
@@ -34739,17 +35776,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>魔術師クノンは見えている</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第45話➁</t>
+          <t>223撃目</t>
         </is>
       </c>
     </row>
@@ -34759,17 +35796,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>不徳のギルド</t>
+          <t>異種族レビュアーズ</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>河添太一</t>
+          <t>天原(原作) masha(作画)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第１０４話：dskb大作戦</t>
+          <t>第91話</t>
         </is>
       </c>
     </row>
@@ -34779,17 +35816,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第77話</t>
+          <t>第21話-2「乙女心」</t>
         </is>
       </c>
     </row>
@@ -34799,17 +35836,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第７５話　密室ホラーな戦いが始まった（２）</t>
+          <t>第７５話『黒兎停止』③</t>
         </is>
       </c>
     </row>
@@ -34819,17 +35856,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第７５話『黒兎停止』②</t>
+          <t>第７６話　ホットヨガの戦いが始まった（１）</t>
         </is>
       </c>
     </row>
@@ -34839,17 +35876,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>いとこのこ</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>いぬちく(著者)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第147話	着ぐるみありすの災難</t>
+          <t>第47話</t>
         </is>
       </c>
     </row>
@@ -34859,17 +35896,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>いとこのこ</t>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>いぬちく(著者)</t>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>特別編7（かーうち先生、しゅる版先生、大川ぶくぶ先生、肉丸先生、肉村Q先生、ぎんもく先生）</t>
+          <t>第8話 後編</t>
         </is>
       </c>
     </row>
@@ -34879,17 +35916,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第8話 前編</t>
+          <t>第84話その2</t>
         </is>
       </c>
     </row>
@@ -34899,17 +35936,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+          <t>帰ってください！ 阿久津さん</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+          <t>長岡太一(著者)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第39話①</t>
+          <t>第203話</t>
         </is>
       </c>
     </row>
@@ -34919,17 +35956,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ダンジョンの幼なじみ</t>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>久真やすひさ(著者)</t>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第62話</t>
+          <t>第20話後半</t>
         </is>
       </c>
     </row>
@@ -34939,17 +35976,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第17話-1</t>
+          <t>第7話前半</t>
         </is>
       </c>
     </row>
@@ -34959,17 +35996,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>金属スライムを倒しまくった俺が【黒鋼の王】と呼ばれるまで</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>藤屋いずこ(著者) 温泉カピバラ(原作) 山椒魚(キャラクター原案)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第20話前半</t>
+          <t>第18章-2</t>
         </is>
       </c>
     </row>
@@ -34989,7 +36026,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第５８話　真相を知った器用貧乏（２）</t>
+          <t>第５８話　真相を知った器用貧乏（３）</t>
         </is>
       </c>
     </row>
@@ -35009,7 +36046,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第140話　ティアの誘い</t>
+          <t>第141話　とまどい</t>
         </is>
       </c>
     </row>
@@ -35019,17 +36056,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ダークサモナーとデキている</t>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>車王(著者)</t>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第86話</t>
+          <t>第92話　小細工</t>
         </is>
       </c>
     </row>
@@ -35049,7 +36086,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第134話　王都炎上Ⅰ（中編）</t>
+          <t>第134話　王都炎上Ⅰ（後編）</t>
         </is>
       </c>
     </row>
@@ -35059,17 +36096,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>魔のものたちは企てる</t>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>加藤拓弐(原作) ガしガし(作画)</t>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第35話</t>
+          <t>第37話</t>
         </is>
       </c>
     </row>
@@ -35079,17 +36116,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+          <t>まんきつしたい常連さん</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+          <t>しんみりん(著者)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第15話-2</t>
+          <t>第54話後編</t>
         </is>
       </c>
     </row>
@@ -35099,17 +36136,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第5話前編：未練</t>
+          <t>第43話-2</t>
         </is>
       </c>
     </row>
@@ -35119,17 +36156,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>不純な彼女達は懺悔しない</t>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ポロロッカ(著者)</t>
+          <t>モリタ Ｕ４ nima</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第36話</t>
+          <t>第15話（４）　お嬢様と宰相と、とびきりの滋養食（４）</t>
         </is>
       </c>
     </row>
@@ -35139,17 +36176,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+          <t>田舎で恋は難しい!?</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>三部べべ(漫画) ねうしとら(原作)</t>
+          <t>ねこうめ(著者)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第7話-2</t>
+          <t>5話おまけ</t>
         </is>
       </c>
     </row>
@@ -35159,17 +36196,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>淫獄団地</t>
+          <t>ぽんドロイド！ はまさん</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+          <t>はれやまはれぞう(著者)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第55話（後編）</t>
+          <t>第17話</t>
         </is>
       </c>
     </row>
@@ -35179,17 +36216,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第46話　奴は再会する（前編）</t>
+          <t>第3話⑤</t>
         </is>
       </c>
     </row>
@@ -35199,17 +36236,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
+          <t>王たる股冠の輝きよ</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>夜州 nini 藻</t>
+          <t>原作：御城夏 作画：綿和わた</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第73話(前編)</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -35219,17 +36256,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>美人女上司滝沢さん</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>やんBARU(著者)</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第215話</t>
+          <t>第63話①　冷蔵庫を作ってみた</t>
         </is>
       </c>
     </row>
@@ -35239,17 +36276,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第2話 ネトル（前編）</t>
+          <t>第8話前編</t>
         </is>
       </c>
     </row>
@@ -35259,17 +36296,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>リアデイルの大地にて</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>月見だしお(著者) Ceez(原作) てんまそ(キャラクター原案) 涼風涼(構成)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第４６話　勇者、ラファエルとのRAPバトルでドープな韻のパンチライン＆ディープなリリックはアゲアゲで会場を沸かす（１）</t>
+          <t>第41章-2</t>
         </is>
       </c>
     </row>
@@ -35279,17 +36316,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+          <t>お気楽領主の楽しい領地防衛 ～生産系魔術で名もなき村を最強の城塞都市に～</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+          <t>青色まろ（漫画） 赤池宗（原作） 転（原作イラスト）</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>【お知らせ】コミックス第9巻、本日発売！</t>
+          <t>第38話　撤退</t>
         </is>
       </c>
     </row>
@@ -35299,17 +36336,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第12話-2：行き止まりの先</t>
+          <t>第30話②</t>
         </is>
       </c>
     </row>
@@ -35319,17 +36356,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>クール教信者</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第3話④</t>
+          <t>第162話</t>
         </is>
       </c>
     </row>
@@ -35339,17 +36376,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>アザミヤコを好きになる</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第14話後編</t>
+          <t>第150話 よくわからないけれど侵略しにきたみたいでゲソ（２）</t>
         </is>
       </c>
     </row>
@@ -35359,17 +36396,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>理想のヒモ生活</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第105話　その2</t>
+          <t>拷問175</t>
         </is>
       </c>
     </row>
@@ -35379,17 +36416,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第150話 よくわからないけれど侵略しにきたみたいでゲソ（１）</t>
+          <t>第４６話　勇者、ラファエルとのRAPバトルでドープな韻のパンチライン＆ディープなリリックはアゲアゲで会場を沸かす（２）</t>
         </is>
       </c>
     </row>
@@ -35399,17 +36436,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>板垣恵介 林たかあき</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第86話(前編)その3</t>
+          <t>第66話 半信半疑</t>
         </is>
       </c>
     </row>
@@ -35419,17 +36456,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>悪友の俺がポンコツ騎士を見てられないんだが、どう世話を焼きゃいい？ ～まどめ外伝～</t>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>原作：手島史詞 漫画：双葉もも キャラクター原案：COMTA 構成：板垣ハコ</t>
+          <t>KAKERU</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第20話</t>
+          <t>第74話「弓王3」（後半）</t>
         </is>
       </c>
     </row>
@@ -35439,17 +36476,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+          <t>ウォルテニア戦記</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+          <t>漫画：八木ゆかり 原作：保利亮太 キャラクター原案：bob</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第6話-2</t>
+          <t>第60話</t>
         </is>
       </c>
     </row>
@@ -35459,17 +36496,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>拷問174</t>
+          <t>第83話 ケンシロウ橘、脚本と対決す!!</t>
         </is>
       </c>
     </row>
@@ -35479,17 +36516,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>三枝さんはメガネ先輩と恋を描く</t>
+          <t>遊び人な少女たちは今日も放課後ヤっている</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>セレビィ量産型(著者)</t>
+          <t>逢上おかき(著者)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第25.5話</t>
+          <t>第3話</t>
         </is>
       </c>
     </row>
@@ -35499,17 +36536,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>サーシャちゃんとクラスメイトオタクくん</t>
+          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>はぐはぐ(著者)</t>
+          <t>六志麻あさ 業務用餅 kisui</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第95話</t>
+          <t>第８３話</t>
         </is>
       </c>
     </row>
@@ -35519,17 +36556,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+          <t>Lv２からチートだった元勇者候補のまったり異世界ライフ</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+          <t>糸町秋音（漫画） 鬼ノ城ミヤ（原作） 片桐（キャラクター原案）</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>コミックス５巻ついに発売!!!</t>
+          <t>第66話　出会いと構築（前編）</t>
         </is>
       </c>
     </row>
@@ -35539,17 +36576,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>原作:剃り残し 漫画:大窪太一</t>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第4話</t>
+          <t>第7話-2：暗躍する者たち</t>
         </is>
       </c>
     </row>
@@ -35559,17 +36596,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+          <t>漫画/すたひろ 原作/Y.A</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第3話(2)</t>
+          <t>chapter82【43話①】</t>
         </is>
       </c>
     </row>
@@ -35579,17 +36616,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>バーサス</t>
+          <t>黄金の経験値</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+          <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第32話　蜷局山と…（1）</t>
+          <t>第23話（前編）</t>
         </is>
       </c>
     </row>
@@ -35599,17 +36636,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第93話</t>
+          <t>第18話　最弱貴族、奔走する（３）</t>
         </is>
       </c>
     </row>
@@ -35619,17 +36656,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>最果てのパラディン</t>
+          <t>役目を果たした日陰の勇者は、辺境で自由に生きていきます</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>奥橋睦（漫画） 柳野かなた（原作） 輪くすさが（キャラクター原案）</t>
+          <t>船野真帆(作画) 丘野優(原作) 布施龍太(キャラクター原案)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第70話　無敵の巨人Ⅲ</t>
+          <t>第13話前半</t>
         </is>
       </c>
     </row>
@@ -35639,17 +36676,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>インフィニット・デンドログラム</t>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第76話</t>
+          <t>第3話(3)</t>
         </is>
       </c>
     </row>
@@ -35659,17 +36696,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+          <t>ダメ人間の愛しかた</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+          <t>岩葉(著者)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第7話-1</t>
+          <t>第25話前編　ダメ人間と彼女たちのクリスマス</t>
         </is>
       </c>
     </row>
@@ -35679,17 +36716,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>異世界でも無難に生きたい症候群</t>
+          <t>オタクに優しいギャルはいない!?</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>原作：安泰（一二三書房刊） 漫画：笹峰コウ キャラクター原案：ひたきゆう</t>
+          <t>のりしろちゃん 魚住さかな</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>【お知らせ】コミックス第7巻、本日発売！</t>
+          <t>【#183】テレ・トーク！</t>
         </is>
       </c>
     </row>
@@ -35699,17 +36736,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ディーふらぐ！</t>
+          <t>勇者の元仲間夫婦は田舎でのんびり幸せに暮らす</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>春野友矢(著者)</t>
+          <t>薊マスラオ(漫画) 相野仁(原作) nima(キャラクター原案)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第177話</t>
+          <t>第2話-1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-03-30
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -47,6 +47,7 @@
     <sheet name="2026-03-09" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="2026-03-16" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="2026-03-23" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="2026-03-30" sheetId="42" state="visible" r:id="rId42"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -35751,22 +35752,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第133話</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>ワンパンマン</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>223撃目</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>異種族レビュアーズ</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>天原(原作) masha(作画)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第91話</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第21話-2「乙女心」</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第７５話『黒兎停止』③</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第７６話　ホットヨガの戦いが始まった（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>いとこのこ</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>いぬちく(著者)</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第47話</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第8話 後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第84話その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>帰ってください！ 阿久津さん</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>長岡太一(著者)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第203話</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第20話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第7話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>金属スライムを倒しまくった俺が【黒鋼の王】と呼ばれるまで</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>藤屋いずこ(著者) 温泉カピバラ(原作) 山椒魚(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第18章-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第５８話　真相を知った器用貧乏（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第141話　とまどい</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第92話　小細工</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第134話　王都炎上Ⅰ（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第37話</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>まんきつしたい常連さん</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>しんみりん(著者)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第54話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第43話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>モリタ Ｕ４ nima</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第15話（４）　お嬢様と宰相と、とびきりの滋養食（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>田舎で恋は難しい!?</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>ねこうめ(著者)</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>5話おまけ</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>ぽんドロイド！ はまさん</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>はれやまはれぞう(著者)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第17話</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第3話⑤</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>王たる股冠の輝きよ</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>原作：御城夏 作画：綿和わた</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第63話①　冷蔵庫を作ってみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第8話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>リアデイルの大地にて</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>月見だしお(著者) Ceez(原作) てんまそ(キャラクター原案) 涼風涼(構成)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第41章-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>お気楽領主の楽しい領地防衛 ～生産系魔術で名もなき村を最強の城塞都市に～</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>青色まろ（漫画） 赤池宗（原作） 転（原作イラスト）</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第38話　撤退</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第30話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>小林さんちのメイドラゴン</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>クール教信者</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第162話</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第150話 よくわからないけれど侵略しにきたみたいでゲソ（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>拷問175</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第４６話　勇者、ラファエルとのRAPバトルでドープな韻のパンチライン＆ディープなリリックはアゲアゲで会場を沸かす（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 林たかあき</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第66話 半信半疑</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>KAKERU</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第74話「弓王3」（後半）</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>ウォルテニア戦記</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>漫画：八木ゆかり 原作：保利亮太 キャラクター原案：bob</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第60話</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第83話 ケンシロウ橘、脚本と対決す!!</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>遊び人な少女たちは今日も放課後ヤっている</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>逢上おかき(著者)</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第3話</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>六志麻あさ 業務用餅 kisui</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第８３話</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>Lv２からチートだった元勇者候補のまったり異世界ライフ</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>糸町秋音（漫画） 鬼ノ城ミヤ（原作） 片桐（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第66話　出会いと構築（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第7話-2：暗躍する者たち</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>漫画/すたひろ 原作/Y.A</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>chapter82【43話①】</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>黄金の経験値</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第23話（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>空野進 sorani ファルまろ</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第18話　最弱貴族、奔走する（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>役目を果たした日陰の勇者は、辺境で自由に生きていきます</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>船野真帆(作画) 丘野優(原作) 布施龍太(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第13話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第3話(3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>ダメ人間の愛しかた</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>岩葉(著者)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第25話前編　ダメ人間と彼女たちのクリスマス</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>オタクに優しいギャルはいない!?</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>のりしろちゃん 魚住さかな</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>【#183】テレ・トーク！</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>勇者の元仲間夫婦は田舎でのんびり幸せに暮らす</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>薊マスラオ(漫画) 相野仁(原作) nima(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第2話-1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>宇崎ちゃんは遊びたい！</t>
+          <t>異世界おじさん</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>丈(著者)</t>
+          <t>殆ど死んでいる(著者)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第133話</t>
+          <t>番外編13</t>
         </is>
       </c>
     </row>
@@ -35776,17 +36813,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ワンパンマン</t>
+          <t>魔術師クノンは見えている</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>原作/ＯＮＥ 作画/村田雄介</t>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>223撃目</t>
+          <t>第46話①</t>
         </is>
       </c>
     </row>
@@ -35796,17 +36833,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>異種族レビュアーズ</t>
+          <t>蜘蛛ですが、なにか？</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>天原(原作) masha(作画)</t>
+          <t>かかし朝浩(著者) 馬場翁(原作) 輝竜司(キャラクター原案)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第91話</t>
+          <t>第78話その2</t>
         </is>
       </c>
     </row>
@@ -35816,17 +36853,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第21話-2「乙女心」</t>
+          <t>第７５話『黒兎停止』④</t>
         </is>
       </c>
     </row>
@@ -35836,17 +36873,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>むちまろ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第７５話『黒兎停止』③</t>
+          <t>第148話	虎丸後輩とこまろ先輩</t>
         </is>
       </c>
     </row>
@@ -35866,7 +36903,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第７６話　ホットヨガの戦いが始まった（１）</t>
+          <t>第７６話　ホットヨガの戦いが始まった（２）</t>
         </is>
       </c>
     </row>
@@ -35876,17 +36913,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>いとこのこ</t>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>いぬちく(著者)</t>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第47話</t>
+          <t>第39話②</t>
         </is>
       </c>
     </row>
@@ -35896,17 +36933,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第8話 後編</t>
+          <t>第17話-2</t>
         </is>
       </c>
     </row>
@@ -35916,17 +36953,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+          <t>クセ強彼女は床にいざなう</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+          <t>須河篤志(著者)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第84話その2</t>
+          <t>第20話後半</t>
         </is>
       </c>
     </row>
@@ -35936,17 +36973,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>帰ってください！ 阿久津さん</t>
+          <t>異世界居酒屋「のぶ」</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>長岡太一(著者)</t>
+          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第203話</t>
+          <t>第131話</t>
         </is>
       </c>
     </row>
@@ -35956,17 +36993,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+          <t>「おかえり、パパ」</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+          <t>蝉丸</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第20話後半</t>
+          <t>第34話　デート</t>
         </is>
       </c>
     </row>
@@ -35976,17 +37013,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第7話前半</t>
+          <t>第５８話　真相を知った器用貧乏（４）</t>
         </is>
       </c>
     </row>
@@ -35996,17 +37033,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>金属スライムを倒しまくった俺が【黒鋼の王】と呼ばれるまで</t>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>藤屋いずこ(著者) 温泉カピバラ(原作) 山椒魚(キャラクター原案)</t>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第18章-2</t>
+          <t>第8話-1</t>
         </is>
       </c>
     </row>
@@ -36016,17 +37053,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第５８話　真相を知った器用貧乏（３）</t>
+          <t>第5話後編：未練</t>
         </is>
       </c>
     </row>
@@ -36036,17 +37073,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>ダークサモナーとデキている</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>車王(著者)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第141話　とまどい</t>
+          <t>第87話</t>
         </is>
       </c>
     </row>
@@ -36056,17 +37093,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+          <t>異世界のんびり農家</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>板垣恵介 猪原賽 陸井栄史</t>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第92話　小細工</t>
+          <t>第319話</t>
         </is>
       </c>
     </row>
@@ -36076,17 +37113,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第134話　王都炎上Ⅰ（後編）</t>
+          <t>おまけ71</t>
         </is>
       </c>
     </row>
@@ -36096,17 +37133,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+          <t>淫獄団地</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第37話</t>
+          <t>第56話（前編）</t>
         </is>
       </c>
     </row>
@@ -36116,17 +37153,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>まんきつしたい常連さん</t>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>しんみりん(著者)</t>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第54話後編</t>
+          <t>第２８食　レッドワイバーンさんのシチュー、パクパクですわ！（２）</t>
         </is>
       </c>
     </row>
@@ -36136,17 +37173,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
+          <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
+          <t>安田剛助(著者)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第43話-2</t>
+          <t>第55話</t>
         </is>
       </c>
     </row>
@@ -36156,17 +37193,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>モリタ Ｕ４ nima</t>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第15話（４）　お嬢様と宰相と、とびきりの滋養食（４）</t>
+          <t>第38話 独身貴族は野鳥を撮りたい（1）</t>
         </is>
       </c>
     </row>
@@ -36176,17 +37213,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>田舎で恋は難しい!?</t>
+          <t>物語の黒幕に転生して</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ねこうめ(著者)</t>
+          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>5話おまけ</t>
+          <t>第40話</t>
         </is>
       </c>
     </row>
@@ -36196,17 +37233,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ぽんドロイド！ はまさん</t>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>はれやまはれぞう(著者)</t>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第17話</t>
+          <t>第46話　奴は再会する（後編）</t>
         </is>
       </c>
     </row>
@@ -36216,17 +37253,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>美人女上司滝沢さん</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>やんBARU(著者)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第3話⑤</t>
+          <t>第216話</t>
         </is>
       </c>
     </row>
@@ -36236,17 +37273,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>王たる股冠の輝きよ</t>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>原作：御城夏 作画：綿和わた</t>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>第2話 ネトル（後編）</t>
         </is>
       </c>
     </row>
@@ -36266,7 +37303,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第63話①　冷蔵庫を作ってみた</t>
+          <t>第63話②　冷蔵庫を作ってみた</t>
         </is>
       </c>
     </row>
@@ -36276,17 +37313,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+          <t>おとなりのダウナーさんは無理させない</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+          <t>瑠璃いろ(著者)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第8話前編</t>
+          <t>第15話</t>
         </is>
       </c>
     </row>
@@ -36296,17 +37333,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>リアデイルの大地にて</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>月見だしお(著者) Ceez(原作) てんまそ(キャラクター原案) 涼風涼(構成)</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第41章-2</t>
+          <t>第151話 よくわからないけれどイカす宴のようです（１）</t>
         </is>
       </c>
     </row>
@@ -36316,17 +37353,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>お気楽領主の楽しい領地防衛 ～生産系魔術で名もなき村を最強の城塞都市に～</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>青色まろ（漫画） 赤池宗（原作） 転（原作イラスト）</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第38話　撤退</t>
+          <t>第４６話　勇者、ラファエルとのRAPバトルでドープな韻のパンチライン＆ディープなリリックはアゲアゲで会場を沸かす（３）</t>
         </is>
       </c>
     </row>
@@ -36336,17 +37373,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>女友達は頼めば意外とヤらせてくれる</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ろくろ(漫画) 鏡遊(原作)</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第30話②</t>
+          <t>拷問176</t>
         </is>
       </c>
     </row>
@@ -36356,17 +37393,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>小林さんちのメイドラゴン</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>クール教信者</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第162話</t>
+          <t>第86話(後編)その1</t>
         </is>
       </c>
     </row>
@@ -36376,17 +37413,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>幼女戦記</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第150話 よくわからないけれど侵略しにきたみたいでゲソ（２）</t>
+          <t>第百十三章：ドードーバード航空戦Ⅷ</t>
         </is>
       </c>
     </row>
@@ -36396,17 +37433,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>拷問175</t>
+          <t>第133話</t>
         </is>
       </c>
     </row>
@@ -36416,17 +37453,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>原作:剃り残し 漫画:大窪太一</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第４６話　勇者、ラファエルとのRAPバトルでドープな韻のパンチライン＆ディープなリリックはアゲアゲで会場を沸かす（２）</t>
+          <t>第5話</t>
         </is>
       </c>
     </row>
@@ -36436,17 +37473,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+          <t>くらいあの子としたいこと</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>板垣恵介 林たかあき</t>
+          <t>碇マナツ(著者)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第66話 半信半疑</t>
+          <t>第94話</t>
         </is>
       </c>
     </row>
@@ -36456,17 +37493,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>KAKERU</t>
+          <t>セレビィ量産型(著者)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第74話「弓王3」（後半）</t>
+          <t>第26話前半</t>
         </is>
       </c>
     </row>
@@ -36476,17 +37513,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ウォルテニア戦記</t>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>漫画：八木ゆかり 原作：保利亮太 キャラクター原案：bob</t>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第60話</t>
+          <t>第7話-2</t>
         </is>
       </c>
     </row>
@@ -36496,17 +37533,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+          <t>バーサス</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第83話 ケンシロウ橘、脚本と対決す!!</t>
+          <t>第32話 蜷局山と…（2）</t>
         </is>
       </c>
     </row>
@@ -36516,17 +37553,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>遊び人な少女たちは今日も放課後ヤっている</t>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>逢上おかき(著者)</t>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第3話</t>
+          <t>第23話①</t>
         </is>
       </c>
     </row>
@@ -36536,17 +37573,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
+          <t>魔王になったので、ダンジョン造って人外娘とほのぼのする</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>六志麻あさ 業務用餅 kisui</t>
+          <t>遠野ノオト(作画) 流優(原作) だぶ竜(キャラクター原案)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第８３話</t>
+          <t>第88話後半</t>
         </is>
       </c>
     </row>
@@ -36556,17 +37593,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Lv２からチートだった元勇者候補のまったり異世界ライフ</t>
+          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>糸町秋音（漫画） 鬼ノ城ミヤ（原作） 片桐（キャラクター原案）</t>
+          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第66話　出会いと構築（前編）</t>
+          <t>休載告知</t>
         </is>
       </c>
     </row>
@@ -36576,17 +37613,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+          <t>おせっかい女子、恋をする</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+          <t>音竹 ひかる(著者)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第7話-2：暗躍する者たち</t>
+          <t>第9話</t>
         </is>
       </c>
     </row>
@@ -36596,17 +37633,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>漫画/すたひろ 原作/Y.A</t>
+          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>chapter82【43話①】</t>
+          <t>第9話②「勇気の出しかた」</t>
         </is>
       </c>
     </row>
@@ -36616,17 +37653,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>黄金の経験値</t>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
+          <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第23話（前編）</t>
+          <t>第19話　最弱貴族、魔王と聖女を仲裁する（１）</t>
         </is>
       </c>
     </row>
@@ -36636,17 +37673,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+          <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>空野進 sorani ファルまろ</t>
+          <t>岡沢六十四 るれくちぇ sage・ジョー</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第18話　最弱貴族、奔走する（３）</t>
+          <t>第79話(前編) 最強の夫婦</t>
         </is>
       </c>
     </row>
@@ -36656,17 +37693,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>役目を果たした日陰の勇者は、辺境で自由に生きていきます</t>
+          <t>めっちゃ召喚された件 THE COMIC</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>船野真帆(作画) 丘野優(原作) 布施龍太(キャラクター原案)</t>
+          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第13話前半</t>
+          <t>第54話①</t>
         </is>
       </c>
     </row>
@@ -36676,17 +37713,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+          <t>お前がヤったんだろ！</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+          <t>クシザキ</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第3話(3)</t>
+          <t>第7話	エロい家</t>
         </is>
       </c>
     </row>
@@ -36696,17 +37733,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ダメ人間の愛しかた</t>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>岩葉(著者)</t>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第25話前編　ダメ人間と彼女たちのクリスマス</t>
+          <t>第4話(1)</t>
         </is>
       </c>
     </row>
@@ -36716,17 +37753,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>オタクに優しいギャルはいない!?</t>
+          <t>地味子な三葉さんが僕を誘惑する</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>のりしろちゃん 魚住さかな</t>
+          <t>はぶらえる(著者)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>【#183】テレ・トーク！</t>
+          <t>第14話後半</t>
         </is>
       </c>
     </row>
@@ -36736,17 +37773,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>勇者の元仲間夫婦は田舎でのんびり幸せに暮らす</t>
+          <t>ぽんドロイド！ はまさん</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>薊マスラオ(漫画) 相野仁(原作) nima(キャラクター原案)</t>
+          <t>はれやまはれぞう(著者)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第2話-1</t>
+          <t>コミックス告知</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-04-06
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -48,6 +48,7 @@
     <sheet name="2026-03-16" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="2026-03-23" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="2026-03-30" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="2026-04-06" sheetId="43" state="visible" r:id="rId43"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -36788,22 +36789,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>異世界おじさん</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>殆ど死んでいる(著者)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>番外編13</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第46話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>蜘蛛ですが、なにか？</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>かかし朝浩(著者) 馬場翁(原作) 輝竜司(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第78話その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第７５話『黒兎停止』④</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第148話	虎丸後輩とこまろ先輩</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第７６話　ホットヨガの戦いが始まった（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第39話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第17話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第20話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>異世界居酒屋「のぶ」</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第131話</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>「おかえり、パパ」</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>蝉丸</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第34話　デート</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第５８話　真相を知った器用貧乏（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第8話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第5話後編：未練</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第87話</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第319話</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>おまけ71</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>淫獄団地</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第56話（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第２８食　レッドワイバーンさんのシチュー、パクパクですわ！（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>安田剛助(著者)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第55話</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第38話 独身貴族は野鳥を撮りたい（1）</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>物語の黒幕に転生して</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第40話</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第46話　奴は再会する（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>美人女上司滝沢さん</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>やんBARU(著者)</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第216話</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第2話 ネトル（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第63話②　冷蔵庫を作ってみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>おとなりのダウナーさんは無理させない</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>瑠璃いろ(著者)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第15話</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第151話 よくわからないけれどイカす宴のようです（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第４６話　勇者、ラファエルとのRAPバトルでドープな韻のパンチライン＆ディープなリリックはアゲアゲで会場を沸かす（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>拷問176</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第86話(後編)その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>幼女戦記</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第百十三章：ドードーバード航空戦Ⅷ</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第133話</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>原作:剃り残し 漫画:大窪太一</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第5話</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第94話</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第26話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第7話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>バーサス</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第32話 蜷局山と…（2）</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第23話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>魔王になったので、ダンジョン造って人外娘とほのぼのする</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>遠野ノオト(作画) 流優(原作) だぶ竜(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第88話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>休載告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第9話</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第9話②「勇気の出しかた」</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>空野進 sorani ファルまろ</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第19話　最弱貴族、魔王と聖女を仲裁する（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>岡沢六十四 るれくちぇ sage・ジョー</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第79話(前編) 最強の夫婦</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>めっちゃ召喚された件 THE COMIC</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第54話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>クシザキ</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第7話	エロい家</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第4話(1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>地味子な三葉さんが僕を誘惑する</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>はぶらえる(著者)</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第14話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>ぽんドロイド！ はまさん</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>はれやまはれぞう(著者)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>コミックス告知</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>異世界おじさん</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>殆ど死んでいる(著者)</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>番外編13</t>
+          <t>第134話</t>
         </is>
       </c>
     </row>
@@ -36813,17 +37850,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>魔術師クノンは見えている</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第46話①</t>
+          <t>224撃目</t>
         </is>
       </c>
     </row>
@@ -36833,17 +37870,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>蜘蛛ですが、なにか？</t>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>かかし朝浩(著者) 馬場翁(原作) 輝竜司(キャラクター原案)</t>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第78話その2</t>
+          <t>第77話</t>
         </is>
       </c>
     </row>
@@ -36853,17 +37890,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第７５話『黒兎停止』④</t>
+          <t>第22話-1「子供たちはどこだ？」</t>
         </is>
       </c>
     </row>
@@ -36873,17 +37910,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>王子様の友達</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>すけろく(著者)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第148話	虎丸後輩とこまろ先輩</t>
+          <t>第36話</t>
         </is>
       </c>
     </row>
@@ -36893,17 +37930,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第７６話　ホットヨガの戦いが始まった（２）</t>
+          <t>第85話その1</t>
         </is>
       </c>
     </row>
@@ -36913,17 +37950,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+          <t>いとこのこ</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+          <t>いぬちく(著者)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第39話②</t>
+          <t>第48話</t>
         </is>
       </c>
     </row>
@@ -36933,17 +37970,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+          <t>帰ってください！ 阿久津さん</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+          <t>長岡太一(著者)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第17話-2</t>
+          <t>第204話</t>
         </is>
       </c>
     </row>
@@ -36953,17 +37990,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第20話後半</t>
+          <t>第21話前半</t>
         </is>
       </c>
     </row>
@@ -36973,17 +38010,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>異世界居酒屋「のぶ」</t>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第131話</t>
+          <t>第7話後半</t>
         </is>
       </c>
     </row>
@@ -36993,17 +38030,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>「おかえり、パパ」</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>蝉丸</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第34話　デート</t>
+          <t>第５８話　真相を知った器用貧乏（４）</t>
         </is>
       </c>
     </row>
@@ -37013,17 +38050,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第５８話　真相を知った器用貧乏（４）</t>
+          <t>第142話　テレジア参戦！・前編</t>
         </is>
       </c>
     </row>
@@ -37033,17 +38070,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>三部べべ(漫画) ねうしとら(原作)</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第8話-1</t>
+          <t>第135話　王都炎上Ⅱ（前編）</t>
         </is>
       </c>
     </row>
@@ -37053,17 +38090,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+          <t>剥かせて！竜ケ崎さん</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+          <t>一智和智</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第5話後編：未練</t>
+          <t>大学生編 第19話</t>
         </is>
       </c>
     </row>
@@ -37073,17 +38110,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ダークサモナーとデキている</t>
+          <t>不純な彼女達は懺悔しない</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>車王(著者)</t>
+          <t>ポロロッカ(著者)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第87話</t>
+          <t>第37話</t>
         </is>
       </c>
     </row>
@@ -37093,17 +38130,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>異世界のんびり農家</t>
+          <t>まんきつしたい常連さん</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+          <t>しんみりん(著者)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第319話</t>
+          <t>第55話前編</t>
         </is>
       </c>
     </row>
@@ -37113,17 +38150,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>田舎で恋は難しい!?</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>ねこうめ(著者)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>おまけ71</t>
+          <t>第6話</t>
         </is>
       </c>
     </row>
@@ -37133,17 +38170,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>淫獄団地</t>
+          <t>このヒーラー、めんどくさい</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+          <t>丹念に発酵(著者)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第56話（前編）</t>
+          <t>第96話：解釈</t>
         </is>
       </c>
     </row>
@@ -37153,17 +38190,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>島知宏 音速炒飯 有都あらゆる</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第２８食　レッドワイバーンさんのシチュー、パクパクですわ！（２）</t>
+          <t>第79話</t>
         </is>
       </c>
     </row>
@@ -37173,17 +38210,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>安田剛助(著者)</t>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第55話</t>
+          <t>第２８食　レッドワイバーンさんのシチュー、パクパクですわ！（３）</t>
         </is>
       </c>
     </row>
@@ -37203,7 +38240,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第38話 独身貴族は野鳥を撮りたい（1）</t>
+          <t>第38話 独身貴族は野鳥を撮りたい（2）</t>
         </is>
       </c>
     </row>
@@ -37213,17 +38250,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>物語の黒幕に転生して</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第40話</t>
+          <t>第4話①</t>
         </is>
       </c>
     </row>
@@ -37233,17 +38270,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+          <t>虚無ねーちゃんはかまってほしい</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+          <t>観音リツ(著者)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第46話　奴は再会する（後編）</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -37253,17 +38290,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>美人女上司滝沢さん</t>
+          <t>ぽんドロイド！ はまさん</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>やんBARU(著者)</t>
+          <t>はれやまはれぞう(著者)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第216話</t>
+          <t>第18話</t>
         </is>
       </c>
     </row>
@@ -37273,17 +38310,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第2話 ネトル（後編）</t>
+          <t>第64話①　鍛冶を見学してみた</t>
         </is>
       </c>
     </row>
@@ -37293,17 +38330,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>聖者無双</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第63話②　冷蔵庫を作ってみた</t>
+          <t>第97話　消えた魔物の死体・蟻の生態①</t>
         </is>
       </c>
     </row>
@@ -37313,17 +38350,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>おとなりのダウナーさんは無理させない</t>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>瑠璃いろ(著者)</t>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第15話</t>
+          <t>第8話後編</t>
         </is>
       </c>
     </row>
@@ -37333,17 +38370,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第151話 よくわからないけれどイカす宴のようです（１）</t>
+          <t>第31話①</t>
         </is>
       </c>
     </row>
@@ -37353,17 +38390,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第４６話　勇者、ラファエルとのRAPバトルでドープな韻のパンチライン＆ディープなリリックはアゲアゲで会場を沸かす（３）</t>
+          <t>第13話-1：思い出の写真</t>
         </is>
       </c>
     </row>
@@ -37373,17 +38410,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>拷問176</t>
+          <t>第151話 よくわからないけれどイカす宴のようです（２）</t>
         </is>
       </c>
     </row>
@@ -37393,17 +38430,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第86話(後編)その1</t>
+          <t>第４６話　勇者、ラファエルとのRAPバトルでドープな韻のパンチライン＆ディープなリリックはアゲアゲで会場を沸かす（４）</t>
         </is>
       </c>
     </row>
@@ -37413,17 +38450,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>幼女戦記</t>
+          <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
+          <t>クール教信者</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第百十三章：ドードーバード航空戦Ⅷ</t>
+          <t>第163話</t>
         </is>
       </c>
     </row>
@@ -37433,17 +38470,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>宇崎ちゃんは遊びたい！</t>
+          <t>黄金の経験値</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>丈(著者)</t>
+          <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第133話</t>
+          <t>第23話（後編）</t>
         </is>
       </c>
     </row>
@@ -37453,17 +38490,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>原作:剃り残し 漫画:大窪太一</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第5話</t>
+          <t>拷問177</t>
         </is>
       </c>
     </row>
@@ -37473,17 +38510,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第94話</t>
+          <t>第84話 トキ役大石、最後の輝き!!</t>
         </is>
       </c>
     </row>
@@ -37493,17 +38530,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>三枝さんはメガネ先輩と恋を描く</t>
+          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>セレビィ量産型(著者)</t>
+          <t>六志麻あさ 業務用餅 kisui</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第26話前半</t>
+          <t>第８４話</t>
         </is>
       </c>
     </row>
@@ -37513,17 +38550,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+          <t>遊遊じてき。</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+          <t>カンケー</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第7話-2</t>
+          <t>閑話（単行本版発売記念）</t>
         </is>
       </c>
     </row>
@@ -37533,17 +38570,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>バーサス</t>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+          <t>はぐはぐ(著者)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第32話 蜷局山と…（2）</t>
+          <t>第96話</t>
         </is>
       </c>
     </row>
@@ -37553,17 +38590,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+          <t>異世界居酒屋「のぶ」</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第23話①</t>
+          <t>第131話</t>
         </is>
       </c>
     </row>
@@ -37573,17 +38610,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>魔王になったので、ダンジョン造って人外娘とほのぼのする</t>
+          <t>迷宮の王</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>遠野ノオト(作画) 流優(原作) だぶ竜(キャラクター原案)</t>
+          <t>漫画：K9 脚本：小林裕和 原作：支援BIS</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第88話後半</t>
+          <t>第十六話　血戦（一）</t>
         </is>
       </c>
     </row>
@@ -37593,17 +38630,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>休載告知</t>
+          <t>第8話-1：子供の守り神</t>
         </is>
       </c>
     </row>
@@ -37613,17 +38650,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>おせっかい女子、恋をする</t>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>音竹 ひかる(著者)</t>
+          <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第9話</t>
+          <t>第19話　最弱貴族、魔王と聖女を仲裁する（２）</t>
         </is>
       </c>
     </row>
@@ -37633,17 +38670,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
+          <t>おせっかい女子、恋をする</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
+          <t>音竹 ひかる(著者)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第9話②「勇気の出しかた」</t>
+          <t>第10話</t>
         </is>
       </c>
     </row>
@@ -37653,17 +38690,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>空野進 sorani ファルまろ</t>
+          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第19話　最弱貴族、魔王と聖女を仲裁する（１）</t>
+          <t>第41話</t>
         </is>
       </c>
     </row>
@@ -37673,17 +38710,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>岡沢六十四 るれくちぇ sage・ジョー</t>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第79話(前編) 最強の夫婦</t>
+          <t>第4話(2)</t>
         </is>
       </c>
     </row>
@@ -37693,17 +38730,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>めっちゃ召喚された件 THE COMIC</t>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第54話①</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -37713,17 +38750,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>お前がヤったんだろ！</t>
+          <t>世界最高の暗殺者、異世界貴族に転生する</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>クシザキ</t>
+          <t>月夜涙(原作) 皇ハマオ(漫画) れい亜(キャラクター原案)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第7話	エロい家</t>
+          <t>第42話-1</t>
         </is>
       </c>
     </row>
@@ -37733,17 +38770,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+          <t>オタクに優しいギャルはいない!?</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+          <t>のりしろちゃん 魚住さかな</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第4話(1)</t>
+          <t>【#185】ベッドの上の葛藤</t>
         </is>
       </c>
     </row>
@@ -37753,17 +38790,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>地味子な三葉さんが僕を誘惑する</t>
+          <t>ダメ人間の愛しかた</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>はぶらえる(著者)</t>
+          <t>岩葉(著者)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第14話後半</t>
+          <t>第25話後編　ダメ人間と彼女たちのクリスマス</t>
         </is>
       </c>
     </row>
@@ -37773,17 +38810,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ぽんドロイド！ はまさん</t>
+          <t>ひとりぼっちの異世界攻略</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>はれやまはれぞう(著者)</t>
+          <t>びび（漫画） 五示正司（原作）</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>コミックス告知</t>
+          <t>第264話　最後は悦んでた？</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-04-13
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -49,6 +49,7 @@
     <sheet name="2026-03-23" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="2026-03-30" sheetId="42" state="visible" r:id="rId42"/>
     <sheet name="2026-04-06" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="2026-04-13" sheetId="44" state="visible" r:id="rId44"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -37825,22 +37826,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第134話</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>ワンパンマン</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>224撃目</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第77話</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第22話-1「子供たちはどこだ？」</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>王子様の友達</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>すけろく(著者)</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第36話</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第85話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>いとこのこ</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>いぬちく(著者)</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第48話</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>帰ってください！ 阿久津さん</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>長岡太一(著者)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第204話</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第21話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第7話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第５８話　真相を知った器用貧乏（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第142話　テレジア参戦！・前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第135話　王都炎上Ⅱ（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>剥かせて！竜ケ崎さん</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>一智和智</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>大学生編 第19話</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>不純な彼女達は懺悔しない</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>ポロロッカ(著者)</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第37話</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>まんきつしたい常連さん</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>しんみりん(著者)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第55話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>田舎で恋は難しい!?</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>ねこうめ(著者)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第6話</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>このヒーラー、めんどくさい</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>丹念に発酵(著者)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第96話：解釈</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第79話</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第２８食　レッドワイバーンさんのシチュー、パクパクですわ！（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第38話 独身貴族は野鳥を撮りたい（2）</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第4話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>虚無ねーちゃんはかまってほしい</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>観音リツ(著者)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>ぽんドロイド！ はまさん</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>はれやまはれぞう(著者)</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第18話</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第64話①　鍛冶を見学してみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>聖者無双</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第97話　消えた魔物の死体・蟻の生態①</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第8話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第31話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第13話-1：思い出の写真</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第151話 よくわからないけれどイカす宴のようです（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第４６話　勇者、ラファエルとのRAPバトルでドープな韻のパンチライン＆ディープなリリックはアゲアゲで会場を沸かす（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>小林さんちのメイドラゴン</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>クール教信者</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第163話</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>黄金の経験値</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第23話（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>拷問177</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第84話 トキ役大石、最後の輝き!!</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>六志麻あさ 業務用餅 kisui</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第８４話</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>遊遊じてき。</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>カンケー</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>閑話（単行本版発売記念）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>はぐはぐ(著者)</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第96話</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>異世界居酒屋「のぶ」</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第131話</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>迷宮の王</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>漫画：K9 脚本：小林裕和 原作：支援BIS</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第十六話　血戦（一）</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第8話-1：子供の守り神</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>空野進 sorani ファルまろ</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第19話　最弱貴族、魔王と聖女を仲裁する（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第10話</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第41話</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第4話(2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>世界最高の暗殺者、異世界貴族に転生する</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>月夜涙(原作) 皇ハマオ(漫画) れい亜(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第42話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>オタクに優しいギャルはいない!?</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>のりしろちゃん 魚住さかな</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>【#185】ベッドの上の葛藤</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>ダメ人間の愛しかた</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>岩葉(著者)</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第25話後編　ダメ人間と彼女たちのクリスマス</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>ひとりぼっちの異世界攻略</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>びび（漫画） 五示正司（原作）</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第264話　最後は悦んでた？</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>宇崎ちゃんは遊びたい！</t>
+          <t>魔術師クノンは見えている</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>丈(著者)</t>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第134話</t>
+          <t>第46話➁</t>
         </is>
       </c>
     </row>
@@ -37850,17 +38887,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ワンパンマン</t>
+          <t>不徳のギルド</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>原作/ＯＮＥ 作画/村田雄介</t>
+          <t>河添太一</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>224撃目</t>
+          <t>第１０５話：丸裸の思い</t>
         </is>
       </c>
     </row>
@@ -37870,17 +38907,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第77話</t>
+          <t>第37話：キモい動き①</t>
         </is>
       </c>
     </row>
@@ -37890,17 +38927,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第22話-1「子供たちはどこだ？」</t>
+          <t>第9話 前編</t>
         </is>
       </c>
     </row>
@@ -37910,17 +38947,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>王子様の友達</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>すけろく(著者)</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第36話</t>
+          <t>第７６話『渦中停止』①</t>
         </is>
       </c>
     </row>
@@ -37930,17 +38967,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第85話その1</t>
+          <t>第７７話　音ゲーの戦いが始まった（１）</t>
         </is>
       </c>
     </row>
@@ -37950,17 +38987,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>いとこのこ</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>いぬちく(著者)</t>
+          <t>むちまろ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第48話</t>
+          <t>第149話	有栖の足つぼ！</t>
         </is>
       </c>
     </row>
@@ -37970,17 +39007,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>帰ってください！ 阿久津さん</t>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>長岡太一(著者)</t>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第204話</t>
+          <t>第40話①</t>
         </is>
       </c>
     </row>
@@ -37990,17 +39027,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+          <t>ダンジョンの幼なじみ</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+          <t>久真やすひさ(著者)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第21話前半</t>
+          <t>第63話</t>
         </is>
       </c>
     </row>
@@ -38010,17 +39047,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第7話後半</t>
+          <t>第18話-1</t>
         </is>
       </c>
     </row>
@@ -38030,17 +39067,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>異世界のんびり農家</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第５８話　真相を知った器用貧乏（４）</t>
+          <t>第320話</t>
         </is>
       </c>
     </row>
@@ -38050,17 +39087,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>クセ強彼女は床にいざなう</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>須河篤志(著者)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第142話　テレジア参戦！・前編</t>
+          <t>番外編</t>
         </is>
       </c>
     </row>
@@ -38070,17 +39107,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第135話　王都炎上Ⅱ（前編）</t>
+          <t>第12話</t>
         </is>
       </c>
     </row>
@@ -38090,17 +39127,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>剥かせて！竜ケ崎さん</t>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>一智和智</t>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>大学生編 第19話</t>
+          <t>番外編②</t>
         </is>
       </c>
     </row>
@@ -38110,17 +39147,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>不純な彼女達は懺悔しない</t>
+          <t>ダークサモナーとデキている</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ポロロッカ(著者)</t>
+          <t>車王(著者)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第37話</t>
+          <t>第88話</t>
         </is>
       </c>
     </row>
@@ -38130,17 +39167,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>まんきつしたい常連さん</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>しんみりん(著者)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第55話前編</t>
+          <t>第142話　テレジア参戦！・後編</t>
         </is>
       </c>
     </row>
@@ -38150,17 +39187,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>田舎で恋は難しい!?</t>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ねこうめ(著者)</t>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第6話</t>
+          <t>第93話　幻影魔法(イリュージョン)</t>
         </is>
       </c>
     </row>
@@ -38170,17 +39207,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>このヒーラー、めんどくさい</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>丹念に発酵(著者)</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第96話：解釈</t>
+          <t>第135話　王都炎上Ⅱ（中編）</t>
         </is>
       </c>
     </row>
@@ -38190,17 +39227,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>魔のものたちは企てる</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>加藤拓弐(原作) ガしガし(作画)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第79話</t>
+          <t>第36話</t>
         </is>
       </c>
     </row>
@@ -38210,17 +39247,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+          <t>淫獄団地</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>島知宏 音速炒飯 有都あらゆる</t>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第２８食　レッドワイバーンさんのシチュー、パクパクですわ！（３）</t>
+          <t>第56話（後編）</t>
         </is>
       </c>
     </row>
@@ -38230,17 +39267,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第38話 独身貴族は野鳥を撮りたい（2）</t>
+          <t>第80話①</t>
         </is>
       </c>
     </row>
@@ -38250,17 +39287,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第4話①</t>
+          <t>第3話 ちゅう</t>
         </is>
       </c>
     </row>
@@ -38270,17 +39307,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>虚無ねーちゃんはかまってほしい</t>
+          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>観音リツ(著者)</t>
+          <t>久遠まこと(著者) 石のやっさん(原作)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>休載イラスト</t>
         </is>
       </c>
     </row>
@@ -38290,17 +39327,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ぽんドロイド！ はまさん</t>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>はれやまはれぞう(著者)</t>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第18話</t>
+          <t>第38話 独身貴族は野鳥を撮りたい（3）</t>
         </is>
       </c>
     </row>
@@ -38310,17 +39347,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第64話①　鍛冶を見学してみた</t>
+          <t>孤島の主のミステリーですわ！</t>
         </is>
       </c>
     </row>
@@ -38330,17 +39367,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>聖者無双</t>
+          <t>美人女上司滝沢さん</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+          <t>やんBARU(著者)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第97話　消えた魔物の死体・蟻の生態①</t>
+          <t>第217話</t>
         </is>
       </c>
     </row>
@@ -38350,17 +39387,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第8話後編</t>
+          <t>休載イラスト</t>
         </is>
       </c>
     </row>
@@ -38370,17 +39407,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>女友達は頼めば意外とヤらせてくれる</t>
+          <t>アザミヤコを好きになる</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ろくろ(漫画) 鏡遊(原作)</t>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第31話①</t>
+          <t>第15話前編</t>
         </is>
       </c>
     </row>
@@ -38390,17 +39427,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+          <t>ケツバトラー</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+          <t>高出なおたか ©面白法人カヤック／小学館</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第13話-1：思い出の写真</t>
+          <t>第32話</t>
         </is>
       </c>
     </row>
@@ -38410,17 +39447,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第151話 よくわからないけれどイカす宴のようです（２）</t>
+          <t>第64話②　鍛冶を見学してみた</t>
         </is>
       </c>
     </row>
@@ -38430,17 +39467,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第４６話　勇者、ラファエルとのRAPバトルでドープな韻のパンチライン＆ディープなリリックはアゲアゲで会場を沸かす（４）</t>
+          <t>第47話　奴のともだち（前編）</t>
         </is>
       </c>
     </row>
@@ -38450,17 +39487,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>小林さんちのメイドラゴン</t>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>クール教信者</t>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第163話</t>
+          <t>第7話-1</t>
         </is>
       </c>
     </row>
@@ -38470,17 +39507,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>黄金の経験値</t>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第23話（後編）</t>
+          <t>第2話-①</t>
         </is>
       </c>
     </row>
@@ -38490,17 +39527,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>KAKERU</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>拷問177</t>
+          <t>第75話「魔術師の森（お呼ばれ）」（前半）</t>
         </is>
       </c>
     </row>
@@ -38510,17 +39547,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+          <t>板垣恵介 林たかあき</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第84話 トキ役大石、最後の輝き!!</t>
+          <t>第67話 闘志</t>
         </is>
       </c>
     </row>
@@ -38530,17 +39567,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>六志麻あさ 業務用餅 kisui</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第８４話</t>
+          <t>拷問178</t>
         </is>
       </c>
     </row>
@@ -38550,17 +39587,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>遊遊じてき。</t>
+          <t>お前がヤったんだろ！</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>カンケー</t>
+          <t>クシザキ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>閑話（単行本版発売記念）</t>
+          <t>第8話	教育者Xの献身</t>
         </is>
       </c>
     </row>
@@ -38570,17 +39607,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>サーシャちゃんとクラスメイトオタクくん</t>
+          <t>理想のヒモ生活</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>はぐはぐ(著者)</t>
+          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第96話</t>
+          <t>第106話　その2</t>
         </is>
       </c>
     </row>
@@ -38590,17 +39627,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>異世界居酒屋「のぶ」</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第131話</t>
+          <t>第４６話　勇者、ラファエルとのRAPバトルでドープな韻のパンチライン＆ディープなリリックはアゲアゲで会場を沸かす（５）</t>
         </is>
       </c>
     </row>
@@ -38610,17 +39647,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>迷宮の王</t>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>漫画：K9 脚本：小林裕和 原作：支援BIS</t>
+          <t>原作:剃り残し 漫画:大窪太一</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第十六話　血戦（一）</t>
+          <t>第6話</t>
         </is>
       </c>
     </row>
@@ -38630,17 +39667,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第8話-1：子供の守り神</t>
+          <t>第86話(後編)その2</t>
         </is>
       </c>
     </row>
@@ -38650,17 +39687,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>空野進 sorani ファルまろ</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第19話　最弱貴族、魔王と聖女を仲裁する（２）</t>
+          <t>第134話</t>
         </is>
       </c>
     </row>
@@ -38670,17 +39707,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>おせっかい女子、恋をする</t>
+          <t>くらいあの子としたいこと</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>音竹 ひかる(著者)</t>
+          <t>碇マナツ(著者)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第10話</t>
+          <t>第95話</t>
         </is>
       </c>
     </row>
@@ -38690,17 +39727,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
+          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
+          <t>FUNA 東西 モトエ恵介</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第41話</t>
+          <t>第128話　襲撃［その７］</t>
         </is>
       </c>
     </row>
@@ -38710,17 +39747,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+          <t>はぐはぐ(著者)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第4話(2)</t>
+          <t>第97話</t>
         </is>
       </c>
     </row>
@@ -38730,17 +39767,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+          <t>セレビィ量産型(著者)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>第26話後半</t>
         </is>
       </c>
     </row>
@@ -38750,17 +39787,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>世界最高の暗殺者、異世界貴族に転生する</t>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>月夜涙(原作) 皇ハマオ(漫画) れい亜(キャラクター原案)</t>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第42話-1</t>
+          <t>第23話②</t>
         </is>
       </c>
     </row>
@@ -38770,17 +39807,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>オタクに優しいギャルはいない!?</t>
+          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>のりしろちゃん 魚住さかな</t>
+          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>【#185】ベッドの上の葛藤</t>
+          <t>第63話　逢魔が刻</t>
         </is>
       </c>
     </row>
@@ -38790,17 +39827,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ダメ人間の愛しかた</t>
+          <t>塔の管理をしてみよう</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>岩葉(著者)</t>
+          <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第25話後編　ダメ人間と彼女たちのクリスマス</t>
+          <t>第99話後編</t>
         </is>
       </c>
     </row>
@@ -38810,17 +39847,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ひとりぼっちの異世界攻略</t>
+          <t>おせっかい女子、恋をする</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>びび（漫画） 五示正司（原作）</t>
+          <t>音竹 ひかる(著者)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第264話　最後は悦んでた？</t>
+          <t>第11話</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-04-20
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -50,6 +50,7 @@
     <sheet name="2026-03-30" sheetId="42" state="visible" r:id="rId42"/>
     <sheet name="2026-04-06" sheetId="43" state="visible" r:id="rId43"/>
     <sheet name="2026-04-13" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="2026-04-20" sheetId="45" state="visible" r:id="rId45"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -38862,22 +38863,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第46話➁</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>不徳のギルド</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>河添太一</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第１０５話：丸裸の思い</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第37話：キモい動き①</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第9話 前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第７６話『渦中停止』①</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第７７話　音ゲーの戦いが始まった（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第149話	有栖の足つぼ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第40話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>ダンジョンの幼なじみ</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>久真やすひさ(著者)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第63話</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第18話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第320話</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>番外編</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第12話</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>番外編②</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第88話</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第142話　テレジア参戦！・後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第93話　幻影魔法(イリュージョン)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第135話　王都炎上Ⅱ（中編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>魔のものたちは企てる</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>加藤拓弐(原作) ガしガし(作画)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第36話</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>淫獄団地</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第56話（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第80話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第3話 ちゅう</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>久遠まこと(著者) 石のやっさん(原作)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>休載イラスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第38話 独身貴族は野鳥を撮りたい（3）</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>孤島の主のミステリーですわ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>美人女上司滝沢さん</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>やんBARU(著者)</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第217話</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>休載イラスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>アザミヤコを好きになる</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第15話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>ケツバトラー</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>高出なおたか ©面白法人カヤック／小学館</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第32話</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第64話②　鍛冶を見学してみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第47話　奴のともだち（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第7話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第2話-①</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>KAKERU</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第75話「魔術師の森（お呼ばれ）」（前半）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 林たかあき</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第67話 闘志</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>拷問178</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>クシザキ</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第8話	教育者Xの献身</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>理想のヒモ生活</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第106話　その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第４６話　勇者、ラファエルとのRAPバトルでドープな韻のパンチライン＆ディープなリリックはアゲアゲで会場を沸かす（５）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>原作:剃り残し 漫画:大窪太一</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第6話</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第86話(後編)その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第134話</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第95話</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>FUNA 東西 モトエ恵介</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第128話　襲撃［その７］</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>はぐはぐ(著者)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第97話</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第26話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第23話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第63話　逢魔が刻</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>塔の管理をしてみよう</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第99話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第11話</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>魔術師クノンは見えている</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第46話➁</t>
+          <t>第135話</t>
         </is>
       </c>
     </row>
@@ -38887,17 +39924,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>不徳のギルド</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>河添太一</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第１０５話：丸裸の思い</t>
+          <t>225撃目</t>
         </is>
       </c>
     </row>
@@ -38907,17 +39944,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+          <t>異世界おじさん</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>zunta(作画) はらわたさいぞう(原作)</t>
+          <t>殆ど死んでいる(著者)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第37話：キモい動き①</t>
+          <t>コミックス第15巻発売告知</t>
         </is>
       </c>
     </row>
@@ -38927,17 +39964,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第9話 前編</t>
+          <t>第37話：キモい動き②</t>
         </is>
       </c>
     </row>
@@ -38947,17 +39984,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第７６話『渦中停止』①</t>
+          <t>第22話-2「子供たちはどこだ？」</t>
         </is>
       </c>
     </row>
@@ -38977,7 +40014,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第７７話　音ゲーの戦いが始まった（１）</t>
+          <t>第７７話　音ゲーの戦いが始まった（２）</t>
         </is>
       </c>
     </row>
@@ -38987,17 +40024,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第149話	有栖の足つぼ！</t>
+          <t>第７６話『渦中停止』②</t>
         </is>
       </c>
     </row>
@@ -39007,17 +40044,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+          <t>いとこのこ</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+          <t>いぬちく(著者)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第40話①</t>
+          <t>第49話</t>
         </is>
       </c>
     </row>
@@ -39027,17 +40064,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ダンジョンの幼なじみ</t>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>久真やすひさ(著者)</t>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第63話</t>
+          <t>第85話その2</t>
         </is>
       </c>
     </row>
@@ -39047,17 +40084,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第18話-1</t>
+          <t>第8話</t>
         </is>
       </c>
     </row>
@@ -39067,17 +40104,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>異世界のんびり農家</t>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第320話</t>
+          <t>第21話後半</t>
         </is>
       </c>
     </row>
@@ -39087,17 +40124,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>帰ってください！ 阿久津さん</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>長岡太一(著者)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>番外編</t>
+          <t>番外編㉗</t>
         </is>
       </c>
     </row>
@@ -39107,17 +40144,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
+          <t>まんきつしたい常連さん</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
+          <t>しんみりん(著者)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第12話</t>
+          <t>第55話中編</t>
         </is>
       </c>
     </row>
@@ -39127,17 +40164,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>番外編②</t>
+          <t>第５９話　新メンバーを迎える器用貧乏（２）</t>
         </is>
       </c>
     </row>
@@ -39147,17 +40184,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ダークサモナーとデキている</t>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>車王(著者)</t>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第88話</t>
+          <t>第8話-2</t>
         </is>
       </c>
     </row>
@@ -39167,17 +40204,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>異世界のんびり農家</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第142話　テレジア参戦！・後編</t>
+          <t>第321話</t>
         </is>
       </c>
     </row>
@@ -39187,17 +40224,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>板垣恵介 猪原賽 陸井栄史</t>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第93話　幻影魔法(イリュージョン)</t>
+          <t>第38話</t>
         </is>
       </c>
     </row>
@@ -39207,17 +40244,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第135話　王都炎上Ⅱ（中編）</t>
+          <t>第143話　ラスト４人！・前編</t>
         </is>
       </c>
     </row>
@@ -39227,17 +40264,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>魔のものたちは企てる</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>加藤拓弐(原作) ガしガし(作画)</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第36話</t>
+          <t>第135話　王都炎上Ⅱ（後編）</t>
         </is>
       </c>
     </row>
@@ -39247,17 +40284,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>淫獄団地</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第56話（後編）</t>
+          <t>第4話②</t>
         </is>
       </c>
     </row>
@@ -39277,7 +40314,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第80話①</t>
+          <t>第80話➁</t>
         </is>
       </c>
     </row>
@@ -39287,17 +40324,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+          <t>望まぬ不死の冒険者</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+          <t>中曽根ハイジ（漫画） 丘野 優（原作） じゃいあん（キャラクター原案）</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第3話 ちゅう</t>
+          <t>第64話　対立</t>
         </is>
       </c>
     </row>
@@ -39307,17 +40344,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
+          <t>アザミヤコを好きになる</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>久遠まこと(著者) 石のやっさん(原作)</t>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>休載イラスト</t>
+          <t>コミックス第3巻発売告知！</t>
         </is>
       </c>
     </row>
@@ -39327,17 +40364,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第38話 独身貴族は野鳥を撮りたい（3）</t>
+          <t>第44話-2</t>
         </is>
       </c>
     </row>
@@ -39367,17 +40404,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>美人女上司滝沢さん</t>
+          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>やんBARU(著者)</t>
+          <t>夜州 nini 藻</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第217話</t>
+          <t>第73話(後編)</t>
         </is>
       </c>
     </row>
@@ -39387,17 +40424,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>休載イラスト</t>
+          <t>第38話 独身貴族は野鳥を撮りたい（4）</t>
         </is>
       </c>
     </row>
@@ -39407,17 +40444,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>アザミヤコを好きになる</t>
+          <t>お気楽領主の楽しい領地防衛 ～生産系魔術で名もなき村を最強の城塞都市に～</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+          <t>青色まろ（漫画） 赤池宗（原作） 転（原作イラスト）</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第15話前編</t>
+          <t>第39話　覚悟の戦い</t>
         </is>
       </c>
     </row>
@@ -39427,17 +40464,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ケツバトラー</t>
+          <t>聖者無双</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>高出なおたか ©面白法人カヤック／小学館</t>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第32話</t>
+          <t>第97話　消えた魔物の死体・蟻の生態②</t>
         </is>
       </c>
     </row>
@@ -39447,17 +40484,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第64話②　鍛冶を見学してみた</t>
+          <t>第13話-2：思い出の写真</t>
         </is>
       </c>
     </row>
@@ -39467,17 +40504,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第47話　奴のともだち（前編）</t>
+          <t>第152話 よくわからないけれど酒と潮と男と女みたいです（１）</t>
         </is>
       </c>
     </row>
@@ -39487,17 +40524,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第7話-1</t>
+          <t>第31話②</t>
         </is>
       </c>
     </row>
@@ -39507,17 +40544,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+          <t>久遠まこと(著者) 石のやっさん(原作)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第2話-①</t>
+          <t>コミックス７巻発売告知</t>
         </is>
       </c>
     </row>
@@ -39527,17 +40564,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>KAKERU</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第75話「魔術師の森（お呼ばれ）」（前半）</t>
+          <t>拷問179</t>
         </is>
       </c>
     </row>
@@ -39547,17 +40584,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>板垣恵介 林たかあき</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第67話 闘志</t>
+          <t>第４７話　勇者、神々にメンチを切る。そしてエリーゼ、闇堕ちする（１）</t>
         </is>
       </c>
     </row>
@@ -39567,17 +40604,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>クール教信者</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>拷問178</t>
+          <t>第164話</t>
         </is>
       </c>
     </row>
@@ -39587,17 +40624,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>お前がヤったんだろ！</t>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>クシザキ</t>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第8話	教育者Xの献身</t>
+          <t>第85話 島田、一筋の涙!!!</t>
         </is>
       </c>
     </row>
@@ -39607,17 +40644,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>理想のヒモ生活</t>
+          <t>俺は星間国家の悪徳領主！</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
+          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第106話　その2</t>
+          <t>第46話　王者の戦い方（前編）</t>
         </is>
       </c>
     </row>
@@ -39627,17 +40664,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>インフィニット・デンドログラム</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第４６話　勇者、ラファエルとのRAPバトルでドープな韻のパンチライン＆ディープなリリックはアゲアゲで会場を沸かす（５）</t>
+          <t>第77話</t>
         </is>
       </c>
     </row>
@@ -39647,17 +40684,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>原作:剃り残し 漫画:大窪太一</t>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第6話</t>
+          <t>第8話-2：子供の守り神</t>
         </is>
       </c>
     </row>
@@ -39667,17 +40704,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>最弱テイマーはゴミ拾いの旅を始めました。@COMIC</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>漫画：蕗野 冬 原作：ほのぼのる500 キャラクター原案：なま</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第86話(後編)その2</t>
+          <t>第30話 ①</t>
         </is>
       </c>
     </row>
@@ -39687,17 +40724,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>宇崎ちゃんは遊びたい！</t>
+          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>丈(著者)</t>
+          <t>六志麻あさ 業務用餅 kisui</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第134話</t>
+          <t>第８５話</t>
         </is>
       </c>
     </row>
@@ -39707,17 +40744,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>めっちゃ召喚された件 THE COMIC</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第95話</t>
+          <t>12巻発売＆お知らせ!!</t>
         </is>
       </c>
     </row>
@@ -39727,17 +40764,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>FUNA 東西 モトエ恵介</t>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第128話　襲撃［その７］</t>
+          <t>第8話-1</t>
         </is>
       </c>
     </row>
@@ -39747,17 +40784,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>サーシャちゃんとクラスメイトオタクくん</t>
+          <t>ライブダンジョン！</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>はぐはぐ(著者)</t>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第97話</t>
+          <t>第95話前半</t>
         </is>
       </c>
     </row>
@@ -39767,17 +40804,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>三枝さんはメガネ先輩と恋を描く</t>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>セレビィ量産型(著者)</t>
+          <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第26話後半</t>
+          <t>第19話　最弱貴族、魔王と聖女を仲裁する（４）</t>
         </is>
       </c>
     </row>
@@ -39787,17 +40824,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+          <t>おせっかい女子、恋をする</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+          <t>音竹 ひかる(著者)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第23話②</t>
+          <t>第12話</t>
         </is>
       </c>
     </row>
@@ -39807,17 +40844,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
+          <t>アイドル辞めるけど結婚してくれますか!?</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
+          <t>三吉汐美(著者)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第63話　逢魔が刻</t>
+          <t>休載イラスト</t>
         </is>
       </c>
     </row>
@@ -39827,17 +40864,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>塔の管理をしてみよう</t>
+          <t>Lv２からチートだった元勇者候補のまったり異世界ライフ</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
+          <t>糸町秋音（漫画） 鬼ノ城ミヤ（原作） 片桐（キャラクター原案）</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第99話後編</t>
+          <t>第67話　うわさ話</t>
         </is>
       </c>
     </row>
@@ -39847,17 +40884,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>おせっかい女子、恋をする</t>
+          <t>迷宮の王</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>音竹 ひかる(著者)</t>
+          <t>漫画：K9 脚本：小林裕和 原作：支援BIS</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第11話</t>
+          <t>第十七話　血戦（二）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-04-27
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -51,6 +51,7 @@
     <sheet name="2026-04-06" sheetId="43" state="visible" r:id="rId43"/>
     <sheet name="2026-04-13" sheetId="44" state="visible" r:id="rId44"/>
     <sheet name="2026-04-20" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="2026-04-27" sheetId="46" state="visible" r:id="rId46"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -39899,22 +39900,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第135話</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>ワンパンマン</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>225撃目</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>異世界おじさん</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>殆ど死んでいる(著者)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>コミックス第15巻発売告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第37話：キモい動き②</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第22話-2「子供たちはどこだ？」</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第７７話　音ゲーの戦いが始まった（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第７６話『渦中停止』②</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>いとこのこ</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>いぬちく(著者)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第49話</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第85話その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第8話</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第21話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>帰ってください！ 阿久津さん</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>長岡太一(著者)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>番外編㉗</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>まんきつしたい常連さん</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>しんみりん(著者)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第55話中編</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第５９話　新メンバーを迎える器用貧乏（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第8話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第321話</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第38話</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第143話　ラスト４人！・前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第135話　王都炎上Ⅱ（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第4話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第80話➁</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>望まぬ不死の冒険者</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>中曽根ハイジ（漫画） 丘野 優（原作） じゃいあん（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第64話　対立</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>アザミヤコを好きになる</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>コミックス第3巻発売告知！</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第44話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>孤島の主のミステリーですわ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>夜州 nini 藻</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第73話(後編)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第38話 独身貴族は野鳥を撮りたい（4）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>お気楽領主の楽しい領地防衛 ～生産系魔術で名もなき村を最強の城塞都市に～</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>青色まろ（漫画） 赤池宗（原作） 転（原作イラスト）</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第39話　覚悟の戦い</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>聖者無双</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第97話　消えた魔物の死体・蟻の生態②</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第13話-2：思い出の写真</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第152話 よくわからないけれど酒と潮と男と女みたいです（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第31話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>久遠まこと(著者) 石のやっさん(原作)</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>コミックス７巻発売告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>拷問179</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第４７話　勇者、神々にメンチを切る。そしてエリーゼ、闇堕ちする（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>小林さんちのメイドラゴン</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>クール教信者</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第164話</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第85話 島田、一筋の涙!!!</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>俺は星間国家の悪徳領主！</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第46話　王者の戦い方（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>インフィニット・デンドログラム</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第77話</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第8話-2：子供の守り神</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>最弱テイマーはゴミ拾いの旅を始めました。@COMIC</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>漫画：蕗野 冬 原作：ほのぼのる500 キャラクター原案：なま</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第30話 ①</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>六志麻あさ 業務用餅 kisui</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第８５話</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>めっちゃ召喚された件 THE COMIC</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>12巻発売＆お知らせ!!</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第8話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>ライブダンジョン！</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第95話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>空野進 sorani ファルまろ</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第19話　最弱貴族、魔王と聖女を仲裁する（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第12話</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>アイドル辞めるけど結婚してくれますか!?</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>三吉汐美(著者)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>休載イラスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>Lv２からチートだった元勇者候補のまったり異世界ライフ</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>糸町秋音（漫画） 鬼ノ城ミヤ（原作） 片桐（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第67話　うわさ話</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>迷宮の王</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>漫画：K9 脚本：小林裕和 原作：支援BIS</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第十七話　血戦（二）</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>宇崎ちゃんは遊びたい！</t>
+          <t>異世界おじさん</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>丈(著者)</t>
+          <t>殆ど死んでいる(著者)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第135話</t>
+          <t>第76話</t>
         </is>
       </c>
     </row>
@@ -39924,17 +40961,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ワンパンマン</t>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>原作/ＯＮＥ 作画/村田雄介</t>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>225撃目</t>
+          <t>第78話</t>
         </is>
       </c>
     </row>
@@ -39944,17 +40981,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>異世界おじさん</t>
+          <t>異種族レビュアーズ</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>殆ど死んでいる(著者)</t>
+          <t>天原(原作) masha(作画)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>コミックス第15巻発売告知</t>
+          <t>第92話</t>
         </is>
       </c>
     </row>
@@ -39974,7 +41011,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第37話：キモい動き②</t>
+          <t>第37話：キモい動き③</t>
         </is>
       </c>
     </row>
@@ -39984,17 +41021,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+          <t>むちまろ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第22話-2「子供たちはどこだ？」</t>
+          <t>第150話	有栖の足つぼ！（会長編）</t>
         </is>
       </c>
     </row>
@@ -40004,17 +41041,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第７７話　音ゲーの戦いが始まった（２）</t>
+          <t>第７６話『渦中停止』③</t>
         </is>
       </c>
     </row>
@@ -40024,17 +41061,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第７６話『渦中停止』②</t>
+          <t>第７８話　神輿の戦いが始まった（１）</t>
         </is>
       </c>
     </row>
@@ -40044,17 +41081,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>いとこのこ</t>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>いぬちく(著者)</t>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第49話</t>
+          <t>第40話②</t>
         </is>
       </c>
     </row>
@@ -40064,17 +41101,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第85話その2</t>
+          <t>第18話-2</t>
         </is>
       </c>
     </row>
@@ -40084,17 +41121,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+          <t>クセ強彼女は床にいざなう</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+          <t>須河篤志(著者)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第8話</t>
+          <t>第21話前半</t>
         </is>
       </c>
     </row>
@@ -40104,17 +41141,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第21話後半</t>
+          <t>第94話　キング・ヒュドラー拳‼</t>
         </is>
       </c>
     </row>
@@ -40124,17 +41161,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>帰ってください！ 阿久津さん</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>長岡太一(著者)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>番外編㉗</t>
+          <t>第５９話　新メンバーを迎える器用貧乏（３）</t>
         </is>
       </c>
     </row>
@@ -40144,17 +41181,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>まんきつしたい常連さん</t>
+          <t>ダークサモナーとデキている</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>しんみりん(著者)</t>
+          <t>車王(著者)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第55話中編</t>
+          <t>第89話</t>
         </is>
       </c>
     </row>
@@ -40164,17 +41201,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>異世界のんびり農家</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第５９話　新メンバーを迎える器用貧乏（２）</t>
+          <t>第322話</t>
         </is>
       </c>
     </row>
@@ -40184,17 +41221,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>三部べべ(漫画) ねうしとら(原作)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第8話-2</t>
+          <t>第143話　ラスト４人！・後編</t>
         </is>
       </c>
     </row>
@@ -40204,17 +41241,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>異世界のんびり農家</t>
+          <t>ぽんドロイド！ はまさん</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+          <t>はれやまはれぞう(著者)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第321話</t>
+          <t>第19話</t>
         </is>
       </c>
     </row>
@@ -40224,17 +41261,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第38話</t>
+          <t>第80話③</t>
         </is>
       </c>
     </row>
@@ -40244,17 +41281,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>淫獄団地</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第143話　ラスト４人！・前編</t>
+          <t>第57話（前編）</t>
         </is>
       </c>
     </row>
@@ -40264,17 +41301,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第135話　王都炎上Ⅱ（後編）</t>
+          <t>第4話 吸血鬼ハンター</t>
         </is>
       </c>
     </row>
@@ -40284,17 +41321,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>美人女上司滝沢さん</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>やんBARU(著者)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第4話②</t>
+          <t>第218話</t>
         </is>
       </c>
     </row>
@@ -40304,17 +41341,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>モリタ Ｕ４ nima</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第80話➁</t>
+          <t>第16話（１）　太っちょ貴族と摩訶不思議なる肉料理　（１）</t>
         </is>
       </c>
     </row>
@@ -40324,17 +41361,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>望まぬ不死の冒険者</t>
+          <t>骸骨騎士様、只今異世界へお出掛け中</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>中曽根ハイジ（漫画） 丘野 優（原作） じゃいあん（キャラクター原案）</t>
+          <t>サワノアキラ（漫画） 秤猿鬼（原作） KeG（キャラクター原案）</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第64話　対立</t>
+          <t>第67話　エルフ族の決断Ⅵ</t>
         </is>
       </c>
     </row>
@@ -40344,17 +41381,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>アザミヤコを好きになる</t>
+          <t>英雄王、武を極めるため転生す ～そして、世界最強の見習い騎士♀～</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+          <t>漫画‥くろむら基人 原作‥ハヤケン キャラクター原案‥Nagu</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>コミックス第3巻発売告知！</t>
+          <t>第33話 後編</t>
         </is>
       </c>
     </row>
@@ -40364,17 +41401,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第44話-2</t>
+          <t>第47話　奴のともだち（後編）</t>
         </is>
       </c>
     </row>
@@ -40384,17 +41421,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>島知宏 音速炒飯 有都あらゆる</t>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>孤島の主のミステリーですわ！</t>
+          <t>第9話前編</t>
         </is>
       </c>
     </row>
@@ -40404,17 +41441,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
+          <t>濁る瞳で何を願う ハイセルク戦記</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>夜州 nini 藻</t>
+          <t>トルトネン 創-taro 斎藤八呑</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第73話(後編)</t>
+          <t>第39話 亡者の矜持</t>
         </is>
       </c>
     </row>
@@ -40424,17 +41461,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第38話 独身貴族は野鳥を撮りたい（4）</t>
+          <t>第152話 よくわからないけれど酒と潮と男と女みたいです（２）</t>
         </is>
       </c>
     </row>
@@ -40444,17 +41481,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>お気楽領主の楽しい領地防衛 ～生産系魔術で名もなき村を最強の城塞都市に～</t>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>青色まろ（漫画） 赤池宗（原作） 転（原作イラスト）</t>
+          <t>板垣恵介 林たかあき</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第39話　覚悟の戦い</t>
+          <t>第68話 愛煙家</t>
         </is>
       </c>
     </row>
@@ -40464,17 +41501,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>聖者無双</t>
+          <t>物語の黒幕に転生して</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第97話　消えた魔物の死体・蟻の生態②</t>
+          <t>第40話　その2</t>
         </is>
       </c>
     </row>
@@ -40484,17 +41521,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第13話-2：思い出の写真</t>
+          <t>第135話</t>
         </is>
       </c>
     </row>
@@ -40504,17 +41541,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第152話 よくわからないけれど酒と潮と男と女みたいです（１）</t>
+          <t>第30話</t>
         </is>
       </c>
     </row>
@@ -40524,17 +41561,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>女友達は頼めば意外とヤらせてくれる</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ろくろ(漫画) 鏡遊(原作)</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第31話②</t>
+          <t>第65話①　魔人と戦ってみた</t>
         </is>
       </c>
     </row>
@@ -40544,17 +41581,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>久遠まこと(著者) 石のやっさん(原作)</t>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>コミックス７巻発売告知</t>
+          <t>第7話-2</t>
         </is>
       </c>
     </row>
@@ -40564,17 +41601,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>拷問179</t>
+          <t>第４７話　勇者、神々にメンチを切る。そしてエリーゼ、闇堕ちする（２）</t>
         </is>
       </c>
     </row>
@@ -40584,17 +41621,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第４７話　勇者、神々にメンチを切る。そしてエリーゼ、闇堕ちする（１）</t>
+          <t>第86話(後編)その3</t>
         </is>
       </c>
     </row>
@@ -40604,17 +41641,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>小林さんちのメイドラゴン</t>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>クール教信者</t>
+          <t>KAKERU</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第164話</t>
+          <t>第75話「魔術師の森（お呼ばれ）」（後半）</t>
         </is>
       </c>
     </row>
@@ -40624,17 +41661,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第85話 島田、一筋の涙!!!</t>
+          <t>拷問180</t>
         </is>
       </c>
     </row>
@@ -40644,17 +41681,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>俺は星間国家の悪徳領主！</t>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
+          <t>原作:剃り残し 漫画:大窪太一</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第46話　王者の戦い方（前編）</t>
+          <t>第7話</t>
         </is>
       </c>
     </row>
@@ -40664,17 +41701,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>インフィニット・デンドログラム</t>
+          <t>お前がヤったんだろ！</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
+          <t>クシザキ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第77話</t>
+          <t>第9話	ホクロは残されたまま</t>
         </is>
       </c>
     </row>
@@ -40684,17 +41721,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+          <t>くらいあの子としたいこと</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+          <t>碇マナツ(著者)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第8話-2：子供の守り神</t>
+          <t>第96話</t>
         </is>
       </c>
     </row>
@@ -40704,17 +41741,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>最弱テイマーはゴミ拾いの旅を始めました。@COMIC</t>
+          <t>俺は星間国家の悪徳領主！</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>漫画：蕗野 冬 原作：ほのぼのる500 キャラクター原案：なま</t>
+          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第30話 ①</t>
+          <t>第46話　王者の戦い方（後編）</t>
         </is>
       </c>
     </row>
@@ -40724,17 +41761,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
+          <t>バーサス</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>六志麻あさ 業務用餅 kisui</t>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第８５話</t>
+          <t>第33話 本物の勇者（前編-2）</t>
         </is>
       </c>
     </row>
@@ -40744,17 +41781,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>めっちゃ召喚された件 THE COMIC</t>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>12巻発売＆お知らせ!!</t>
+          <t>第23話③</t>
         </is>
       </c>
     </row>
@@ -40764,17 +41801,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+          <t>おせっかい女子、恋をする</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+          <t>音竹 ひかる(著者)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第8話-1</t>
+          <t>第13話</t>
         </is>
       </c>
     </row>
@@ -40784,17 +41821,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ライブダンジョン！</t>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+          <t>セレビィ量産型(著者)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第95話前半</t>
+          <t>第26.5話</t>
         </is>
       </c>
     </row>
@@ -40804,17 +41841,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+          <t>アザミヤコを好きになる</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>空野進 sorani ファルまろ</t>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第19話　最弱貴族、魔王と聖女を仲裁する（４）</t>
+          <t>コミックス3巻PR</t>
         </is>
       </c>
     </row>
@@ -40824,17 +41861,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>おせっかい女子、恋をする</t>
+          <t>塔の管理をしてみよう</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>音竹 ひかる(著者)</t>
+          <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第12話</t>
+          <t>第100話前編</t>
         </is>
       </c>
     </row>
@@ -40844,17 +41881,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>アイドル辞めるけど結婚してくれますか!?</t>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>三吉汐美(著者)</t>
+          <t>漫画/すたひろ 原作/Y.A</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>休載イラスト</t>
+          <t>chapter84【44話①】</t>
         </is>
       </c>
     </row>
@@ -40864,17 +41901,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Lv２からチートだった元勇者候補のまったり異世界ライフ</t>
+          <t>幼女戦記</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>糸町秋音（漫画） 鬼ノ城ミヤ（原作） 片桐（キャラクター原案）</t>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第67話　うわさ話</t>
+          <t>第百十四章：ドードーバード航空戦Ⅸ</t>
         </is>
       </c>
     </row>
@@ -40884,17 +41921,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>迷宮の王</t>
+          <t>回復術士のやり直し</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>漫画：K9 脚本：小林裕和 原作：支援BIS</t>
+          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第十七話　血戦（二）</t>
+          <t>第77話-2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-05-04
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -52,6 +52,7 @@
     <sheet name="2026-04-13" sheetId="44" state="visible" r:id="rId44"/>
     <sheet name="2026-04-20" sheetId="45" state="visible" r:id="rId45"/>
     <sheet name="2026-04-27" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="2026-05-04" sheetId="47" state="visible" r:id="rId47"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -40936,22 +40937,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>異世界おじさん</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>殆ど死んでいる(著者)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第76話</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第78話</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>異種族レビュアーズ</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>天原(原作) masha(作画)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第92話</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第37話：キモい動き③</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第150話	有栖の足つぼ！（会長編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第７６話『渦中停止』③</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第７８話　神輿の戦いが始まった（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第40話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第18話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第21話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第94話　キング・ヒュドラー拳‼</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第５９話　新メンバーを迎える器用貧乏（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第89話</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第322話</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第143話　ラスト４人！・後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>ぽんドロイド！ はまさん</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>はれやまはれぞう(著者)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第19話</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第80話③</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>淫獄団地</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第57話（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第4話 吸血鬼ハンター</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>美人女上司滝沢さん</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>やんBARU(著者)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第218話</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>モリタ Ｕ４ nima</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第16話（１）　太っちょ貴族と摩訶不思議なる肉料理　（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>骸骨騎士様、只今異世界へお出掛け中</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>サワノアキラ（漫画） 秤猿鬼（原作） KeG（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第67話　エルフ族の決断Ⅵ</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>英雄王、武を極めるため転生す ～そして、世界最強の見習い騎士♀～</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>漫画‥くろむら基人 原作‥ハヤケン キャラクター原案‥Nagu</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第33話 後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第47話　奴のともだち（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第9話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>濁る瞳で何を願う ハイセルク戦記</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>トルトネン 創-taro 斎藤八呑</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第39話 亡者の矜持</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第152話 よくわからないけれど酒と潮と男と女みたいです（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 林たかあき</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第68話 愛煙家</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>物語の黒幕に転生して</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第40話　その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第135話</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第30話</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第65話①　魔人と戦ってみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第7話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第４７話　勇者、神々にメンチを切る。そしてエリーゼ、闇堕ちする（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第86話(後編)その3</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>KAKERU</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第75話「魔術師の森（お呼ばれ）」（後半）</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>拷問180</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>原作:剃り残し 漫画:大窪太一</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第7話</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>クシザキ</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第9話	ホクロは残されたまま</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第96話</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>俺は星間国家の悪徳領主！</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第46話　王者の戦い方（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>バーサス</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第33話 本物の勇者（前編-2）</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第23話③</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第13話</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第26.5話</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>アザミヤコを好きになる</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>コミックス3巻PR</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>塔の管理をしてみよう</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第100話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>漫画/すたひろ 原作/Y.A</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>chapter84【44話①】</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>幼女戦記</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第百十四章：ドードーバード航空戦Ⅸ</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>回復術士のやり直し</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第77話-2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>異世界おじさん</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>殆ど死んでいる(著者)</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第76話</t>
+          <t>226撃目</t>
         </is>
       </c>
     </row>
@@ -40961,17 +41998,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+          <t>魔術師クノンは見えている</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第78話</t>
+          <t>第47話</t>
         </is>
       </c>
     </row>
@@ -40981,17 +42018,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>異種族レビュアーズ</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>天原(原作) masha(作画)</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第92話</t>
+          <t>第22話-3「子供たちはどこだ？」</t>
         </is>
       </c>
     </row>
@@ -41001,17 +42038,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>zunta(作画) はらわたさいぞう(原作)</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第37話：キモい動き③</t>
+          <t>第７６話『渦中停止』④</t>
         </is>
       </c>
     </row>
@@ -41021,17 +42058,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第150話	有栖の足つぼ！（会長編）</t>
+          <t>第78話</t>
         </is>
       </c>
     </row>
@@ -41041,17 +42078,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第７６話『渦中停止』③</t>
+          <t>第9話 後編</t>
         </is>
       </c>
     </row>
@@ -41071,7 +42108,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第７８話　神輿の戦いが始まった（１）</t>
+          <t>第７８話　神輿の戦いが始まった（２）</t>
         </is>
       </c>
     </row>
@@ -41081,17 +42118,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第40話②</t>
+          <t>第9話</t>
         </is>
       </c>
     </row>
@@ -41101,17 +42138,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+          <t>いとこのこ</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+          <t>いぬちく(著者)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第18話-2</t>
+          <t>第50話</t>
         </is>
       </c>
     </row>
@@ -41121,17 +42158,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>帰ってください！ 阿久津さん</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>長岡太一(著者)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第21話前半</t>
+          <t>第205話</t>
         </is>
       </c>
     </row>
@@ -41141,17 +42178,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>板垣恵介 猪原賽 陸井栄史</t>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第94話　キング・ヒュドラー拳‼</t>
+          <t>【募集開始】人気投票＆キャラへの質問大募集！【第13巻発売記念】</t>
         </is>
       </c>
     </row>
@@ -41161,17 +42198,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>まんきつしたい常連さん</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>しんみりん(著者)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第５９話　新メンバーを迎える器用貧乏（３）</t>
+          <t>第55話後編</t>
         </is>
       </c>
     </row>
@@ -41181,17 +42218,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ダークサモナーとデキている</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>車王(著者)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第89話</t>
+          <t>おまけ72</t>
         </is>
       </c>
     </row>
@@ -41201,17 +42238,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>異世界のんびり農家</t>
+          <t>不純な彼女達は懺悔しない</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+          <t>ポロロッカ(著者)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第322話</t>
+          <t>第38話</t>
         </is>
       </c>
     </row>
@@ -41221,17 +42258,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>「おかえり、パパ」</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>蝉丸</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第143話　ラスト４人！・後編</t>
+          <t>第35話　水族館</t>
         </is>
       </c>
     </row>
@@ -41241,17 +42278,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ぽんドロイド！ はまさん</t>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>はれやまはれぞう(著者)</t>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第19話</t>
+          <t>第9話-1</t>
         </is>
       </c>
     </row>
@@ -41261,17 +42298,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第80話③</t>
+          <t>第５９話　新メンバーを迎える器用貧乏（４）</t>
         </is>
       </c>
     </row>
@@ -41281,17 +42318,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>淫獄団地</t>
+          <t>剥かせて！竜ケ崎さん</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+          <t>一智和智</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第57話（前編）</t>
+          <t>大学生編 第20話</t>
         </is>
       </c>
     </row>
@@ -41301,17 +42338,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第4話 吸血鬼ハンター</t>
+          <t>第80話④</t>
         </is>
       </c>
     </row>
@@ -41321,17 +42358,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>美人女上司滝沢さん</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>やんBARU(著者)</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第218話</t>
+          <t>第4話③</t>
         </is>
       </c>
     </row>
@@ -41341,17 +42378,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+          <t>田舎で恋は難しい!?</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>モリタ Ｕ４ nima</t>
+          <t>ねこうめ(著者)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第16話（１）　太っちょ貴族と摩訶不思議なる肉料理　（１）</t>
+          <t>第7話</t>
         </is>
       </c>
     </row>
@@ -41361,17 +42398,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>骸骨騎士様、只今異世界へお出掛け中</t>
+          <t>異世界食堂　洋食のねこや</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>サワノアキラ（漫画） 秤猿鬼（原作） KeG（キャラクター原案）</t>
+          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第67話　エルフ族の決断Ⅵ</t>
+          <t>第46話(前半)</t>
         </is>
       </c>
     </row>
@@ -41381,17 +42418,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>英雄王、武を極めるため転生す ～そして、世界最強の見習い騎士♀～</t>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>漫画‥くろむら基人 原作‥ハヤケン キャラクター原案‥Nagu</t>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第33話 後編</t>
+          <t>第2話-②</t>
         </is>
       </c>
     </row>
@@ -41401,17 +42438,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第47話　奴のともだち（後編）</t>
+          <t>第65話②　魔人と戦ってみた</t>
         </is>
       </c>
     </row>
@@ -41421,17 +42458,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+          <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+          <t>安田剛助(著者)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第9話前編</t>
+          <t>第56話</t>
         </is>
       </c>
     </row>
@@ -41441,17 +42478,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>濁る瞳で何を願う ハイセルク戦記</t>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>トルトネン 創-taro 斎藤八呑</t>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第39話 亡者の矜持</t>
+          <t>第14話-1：これからも一緒に</t>
         </is>
       </c>
     </row>
@@ -41461,17 +42498,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第152話 よくわからないけれど酒と潮と男と女みたいです（２）</t>
+          <t>第４７話　勇者、神々にメンチを切る。そしてエリーゼ、闇堕ちする（３）</t>
         </is>
       </c>
     </row>
@@ -41481,17 +42518,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+          <t>クセ強彼女は床にいざなう</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>板垣恵介 林たかあき</t>
+          <t>須河篤志(著者)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第68話 愛煙家</t>
+          <t>コミックス告知</t>
         </is>
       </c>
     </row>
@@ -41501,17 +42538,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>物語の黒幕に転生して</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第40話　その2</t>
+          <t>拷問181</t>
         </is>
       </c>
     </row>
@@ -41521,17 +42558,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>宇崎ちゃんは遊びたい！</t>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>丈(著者)</t>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第135話</t>
+          <t>第32話①</t>
         </is>
       </c>
     </row>
@@ -41541,17 +42578,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
+          <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
+          <t>クール教信者</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第30話</t>
+          <t>第165話</t>
         </is>
       </c>
     </row>
@@ -41561,17 +42598,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第65話①　魔人と戦ってみた</t>
+          <t>第87話その1</t>
         </is>
       </c>
     </row>
@@ -41581,17 +42618,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+          <t>異世界黙示録マイノグーラ ～破滅の文明で始める世界征服～</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+          <t>緑華野菜子(著者) 鹿角フェフ(原作) じゅん(キャラクター原案)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第7話-2</t>
+          <t>第32話　真と偽①</t>
         </is>
       </c>
     </row>
@@ -41601,17 +42638,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>ライブダンジョン！</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第４７話　勇者、神々にメンチを切る。そしてエリーゼ、闇堕ちする（２）</t>
+          <t>第95話後半</t>
         </is>
       </c>
     </row>
@@ -41621,17 +42658,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第86話(後編)その3</t>
+          <t>第9話-1：父親として</t>
         </is>
       </c>
     </row>
@@ -41641,17 +42678,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>KAKERU</t>
+          <t>六志麻あさ 業務用餅 kisui</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第75話「魔術師の森（お呼ばれ）」（後半）</t>
+          <t>第８６話</t>
         </is>
       </c>
     </row>
@@ -41661,17 +42698,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>拷問180</t>
+          <t>第8話-2</t>
         </is>
       </c>
     </row>
@@ -41681,17 +42718,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+          <t>オタクに優しいギャルはいない!?</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>原作:剃り残し 漫画:大窪太一</t>
+          <t>のりしろちゃん 魚住さかな</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第7話</t>
+          <t>【#189】ごまかしあまね</t>
         </is>
       </c>
     </row>
@@ -41701,17 +42738,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>お前がヤったんだろ！</t>
+          <t>迷宮の王</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>クシザキ</t>
+          <t>漫画：K9 脚本：小林裕和 原作：支援BIS</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第9話	ホクロは残されたまま</t>
+          <t>第十八話　血戦（三）</t>
         </is>
       </c>
     </row>
@@ -41721,17 +42758,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第96話</t>
+          <t>第5話(2)</t>
         </is>
       </c>
     </row>
@@ -41741,17 +42778,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>俺は星間国家の悪徳領主！</t>
+          <t>おせっかい女子、恋をする</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
+          <t>音竹 ひかる(著者)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第46話　王者の戦い方（後編）</t>
+          <t>第14話</t>
         </is>
       </c>
     </row>
@@ -41761,17 +42798,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>バーサス</t>
+          <t>異世界でも無難に生きたい症候群</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+          <t>原作：安泰（一二三書房刊） 漫画：笹峰コウ キャラクター原案：ひたきゆう</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第33話 本物の勇者（前編-2）</t>
+          <t>第35話②</t>
         </is>
       </c>
     </row>
@@ -41781,17 +42818,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+          <t>めっちゃ召喚された件 THE COMIC</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第23話③</t>
+          <t>第55話①</t>
         </is>
       </c>
     </row>
@@ -41801,17 +42838,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>おせっかい女子、恋をする</t>
+          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>音竹 ひかる(著者)</t>
+          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第13話</t>
+          <t>第43話</t>
         </is>
       </c>
     </row>
@@ -41821,17 +42858,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>三枝さんはメガネ先輩と恋を描く</t>
+          <t>生徒会役員共</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>セレビィ量産型(著者)</t>
+          <t>氏家ト全</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第26.5話</t>
+          <t>#446</t>
         </is>
       </c>
     </row>
@@ -41841,17 +42878,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>アザミヤコを好きになる</t>
+          <t>異世界帰りの剣聖は、自分の実力に気がつかない　～SSSランクの隠しクエストを受けて帰ってきたらレベル１のF級探索者になったけど、異世界で鍛え上げた剣術が強すぎて王女やS級英雄たちが俺を放ってくれません</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+          <t>夜桜ユノ 吉田屋敷 もきゅ</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>コミックス3巻PR</t>
+          <t>第６話　異世界帰りの剣聖は、”ざまぁの波動”に吞まれる！？（３）</t>
         </is>
       </c>
     </row>
@@ -41861,17 +42898,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>塔の管理をしてみよう</t>
+          <t>自分を押し売りしてきた奴隷ちゃんがドラゴンをワンパンしてた　戯画版</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
+          <t>原作：溝上良 漫画：人生負組 キャラクター原案：ごろー✳︎</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第100話前編</t>
+          <t>第7話「とりちきしょうめ！」</t>
         </is>
       </c>
     </row>
@@ -41881,17 +42918,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+          <t>ガチャを回して仲間を増やす 最強の美少女軍団を作り上げろ</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>漫画/すたひろ 原作/Y.A</t>
+          <t>漫画：晴野しゅー 原作：ちんくるり キャラクター原案：イセ川ヤスタカ</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>chapter84【44話①】</t>
+          <t>第79話後半</t>
         </is>
       </c>
     </row>
@@ -41901,17 +42938,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>幼女戦記</t>
+          <t>ひとりぼっちの異世界攻略</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
+          <t>びび（漫画） 五示正司（原作）</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第百十四章：ドードーバード航空戦Ⅸ</t>
+          <t>第268話　話ついて来れてる？</t>
         </is>
       </c>
     </row>
@@ -41921,17 +42958,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>回復術士のやり直し</t>
+          <t>虚無ねーちゃんはかまってほしい</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
+          <t>観音リツ(著者)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第77話-2</t>
+          <t>第3話</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-05-11
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -53,6 +53,7 @@
     <sheet name="2026-04-20" sheetId="45" state="visible" r:id="rId45"/>
     <sheet name="2026-04-27" sheetId="46" state="visible" r:id="rId46"/>
     <sheet name="2026-05-04" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="2026-05-11" sheetId="48" state="visible" r:id="rId48"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -41973,22 +41974,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>ワンパンマン</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>226撃目</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第47話</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第22話-3「子供たちはどこだ？」</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第７６話『渦中停止』④</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第78話</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第9話 後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第７８話　神輿の戦いが始まった（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第9話</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>いとこのこ</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>いぬちく(著者)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第50話</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>帰ってください！ 阿久津さん</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>長岡太一(著者)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第205話</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>【募集開始】人気投票＆キャラへの質問大募集！【第13巻発売記念】</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>まんきつしたい常連さん</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>しんみりん(著者)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第55話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>おまけ72</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>不純な彼女達は懺悔しない</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>ポロロッカ(著者)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第38話</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>「おかえり、パパ」</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>蝉丸</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第35話　水族館</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第9話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第５９話　新メンバーを迎える器用貧乏（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>剥かせて！竜ケ崎さん</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>一智和智</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>大学生編 第20話</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第80話④</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第4話③</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>田舎で恋は難しい!?</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>ねこうめ(著者)</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第7話</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>異世界食堂　洋食のねこや</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第46話(前半)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第2話-②</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第65話②　魔人と戦ってみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>安田剛助(著者)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第56話</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第14話-1：これからも一緒に</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第４７話　勇者、神々にメンチを切る。そしてエリーゼ、闇堕ちする（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>コミックス告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>拷問181</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第32話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>小林さんちのメイドラゴン</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>クール教信者</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第165話</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第87話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>異世界黙示録マイノグーラ ～破滅の文明で始める世界征服～</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>緑華野菜子(著者) 鹿角フェフ(原作) じゅん(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第32話　真と偽①</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>ライブダンジョン！</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第95話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第9話-1：父親として</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>六志麻あさ 業務用餅 kisui</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第８６話</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第8話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>オタクに優しいギャルはいない!?</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>のりしろちゃん 魚住さかな</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>【#189】ごまかしあまね</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>迷宮の王</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>漫画：K9 脚本：小林裕和 原作：支援BIS</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第十八話　血戦（三）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第5話(2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第14話</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>異世界でも無難に生きたい症候群</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>原作：安泰（一二三書房刊） 漫画：笹峰コウ キャラクター原案：ひたきゆう</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第35話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>めっちゃ召喚された件 THE COMIC</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第55話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第43話</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>生徒会役員共</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>氏家ト全</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>#446</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>異世界帰りの剣聖は、自分の実力に気がつかない　～SSSランクの隠しクエストを受けて帰ってきたらレベル１のF級探索者になったけど、異世界で鍛え上げた剣術が強すぎて王女やS級英雄たちが俺を放ってくれません</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>夜桜ユノ 吉田屋敷 もきゅ</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第６話　異世界帰りの剣聖は、”ざまぁの波動”に吞まれる！？（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>自分を押し売りしてきた奴隷ちゃんがドラゴンをワンパンしてた　戯画版</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>原作：溝上良 漫画：人生負組 キャラクター原案：ごろー✳︎</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第7話「とりちきしょうめ！」</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>ガチャを回して仲間を増やす 最強の美少女軍団を作り上げろ</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>漫画：晴野しゅー 原作：ちんくるり キャラクター原案：イセ川ヤスタカ</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第79話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>ひとりぼっちの異世界攻略</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>びび（漫画） 五示正司（原作）</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第268話　話ついて来れてる？</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>虚無ねーちゃんはかまってほしい</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>観音リツ(著者)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第3話</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ワンパンマン</t>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>原作/ＯＮＥ 作画/村田雄介</t>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>226撃目</t>
+          <t>第38話：劣等感①</t>
         </is>
       </c>
     </row>
@@ -41998,17 +43035,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>魔術師クノンは見えている</t>
+          <t>王子様の友達</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+          <t>すけろく(著者)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第47話</t>
+          <t>第37話</t>
         </is>
       </c>
     </row>
@@ -42018,17 +43055,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+          <t>むちまろ</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第22話-3「子供たちはどこだ？」</t>
+          <t>第151話	海と命と魚つり！</t>
         </is>
       </c>
     </row>
@@ -42048,7 +43085,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第７６話『渦中停止』④</t>
+          <t>第７７話『天空神停止』①</t>
         </is>
       </c>
     </row>
@@ -42058,17 +43095,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第78話</t>
+          <t>第７９話　初キスの戦いが始まった</t>
         </is>
       </c>
     </row>
@@ -42078,17 +43115,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第9話 後編</t>
+          <t>第86話その1</t>
         </is>
       </c>
     </row>
@@ -42098,17 +43135,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第７８話　神輿の戦いが始まった（２）</t>
+          <t>コミックス3巻告知</t>
         </is>
       </c>
     </row>
@@ -42118,17 +43155,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+          <t>クセ強彼女は床にいざなう</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+          <t>須河篤志(著者)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第9話</t>
+          <t>第21話後半</t>
         </is>
       </c>
     </row>
@@ -42138,17 +43175,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>いとこのこ</t>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>いぬちく(著者)</t>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第50話</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -42158,17 +43195,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>帰ってください！ 阿久津さん</t>
+          <t>このヒーラー、めんどくさい</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>長岡太一(著者)</t>
+          <t>丹念に発酵(著者)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第205話</t>
+          <t>第97話：山賊</t>
         </is>
       </c>
     </row>
@@ -42178,17 +43215,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>【募集開始】人気投票＆キャラへの質問大募集！【第13巻発売記念】</t>
+          <t>第136話　ひさびさに本気出してみるⅠ（前編）</t>
         </is>
       </c>
     </row>
@@ -42198,17 +43235,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>まんきつしたい常連さん</t>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>しんみりん(著者)</t>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第55話後編</t>
+          <t>第95話　召喚</t>
         </is>
       </c>
     </row>
@@ -42228,7 +43265,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>おまけ72</t>
+          <t>第144話　帝国皇帝の決断</t>
         </is>
       </c>
     </row>
@@ -42238,17 +43275,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>不純な彼女達は懺悔しない</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ポロロッカ(著者)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第38話</t>
+          <t>第６０話　北西へ旅立つ器用貧乏（１）</t>
         </is>
       </c>
     </row>
@@ -42258,17 +43295,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>「おかえり、パパ」</t>
+          <t>魔のものたちは企てる</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>蝉丸</t>
+          <t>加藤拓弐(原作) ガしガし(作画)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第35話　水族館</t>
+          <t>第36.5話</t>
         </is>
       </c>
     </row>
@@ -42278,17 +43315,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>三部べべ(漫画) ねうしとら(原作)</t>
+          <t>モリタ Ｕ４ nima</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第9話-1</t>
+          <t>第16話（２）　太っちょ貴族と摩訶不思議なる肉料理　（２）</t>
         </is>
       </c>
     </row>
@@ -42298,17 +43335,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第５９話　新メンバーを迎える器用貧乏（４）</t>
+          <t>第81話①</t>
         </is>
       </c>
     </row>
@@ -42318,17 +43355,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>剥かせて！竜ケ崎さん</t>
+          <t>美人女上司滝沢さん</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>一智和智</t>
+          <t>やんBARU(著者)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>大学生編 第20話</t>
+          <t>第219話</t>
         </is>
       </c>
     </row>
@@ -42338,17 +43375,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>板垣恵介 林たかあき</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第80話④</t>
+          <t>第69話 キャリア</t>
         </is>
       </c>
     </row>
@@ -42358,17 +43395,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>ぽんドロイド！ はまさん</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>はれやまはれぞう(著者)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第4話③</t>
+          <t>休載のお知らせ</t>
         </is>
       </c>
     </row>
@@ -42378,17 +43415,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>田舎で恋は難しい!?</t>
+          <t>お前がヤったんだろ！</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ねこうめ(著者)</t>
+          <t>クシザキ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第7話</t>
+          <t>第10話	ガリベンと言う勿れ</t>
         </is>
       </c>
     </row>
@@ -42398,17 +43435,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>異世界食堂　洋食のねこや</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第46話(前半)</t>
+          <t>第66話①　伝説の神龍と戦ってみた</t>
         </is>
       </c>
     </row>
@@ -42418,17 +43455,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第2話-②</t>
+          <t>第４７話　勇者、神々にメンチを切る。そしてエリーゼ、闇堕ちする（４）</t>
         </is>
       </c>
     </row>
@@ -42438,17 +43475,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>聖者無双</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第65話②　魔人と戦ってみた</t>
+          <t>第98話　脅威の黒幕①</t>
         </is>
       </c>
     </row>
@@ -42458,17 +43495,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>安田剛助(著者)</t>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第56話</t>
+          <t>コミックス3巻特典情報</t>
         </is>
       </c>
     </row>
@@ -42478,17 +43515,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第14話-1：これからも一緒に</t>
+          <t>拷問182</t>
         </is>
       </c>
     </row>
@@ -42498,17 +43535,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第４７話　勇者、神々にメンチを切る。そしてエリーゼ、闇堕ちする（３）</t>
+          <t>第87話その2</t>
         </is>
       </c>
     </row>
@@ -42518,17 +43555,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>コミックス告知</t>
+          <t>第2話</t>
         </is>
       </c>
     </row>
@@ -42538,17 +43575,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>インフィニット・デンドログラム</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>拷問181</t>
+          <t>第78話</t>
         </is>
       </c>
     </row>
@@ -42558,17 +43595,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>女友達は頼めば意外とヤらせてくれる</t>
+          <t>くらいあの子としたいこと</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ろくろ(漫画) 鏡遊(原作)</t>
+          <t>碇マナツ(著者)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第32話①</t>
+          <t>第97話</t>
         </is>
       </c>
     </row>
@@ -42578,17 +43615,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>小林さんちのメイドラゴン</t>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>クール教信者</t>
+          <t>はぐはぐ(著者)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第165話</t>
+          <t>第98話</t>
         </is>
       </c>
     </row>
@@ -42598,17 +43635,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>セレビィ量産型(著者)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第87話その1</t>
+          <t>第27話前半</t>
         </is>
       </c>
     </row>
@@ -42618,17 +43655,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>異世界黙示録マイノグーラ ～破滅の文明で始める世界征服～</t>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>緑華野菜子(著者) 鹿角フェフ(原作) じゅん(キャラクター原案)</t>
+          <t>KAKERU</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第32話　真と偽①</t>
+          <t>第76話「フカフカのだんじょん2」（前半）</t>
         </is>
       </c>
     </row>
@@ -42638,17 +43675,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ライブダンジョン！</t>
+          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+          <t>FUNA 東西 モトエ恵介</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第95話後半</t>
+          <t>第129話　襲撃［その８］</t>
         </is>
       </c>
     </row>
@@ -42658,17 +43695,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第9話-1：父親として</t>
+          <t>第86話 ワガママな俳優？</t>
         </is>
       </c>
     </row>
@@ -42678,17 +43715,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>六志麻あさ 業務用餅 kisui</t>
+          <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第８６話</t>
+          <t>第20話 最弱貴族、下着を評価する（２）</t>
         </is>
       </c>
     </row>
@@ -42698,17 +43735,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+          <t>女子高生の無駄づかい</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+          <t>ビーノ(著者)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第8話-2</t>
+          <t>第144話　さくぶん</t>
         </is>
       </c>
     </row>
@@ -42718,17 +43755,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>オタクに優しいギャルはいない!?</t>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>のりしろちゃん 魚住さかな</t>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>【#189】ごまかしあまね</t>
+          <t>EP.26①</t>
         </is>
       </c>
     </row>
@@ -42738,17 +43775,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>迷宮の王</t>
+          <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>漫画：K9 脚本：小林裕和 原作：支援BIS</t>
+          <t>岡沢六十四 るれくちぇ sage・ジョー</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第十八話　血戦（三）</t>
+          <t>第80話(後編) 大いなる作戦</t>
         </is>
       </c>
     </row>
@@ -42758,17 +43795,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+          <t>おせっかい女子、恋をする</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+          <t>音竹 ひかる(著者)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第5話(2)</t>
+          <t>第15話</t>
         </is>
       </c>
     </row>
@@ -42778,17 +43815,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>おせっかい女子、恋をする</t>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>音竹 ひかる(著者)</t>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第14話</t>
+          <t>第24話①</t>
         </is>
       </c>
     </row>
@@ -42798,17 +43835,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>異世界でも無難に生きたい症候群</t>
+          <t>オタクに優しいギャルはいない!?</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>原作：安泰（一二三書房刊） 漫画：笹峰コウ キャラクター原案：ひたきゆう</t>
+          <t>のりしろちゃん 魚住さかな</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第35話②</t>
+          <t>【#190】ぽんこついぢち</t>
         </is>
       </c>
     </row>
@@ -42818,17 +43855,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>めっちゃ召喚された件 THE COMIC</t>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
+          <t>漫画/すたひろ 原作/Y.A</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第55話①</t>
+          <t>chapter85【44話②】</t>
         </is>
       </c>
     </row>
@@ -42838,17 +43875,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
+          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
+          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第43話</t>
+          <t>第10話②「もう一度」</t>
         </is>
       </c>
     </row>
@@ -42858,17 +43895,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>生徒会役員共</t>
+          <t>黄金の経験値</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>氏家ト全</t>
+          <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>#446</t>
+          <t>第24話（後編）</t>
         </is>
       </c>
     </row>
@@ -42878,17 +43915,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>異世界帰りの剣聖は、自分の実力に気がつかない　～SSSランクの隠しクエストを受けて帰ってきたらレベル１のF級探索者になったけど、異世界で鍛え上げた剣術が強すぎて王女やS級英雄たちが俺を放ってくれません</t>
+          <t>美容スキルでクラスの女の子を可愛くしたい</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>夜桜ユノ 吉田屋敷 もきゅ</t>
+          <t>藤白ぺるか(原作) 紺野あずれ(漫画) 水野早桜(キャラクター原案)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第６話　異世界帰りの剣聖は、”ざまぁの波動”に吞まれる！？（３）</t>
+          <t>第3話</t>
         </is>
       </c>
     </row>
@@ -42898,17 +43935,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>自分を押し売りしてきた奴隷ちゃんがドラゴンをワンパンしてた　戯画版</t>
+          <t>陰キャの俺が席替えでS級美少女に囲まれたら秘密の関係が始まった。</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>原作：溝上良 漫画：人生負組 キャラクター原案：ごろー✳︎</t>
+          <t>星野 星野(原作) バラマツヒトミ(漫画) 黒兎 ゆう(キャラクター原案)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第7話「とりちきしょうめ！」</t>
+          <t>第13話</t>
         </is>
       </c>
     </row>
@@ -42918,17 +43955,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ガチャを回して仲間を増やす 最強の美少女軍団を作り上げろ</t>
+          <t>虚無ねーちゃんはかまってほしい</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>漫画：晴野しゅー 原作：ちんくるり キャラクター原案：イセ川ヤスタカ</t>
+          <t>観音リツ(著者)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第79話後半</t>
+          <t>第3話</t>
         </is>
       </c>
     </row>
@@ -42938,17 +43975,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ひとりぼっちの異世界攻略</t>
+          <t>役目を果たした日陰の勇者は、辺境で自由に生きていきます</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>びび（漫画） 五示正司（原作）</t>
+          <t>船野真帆(作画) 丘野優(原作) 布施龍太(キャラクター原案)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第268話　話ついて来れてる？</t>
+          <t>第14話後半</t>
         </is>
       </c>
     </row>
@@ -42958,17 +43995,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>虚無ねーちゃんはかまってほしい</t>
+          <t>地味子な三葉さんが僕を誘惑する</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>観音リツ(著者)</t>
+          <t>はぶらえる(著者)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第3話</t>
+          <t>第15話後半</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-05-18
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -54,6 +54,7 @@
     <sheet name="2026-04-27" sheetId="46" state="visible" r:id="rId46"/>
     <sheet name="2026-05-04" sheetId="47" state="visible" r:id="rId47"/>
     <sheet name="2026-05-11" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="2026-05-18" sheetId="49" state="visible" r:id="rId49"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -43010,22 +43011,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第38話：劣等感①</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>王子様の友達</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>すけろく(著者)</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第37話</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第151話	海と命と魚つり！</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第７７話『天空神停止』①</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第７９話　初キスの戦いが始まった</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第86話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>コミックス3巻告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第21話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>このヒーラー、めんどくさい</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>丹念に発酵(著者)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第97話：山賊</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第136話　ひさびさに本気出してみるⅠ（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第95話　召喚</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第144話　帝国皇帝の決断</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第６０話　北西へ旅立つ器用貧乏（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>魔のものたちは企てる</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>加藤拓弐(原作) ガしガし(作画)</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第36.5話</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>モリタ Ｕ４ nima</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第16話（２）　太っちょ貴族と摩訶不思議なる肉料理　（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第81話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>美人女上司滝沢さん</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>やんBARU(著者)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第219話</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 林たかあき</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第69話 キャリア</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>ぽんドロイド！ はまさん</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>はれやまはれぞう(著者)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>休載のお知らせ</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>クシザキ</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第10話	ガリベンと言う勿れ</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第66話①　伝説の神龍と戦ってみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第４７話　勇者、神々にメンチを切る。そしてエリーゼ、闇堕ちする（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>聖者無双</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第98話　脅威の黒幕①</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>コミックス3巻特典情報</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>拷問182</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第87話その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第2話</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>インフィニット・デンドログラム</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第78話</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第97話</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>はぐはぐ(著者)</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第98話</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第27話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>KAKERU</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第76話「フカフカのだんじょん2」（前半）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>FUNA 東西 モトエ恵介</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第129話　襲撃［その８］</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第86話 ワガママな俳優？</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>空野進 sorani ファルまろ</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第20話 最弱貴族、下着を評価する（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>女子高生の無駄づかい</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>ビーノ(著者)</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第144話　さくぶん</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>EP.26①</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>岡沢六十四 るれくちぇ sage・ジョー</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第80話(後編) 大いなる作戦</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第15話</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第24話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>オタクに優しいギャルはいない!?</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>のりしろちゃん 魚住さかな</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>【#190】ぽんこついぢち</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>漫画/すたひろ 原作/Y.A</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>chapter85【44話②】</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第10話②「もう一度」</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>黄金の経験値</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第24話（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>美容スキルでクラスの女の子を可愛くしたい</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>藤白ぺるか(原作) 紺野あずれ(漫画) 水野早桜(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第3話</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>陰キャの俺が席替えでS級美少女に囲まれたら秘密の関係が始まった。</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>星野 星野(原作) バラマツヒトミ(漫画) 黒兎 ゆう(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第13話</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>虚無ねーちゃんはかまってほしい</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>観音リツ(著者)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第3話</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>役目を果たした日陰の勇者は、辺境で自由に生きていきます</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>船野真帆(作画) 丘野優(原作) 布施龍太(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第14話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>地味子な三葉さんが僕を誘惑する</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>はぶらえる(著者)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第15話後半</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>zunta(作画) はらわたさいぞう(原作)</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第38話：劣等感①</t>
+          <t>第136話</t>
         </is>
       </c>
     </row>
@@ -43035,17 +44072,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>王子様の友達</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>すけろく(著者)</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第37話</t>
+          <t>227撃目</t>
         </is>
       </c>
     </row>
@@ -43055,17 +44092,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>不徳のギルド</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>河添太一</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第151話	海と命と魚つり！</t>
+          <t>第１０６話：未来へ解き放て</t>
         </is>
       </c>
     </row>
@@ -43075,17 +44112,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第７７話『天空神停止』①</t>
+          <t>第38話：劣等感②</t>
         </is>
       </c>
     </row>
@@ -43095,17 +44132,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第７９話　初キスの戦いが始まった</t>
+          <t>第23話-1「情報を引き出せ！」</t>
         </is>
       </c>
     </row>
@@ -43115,17 +44152,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第86話その1</t>
+          <t>第７７話『天空神停止』②</t>
         </is>
       </c>
     </row>
@@ -43135,17 +44172,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+          <t>いとこのこ</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+          <t>いぬちく(著者)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>コミックス3巻告知</t>
+          <t>第51話</t>
         </is>
       </c>
     </row>
@@ -43155,17 +44192,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第21話後半</t>
+          <t>第41話①</t>
         </is>
       </c>
     </row>
@@ -43175,17 +44212,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+          <t>ダンジョンの幼なじみ</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+          <t>久真やすひさ(著者)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>第64話前編</t>
         </is>
       </c>
     </row>
@@ -43195,17 +44232,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>このヒーラー、めんどくさい</t>
+          <t>帰ってください！ 阿久津さん</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>丹念に発酵(著者)</t>
+          <t>長岡太一(著者)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第97話：山賊</t>
+          <t>第206話</t>
         </is>
       </c>
     </row>
@@ -43215,17 +44252,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第136話　ひさびさに本気出してみるⅠ（前編）</t>
+          <t>第19話-1</t>
         </is>
       </c>
     </row>
@@ -43235,17 +44272,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>板垣恵介 猪原賽 陸井栄史</t>
+          <t>久遠まこと(著者) 石のやっさん(原作)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第95話　召喚</t>
+          <t>第36話</t>
         </is>
       </c>
     </row>
@@ -43255,17 +44292,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>フルメタル・パニック！　Family</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>賀東招二(原作) 神反ヲ鬚(作画) 四季童子(キャラクター原案)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第144話　帝国皇帝の決断</t>
+          <t>第14話　神奈川県鎌倉市の海辺の邸宅④-1</t>
         </is>
       </c>
     </row>
@@ -43275,17 +44312,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第６０話　北西へ旅立つ器用貧乏（１）</t>
+          <t>第6話前編：リゼルアルテ</t>
         </is>
       </c>
     </row>
@@ -43295,17 +44332,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>魔のものたちは企てる</t>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>加藤拓弐(原作) ガしガし(作画)</t>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第36.5話</t>
+          <t>第9話-2</t>
         </is>
       </c>
     </row>
@@ -43315,17 +44352,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+          <t>異世界のんびり農家</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>モリタ Ｕ４ nima</t>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第16話（２）　太っちょ貴族と摩訶不思議なる肉料理　（２）</t>
+          <t>第323話</t>
         </is>
       </c>
     </row>
@@ -43335,17 +44372,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>ダークサモナーとデキている</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>車王(著者)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第81話①</t>
+          <t>第90話</t>
         </is>
       </c>
     </row>
@@ -43355,17 +44392,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>美人女上司滝沢さん</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>やんBARU(著者)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第219話</t>
+          <t>第145話　ウラニスの願い</t>
         </is>
       </c>
     </row>
@@ -43375,17 +44412,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>板垣恵介 林たかあき</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第69話 キャリア</t>
+          <t>第136話　ひさびさに本気出してみるⅠ（中編）</t>
         </is>
       </c>
     </row>
@@ -43395,17 +44432,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ぽんドロイド！ はまさん</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>はれやまはれぞう(著者)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>休載のお知らせ</t>
+          <t>第６０話　北西へ旅立つ器用貧乏（２）</t>
         </is>
       </c>
     </row>
@@ -43415,17 +44452,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>お前がヤったんだろ！</t>
+          <t>王子様の友達</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>クシザキ</t>
+          <t>すけろく(著者)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第10話	ガリベンと言う勿れ</t>
+          <t>単行本第5巻速報！</t>
         </is>
       </c>
     </row>
@@ -43435,17 +44472,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>ぽんドロイド！ はまさん</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>はれやまはれぞう(著者)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第66話①　伝説の神龍と戦ってみた</t>
+          <t>第20話</t>
         </is>
       </c>
     </row>
@@ -43455,17 +44492,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>淫獄団地</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第４７話　勇者、神々にメンチを切る。そしてエリーゼ、闇堕ちする（４）</t>
+          <t>第57話（後編）</t>
         </is>
       </c>
     </row>
@@ -43475,17 +44512,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>聖者無双</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第98話　脅威の黒幕①</t>
+          <t>第81話➁</t>
         </is>
       </c>
     </row>
@@ -43495,17 +44532,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>コミックス3巻特典情報</t>
+          <t>第4話④</t>
         </is>
       </c>
     </row>
@@ -43515,17 +44552,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>理想のヒモ生活</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>拷問182</t>
+          <t>第107話　その2</t>
         </is>
       </c>
     </row>
@@ -43535,17 +44572,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第87話その2</t>
+          <t>第5話 「親愛」</t>
         </is>
       </c>
     </row>
@@ -43555,17 +44592,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第2話</t>
+          <t>第14話-2：これからも一緒に</t>
         </is>
       </c>
     </row>
@@ -43575,17 +44612,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>インフィニット・デンドログラム</t>
+          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
+          <t>夜州 nini 藻</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第78話</t>
+          <t>第74話</t>
         </is>
       </c>
     </row>
@@ -43595,17 +44632,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第97話</t>
+          <t>第66話②　伝説の神龍と戦ってみた</t>
         </is>
       </c>
     </row>
@@ -43615,17 +44652,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>サーシャちゃんとクラスメイトオタクくん</t>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>はぐはぐ(著者)</t>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第98話</t>
+          <t>第52話 乾きものと心臓②</t>
         </is>
       </c>
     </row>
@@ -43635,17 +44672,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>三枝さんはメガネ先輩と恋を描く</t>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>セレビィ量産型(著者)</t>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第27話前半</t>
+          <t>第48話　奴と新しい上司（前編）</t>
         </is>
       </c>
     </row>
@@ -43655,17 +44692,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>KAKERU</t>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第76話「フカフカのだんじょん2」（前半）</t>
+          <t>第9話後編</t>
         </is>
       </c>
     </row>
@@ -43675,17 +44712,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
+          <t>お気楽領主の楽しい領地防衛 ～生産系魔術で名もなき村を最強の城塞都市に～</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>FUNA 東西 モトエ恵介</t>
+          <t>青色まろ（漫画） 赤池宗（原作） 転（原作イラスト）</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第129話　襲撃［その８］</t>
+          <t>第40話　帰還</t>
         </is>
       </c>
     </row>
@@ -43695,17 +44732,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第86話 ワガママな俳優？</t>
+          <t>第87話その3</t>
         </is>
       </c>
     </row>
@@ -43715,17 +44752,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>空野進 sorani ファルまろ</t>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第20話 最弱貴族、下着を評価する（２）</t>
+          <t>第9話-2：父親として</t>
         </is>
       </c>
     </row>
@@ -43735,17 +44772,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>女子高生の無駄づかい</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ビーノ(著者)</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第144話　さくぶん</t>
+          <t>第153話 よくわからないけれどデュマってるみたいです（１）</t>
         </is>
       </c>
     </row>
@@ -43755,17 +44792,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>EP.26①</t>
+          <t>第４７話　勇者、神々にメンチを切る。そしてエリーゼ、闇堕ちする（５）</t>
         </is>
       </c>
     </row>
@@ -43775,17 +44812,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
+          <t>アザミヤコを好きになる</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>岡沢六十四 るれくちぇ sage・ジョー</t>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第80話(後編) 大いなる作戦</t>
+          <t>番外1P漫画</t>
         </is>
       </c>
     </row>
@@ -43795,17 +44832,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>おせっかい女子、恋をする</t>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>音竹 ひかる(著者)</t>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第15話</t>
+          <t>第32話②</t>
         </is>
       </c>
     </row>
@@ -43815,17 +44852,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第24話①</t>
+          <t>拷問183</t>
         </is>
       </c>
     </row>
@@ -43835,17 +44872,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>オタクに優しいギャルはいない!?</t>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>のりしろちゃん 魚住さかな</t>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>【#190】ぽんこついぢち</t>
+          <t>第3話-①</t>
         </is>
       </c>
     </row>
@@ -43855,17 +44892,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>漫画/すたひろ 原作/Y.A</t>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>chapter85【44話②】</t>
+          <t>第8話-1</t>
         </is>
       </c>
     </row>
@@ -43875,17 +44912,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
+          <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
+          <t>クール教信者</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第10話②「もう一度」</t>
+          <t>第166話</t>
         </is>
       </c>
     </row>
@@ -43895,17 +44932,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>黄金の経験値</t>
+          <t>俺は星間国家の悪徳領主！</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
+          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第24話（後編）</t>
+          <t>第47話　飽きたな</t>
         </is>
       </c>
     </row>
@@ -43915,17 +44952,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>美容スキルでクラスの女の子を可愛くしたい</t>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>藤白ぺるか(原作) 紺野あずれ(漫画) 水野早桜(キャラクター原案)</t>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第3話</t>
+          <t>第24話②</t>
         </is>
       </c>
     </row>
@@ -43935,17 +44972,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>陰キャの俺が席替えでS級美少女に囲まれたら秘密の関係が始まった。</t>
+          <t>バーサス</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>星野 星野(原作) バラマツヒトミ(漫画) 黒兎 ゆう(キャラクター原案)</t>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第13話</t>
+          <t>第33話 本物の勇者（後編-1）</t>
         </is>
       </c>
     </row>
@@ -43955,17 +44992,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>虚無ねーちゃんはかまってほしい</t>
+          <t>異世界黙示録マイノグーラ ～破滅の文明で始める世界征服～</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>観音リツ(著者)</t>
+          <t>緑華野菜子(著者) 鹿角フェフ(原作) じゅん(キャラクター原案)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第3話</t>
+          <t>第32話　真と偽②</t>
         </is>
       </c>
     </row>
@@ -43975,17 +45012,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>役目を果たした日陰の勇者は、辺境で自由に生きていきます</t>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>船野真帆(作画) 丘野優(原作) 布施龍太(キャラクター原案)</t>
+          <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第14話後半</t>
+          <t>第20話 最弱貴族、下着を評価する（３）</t>
         </is>
       </c>
     </row>
@@ -43995,17 +45032,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>地味子な三葉さんが僕を誘惑する</t>
+          <t>迷宮の王</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>はぶらえる(著者)</t>
+          <t>漫画：K9 脚本：小林裕和 原作：支援BIS</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第15話後半</t>
+          <t>第十九話　血戦（四）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-05-25
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -55,6 +55,7 @@
     <sheet name="2026-05-04" sheetId="47" state="visible" r:id="rId47"/>
     <sheet name="2026-05-11" sheetId="48" state="visible" r:id="rId48"/>
     <sheet name="2026-05-18" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="2026-05-25" sheetId="50" state="visible" r:id="rId50"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -44047,1000 +44048,1000 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>丈(著者)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>第136話</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>ワンパンマン</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>227撃目</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>不徳のギルド</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>河添太一</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>第１０６話：未来へ解き放て</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>zunta(作画) はらわたさいぞう(原作)</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>第38話：劣等感②</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>第23話-1「情報を引き出せ！」</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="0" t="inlineStr">
         <is>
           <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>光永康則</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>第７７話『天空神停止』②</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
         <is>
           <t>いとこのこ</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>いぬちく(著者)</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>第51話</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>クラスで２番目に可愛い女の子と友だちになった</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>第41話①</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="0" t="inlineStr">
         <is>
           <t>ダンジョンの幼なじみ</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>久真やすひさ(著者)</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>第64話前編</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="0" t="inlineStr">
         <is>
           <t>帰ってください！ 阿久津さん</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>長岡太一(著者)</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>第206話</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>第19話-1</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>久遠まこと(著者) 石のやっさん(原作)</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>第36話</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>フルメタル・パニック！　Family</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>賀東招二(原作) 神反ヲ鬚(作画) 四季童子(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>第14話　神奈川県鎌倉市の海辺の邸宅④-1</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>第6話前編：リゼルアルテ</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>三部べべ(漫画) ねうしとら(原作)</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>第9話-2</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>異世界のんびり農家</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>第323話</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="0" t="inlineStr">
         <is>
           <t>ダークサモナーとデキている</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>車王(著者)</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>第90話</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="0" t="inlineStr">
         <is>
           <t>実は俺、最強でした？</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
         <is>
           <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>第145話　ウラニスの願い</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="0" t="inlineStr">
         <is>
           <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="0" t="inlineStr">
         <is>
           <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>第136話　ひさびさに本気出してみるⅠ（中編）</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="0" t="inlineStr">
         <is>
           <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>第６０話　北西へ旅立つ器用貧乏（２）</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="0" t="inlineStr">
         <is>
           <t>王子様の友達</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>すけろく(著者)</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>単行本第5巻速報！</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="0" t="inlineStr">
         <is>
           <t>ぽんドロイド！ はまさん</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>はれやまはれぞう(著者)</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>第20話</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
+      <c r="A24" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="0" t="inlineStr">
         <is>
           <t>淫獄団地</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>搾精研究所(原作) 丈山雄為(漫画)</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>第57話（後編）</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
+      <c r="A25" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="0" t="inlineStr">
         <is>
           <t>リビルドワールド</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>第81話➁</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
+      <c r="A26" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="0" t="inlineStr">
         <is>
           <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>第4話④</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="n">
+      <c r="A27" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="0" t="inlineStr">
         <is>
           <t>理想のヒモ生活</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>第107話　その2</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
+      <c r="A28" s="0" t="n">
         <v>27</v>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="0" t="inlineStr">
         <is>
           <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr">
         <is>
           <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t>第5話 「親愛」</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="0" t="inlineStr">
         <is>
           <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>第14話-2：これからも一緒に</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="n">
+      <c r="A30" s="0" t="n">
         <v>29</v>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="0" t="inlineStr">
         <is>
           <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t>夜州 nini 藻</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="0" t="inlineStr">
         <is>
           <t>第74話</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="0" t="inlineStr">
         <is>
           <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>第66話②　伝説の神龍と戦ってみた</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="n">
+      <c r="A32" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="0" t="inlineStr">
         <is>
           <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="0" t="inlineStr">
         <is>
           <t>第52話 乾きものと心臓②</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="n">
+      <c r="A33" s="0" t="n">
         <v>32</v>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="0" t="inlineStr">
         <is>
           <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t>第48話　奴と新しい上司（前編）</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
+      <c r="A34" s="0" t="n">
         <v>33</v>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="0" t="inlineStr">
         <is>
           <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="0" t="inlineStr">
         <is>
           <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="0" t="inlineStr">
         <is>
           <t>第9話後編</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="n">
+      <c r="A35" s="0" t="n">
         <v>34</v>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="0" t="inlineStr">
         <is>
           <t>お気楽領主の楽しい領地防衛 ～生産系魔術で名もなき村を最強の城塞都市に～</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="0" t="inlineStr">
         <is>
           <t>青色まろ（漫画） 赤池宗（原作） 転（原作イラスト）</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="0" t="inlineStr">
         <is>
           <t>第40話　帰還</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="n">
+      <c r="A36" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="0" t="inlineStr">
         <is>
           <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr">
         <is>
           <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="0" t="inlineStr">
         <is>
           <t>第87話その3</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="n">
+      <c r="A37" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="0" t="inlineStr">
         <is>
           <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr">
         <is>
           <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="0" t="inlineStr">
         <is>
           <t>第9話-2：父親として</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="n">
+      <c r="A38" s="0" t="n">
         <v>37</v>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="0" t="inlineStr">
         <is>
           <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="0" t="inlineStr">
         <is>
           <t>内々けやき あし カオミン</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="0" t="inlineStr">
         <is>
           <t>第153話 よくわからないけれどデュマってるみたいです（１）</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="0" t="inlineStr">
         <is>
           <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="0" t="inlineStr">
         <is>
           <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="0" t="inlineStr">
         <is>
           <t>第４７話　勇者、神々にメンチを切る。そしてエリーゼ、闇堕ちする（５）</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
+      <c r="A40" s="0" t="n">
         <v>39</v>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="0" t="inlineStr">
         <is>
           <t>アザミヤコを好きになる</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="0" t="inlineStr">
         <is>
           <t>ユニティコング(原作) ツノニガウ(作画)</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="0" t="inlineStr">
         <is>
           <t>番外1P漫画</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="n">
+      <c r="A41" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="0" t="inlineStr">
         <is>
           <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="0" t="inlineStr">
         <is>
           <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="0" t="inlineStr">
         <is>
           <t>第32話②</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="n">
+      <c r="A42" s="0" t="n">
         <v>41</v>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="0" t="inlineStr">
         <is>
           <t>姫様“拷問”の時間です</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="0" t="inlineStr">
         <is>
           <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="0" t="inlineStr">
         <is>
           <t>拷問183</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="0" t="inlineStr">
         <is>
           <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="0" t="inlineStr">
         <is>
           <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="0" t="inlineStr">
         <is>
           <t>第3話-①</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="n">
+      <c r="A44" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="0" t="inlineStr">
         <is>
           <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="0" t="inlineStr">
         <is>
           <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="0" t="inlineStr">
         <is>
           <t>第8話-1</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="0" t="inlineStr">
         <is>
           <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="0" t="inlineStr">
         <is>
           <t>クール教信者</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="0" t="inlineStr">
         <is>
           <t>第166話</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
+      <c r="A46" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="0" t="inlineStr">
         <is>
           <t>俺は星間国家の悪徳領主！</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
         <is>
           <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="0" t="inlineStr">
         <is>
           <t>第47話　飽きたな</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="n">
+      <c r="A47" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="0" t="inlineStr">
         <is>
           <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="0" t="inlineStr">
         <is>
           <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="0" t="inlineStr">
         <is>
           <t>第24話②</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="n">
+      <c r="A48" s="0" t="n">
         <v>47</v>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="0" t="inlineStr">
         <is>
           <t>バーサス</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="0" t="inlineStr">
         <is>
           <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="0" t="inlineStr">
         <is>
           <t>第33話 本物の勇者（後編-1）</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="n">
+      <c r="A49" s="0" t="n">
         <v>48</v>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="0" t="inlineStr">
         <is>
           <t>異世界黙示録マイノグーラ ～破滅の文明で始める世界征服～</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="0" t="inlineStr">
         <is>
           <t>緑華野菜子(著者) 鹿角フェフ(原作) じゅん(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="0" t="inlineStr">
         <is>
           <t>第32話　真と偽②</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="n">
+      <c r="A50" s="0" t="n">
         <v>49</v>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="0" t="inlineStr">
         <is>
           <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="0" t="inlineStr">
         <is>
           <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="0" t="inlineStr">
         <is>
           <t>第20話 最弱貴族、下着を評価する（３）</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="n">
+      <c r="A51" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="0" t="inlineStr">
         <is>
           <t>迷宮の王</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="0" t="inlineStr">
         <is>
           <t>漫画：K9 脚本：小林裕和 原作：支援BIS</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="0" t="inlineStr">
         <is>
           <t>第十九話　血戦（四）</t>
         </is>
@@ -46087,6 +46088,1042 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>異世界おじさん</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>殆ど死んでいる(著者)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>第77話</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>第79話 前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>第38話：劣等感③</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>第７７話『天空神停止』③</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>第152話	Trick or KOMARO（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>第86話その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>第22話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>第96話　技</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>第16話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>まんきつしたい常連さん</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>しんみりん(著者)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>第56話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>金属スライムを倒しまくった俺が【黒鋼の王】と呼ばれるまで</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>藤屋いずこ(著者) 温泉カピバラ(原作) 山椒魚(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>第19章-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>第22話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>第324話</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>第146話　国を守るぞ！・前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>第136話　ひさびさに本気出してみるⅠ（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>第６０話　北西へ旅立つ器用貧乏（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>第２９食　聖女様の魔法、ステキですわ！（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>第81話③</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>第45話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>特別イラスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>リアデイルの大地にて</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>月見だしお(著者) Ceez(原作) てんまそ(キャラクター原案) 涼風涼(構成)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>第42章</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>濁る瞳で何を願う ハイセルク戦記</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>トルトネン 創-taro 斎藤八呑</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>第40話 止まらぬ波</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>第27話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>美人女上司滝沢さん</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>やんBARU(著者)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>第220話</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>おとなりのダウナーさんは無理させない</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>瑠璃いろ(著者)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>第16話</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>板垣恵介 林たかあき</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>第70話 不動の綱</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>第136話</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>クシザキ</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>第11話	エンジョイランド</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>聖者無双</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>第98話　脅威の黒幕②</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>第４８話　勇者、弟のために作った剣が、凄すぎて自我を持つ（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>アザミヤコを好きになる</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>番外編④</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>拷問184</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>第153話 よくわからないけれどデュマってるみたいです（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>第98話</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>はぐはぐ(著者)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>第99話</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>KAKERU</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>第76話「フカフカのだんじょん2」（後半）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>やさぐれ召喚者は動かない（コミック）</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>漫画／そらモチ 原作／吉岡剛 キャラクター原案／くろぎり</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>第3話(2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>転生剣豪ズバババァーン！！</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>富士田けやき(原作) 坂崎ふれでぃ(作画)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>第2話</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>EP.26②</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>最弱テイマーはゴミ拾いの旅を始めました。@COMIC</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>漫画：蕗野 冬 原作：ほのぼのる500 キャラクター原案：なま</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>第30話 ②</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>漫画/すたひろ 原作/Y.A</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>chapter86【45話①】</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>岡沢六十四 るれくちぇ sage・ジョー</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>第81話(前編) VS.ドロイエ</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>第24話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>第17話</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ギャル神官はリザレがダルい</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>秋★枝</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>幕間2</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>オタクに優しいギャルはいない!?</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>のりしろちゃん 魚住さかな</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>【#192】天音、大人になる？？</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>天獄で悪魔がボクを魅惑する</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>銀河味めてお(著者)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>第41話</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>第10話③「もう一度」</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>第3話</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add ranking data for 2026-06-01
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -56,6 +56,7 @@
     <sheet name="2026-05-11" sheetId="48" state="visible" r:id="rId48"/>
     <sheet name="2026-05-18" sheetId="49" state="visible" r:id="rId49"/>
     <sheet name="2026-05-25" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="2026-06-01" sheetId="51" state="visible" r:id="rId51"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -46120,22 +46121,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>異世界おじさん</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>殆ど死んでいる(著者)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第77話</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第79話 前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第38話：劣等感③</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第７７話『天空神停止』③</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第152話	Trick or KOMARO（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第86話その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第22話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第96話　技</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第16話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>まんきつしたい常連さん</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>しんみりん(著者)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第56話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>金属スライムを倒しまくった俺が【黒鋼の王】と呼ばれるまで</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>藤屋いずこ(著者) 温泉カピバラ(原作) 山椒魚(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第19章-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第22話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第324話</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第146話　国を守るぞ！・前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第136話　ひさびさに本気出してみるⅠ（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第６０話　北西へ旅立つ器用貧乏（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第２９食　聖女様の魔法、ステキですわ！（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第81話③</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第45話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>特別イラスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>リアデイルの大地にて</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>月見だしお(著者) Ceez(原作) てんまそ(キャラクター原案) 涼風涼(構成)</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第42章</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>濁る瞳で何を願う ハイセルク戦記</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>トルトネン 創-taro 斎藤八呑</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第40話 止まらぬ波</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第27話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>美人女上司滝沢さん</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>やんBARU(著者)</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第220話</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>おとなりのダウナーさんは無理させない</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>瑠璃いろ(著者)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第16話</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 林たかあき</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第70話 不動の綱</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第136話</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>クシザキ</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第11話	エンジョイランド</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>聖者無双</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第98話　脅威の黒幕②</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第４８話　勇者、弟のために作った剣が、凄すぎて自我を持つ（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>アザミヤコを好きになる</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>番外編④</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>拷問184</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第153話 よくわからないけれどデュマってるみたいです（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第98話</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>はぐはぐ(著者)</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第99話</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>KAKERU</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第76話「フカフカのだんじょん2」（後半）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>やさぐれ召喚者は動かない（コミック）</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>漫画／そらモチ 原作／吉岡剛 キャラクター原案／くろぎり</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第3話(2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>転生剣豪ズバババァーン！！</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>富士田けやき(原作) 坂崎ふれでぃ(作画)</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第2話</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>EP.26②</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>最弱テイマーはゴミ拾いの旅を始めました。@COMIC</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>漫画：蕗野 冬 原作：ほのぼのる500 キャラクター原案：なま</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第30話 ②</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>漫画/すたひろ 原作/Y.A</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>chapter86【45話①】</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>岡沢六十四 るれくちぇ sage・ジョー</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第81話(前編) VS.ドロイエ</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第24話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第17話</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>ギャル神官はリザレがダルい</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>秋★枝</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>幕間2</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>オタクに優しいギャルはいない!?</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>のりしろちゃん 魚住さかな</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>【#192】天音、大人になる？？</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>天獄で悪魔がボクを魅惑する</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>銀河味めてお(著者)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第41話</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第10話③「もう一度」</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第3話</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>異世界おじさん</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>殆ど死んでいる(著者)</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第77話</t>
+          <t>第137話</t>
         </is>
       </c>
     </row>
@@ -46145,17 +47182,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+          <t>転生したらスライムだった件</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+          <t>原作：伏瀬 漫画：川上泰樹 キャラクター原案：みっつばー</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第79話 前編</t>
+          <t>第133話　悪魔の囁き</t>
         </is>
       </c>
     </row>
@@ -46165,17 +47202,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>zunta(作画) はらわたさいぞう(原作)</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第38話：劣等感③</t>
+          <t>228撃目</t>
         </is>
       </c>
     </row>
@@ -46185,17 +47222,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>異種族レビュアーズ</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>天原(原作) masha(作画)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第７７話『天空神停止』③</t>
+          <t>第93話</t>
         </is>
       </c>
     </row>
@@ -46205,17 +47242,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>魔術師クノンは見えている</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第152話	Trick or KOMARO（前編）</t>
+          <t>第48話①</t>
         </is>
       </c>
     </row>
@@ -46225,17 +47262,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第86話その2</t>
+          <t>第23話-2「情報を引き出せ！」</t>
         </is>
       </c>
     </row>
@@ -46245,17 +47282,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第22話後半</t>
+          <t>第７７話『天空神停止』④</t>
         </is>
       </c>
     </row>
@@ -46265,17 +47302,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+          <t>いとこのこ</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>板垣恵介 猪原賽 陸井栄史</t>
+          <t>いぬちく(著者)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第96話　技</t>
+          <t>第52話</t>
         </is>
       </c>
     </row>
@@ -46285,17 +47322,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第16話-1</t>
+          <t>第79話</t>
         </is>
       </c>
     </row>
@@ -46305,17 +47342,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>まんきつしたい常連さん</t>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>しんみりん(著者)</t>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第56話前編</t>
+          <t>第10話 前編</t>
         </is>
       </c>
     </row>
@@ -46325,17 +47362,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>金属スライムを倒しまくった俺が【黒鋼の王】と呼ばれるまで</t>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>藤屋いずこ(著者) 温泉カピバラ(原作) 山椒魚(キャラクター原案)</t>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第19章-2</t>
+          <t>第41話②</t>
         </is>
       </c>
     </row>
@@ -46345,17 +47382,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>帰ってください！ 阿久津さん</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>長岡太一(著者)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第22話前半</t>
+          <t>番外編㉘</t>
         </is>
       </c>
     </row>
@@ -46365,17 +47402,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>異世界のんびり農家</t>
+          <t>異世界居酒屋「のぶ」</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第324話</t>
+          <t>第132話</t>
         </is>
       </c>
     </row>
@@ -46385,17 +47422,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第146話　国を守るぞ！・前編</t>
+          <t>第19話-2</t>
         </is>
       </c>
     </row>
@@ -46405,17 +47442,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第136話　ひさびさに本気出してみるⅠ（後編）</t>
+          <t>第10話前半</t>
         </is>
       </c>
     </row>
@@ -46425,17 +47462,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第６０話　北西へ旅立つ器用貧乏（３）</t>
+          <t>第6話後編：リゼルアルテ</t>
         </is>
       </c>
     </row>
@@ -46445,17 +47482,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+          <t>ダンジョンの幼なじみ</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>島知宏 音速炒飯 有都あらゆる</t>
+          <t>久真やすひさ(著者)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第２９食　聖女様の魔法、ステキですわ！（２）</t>
+          <t>第64話後編</t>
         </is>
       </c>
     </row>
@@ -46465,17 +47502,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>異世界のんびり農家</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第81話③</t>
+          <t>第325話</t>
         </is>
       </c>
     </row>
@@ -46485,17 +47522,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
+          <t>ヨウハ(著者)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第45話-2</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -46505,17 +47542,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+          <t>ダークサモナーとデキている</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+          <t>車王(著者)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>特別イラスト</t>
+          <t>第91話</t>
         </is>
       </c>
     </row>
@@ -46525,17 +47562,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>リアデイルの大地にて</t>
+          <t>不純な彼女達は懺悔しない</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>月見だしお(著者) Ceez(原作) てんまそ(キャラクター原案) 涼風涼(構成)</t>
+          <t>ポロロッカ(著者)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第42章</t>
+          <t>第39話</t>
         </is>
       </c>
     </row>
@@ -46545,17 +47582,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>濁る瞳で何を願う ハイセルク戦記</t>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>トルトネン 創-taro 斎藤八呑</t>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第40話 止まらぬ波</t>
+          <t>第10話-1</t>
         </is>
       </c>
     </row>
@@ -46565,17 +47602,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>三枝さんはメガネ先輩と恋を描く</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>セレビィ量産型(著者)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第27話後半</t>
+          <t>おまけ73</t>
         </is>
       </c>
     </row>
@@ -46585,17 +47622,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>美人女上司滝沢さん</t>
+          <t>「おかえり、パパ」</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>やんBARU(著者)</t>
+          <t>蝉丸</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第220話</t>
+          <t>第36話　追跡</t>
         </is>
       </c>
     </row>
@@ -46605,17 +47642,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>おとなりのダウナーさんは無理させない</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>瑠璃いろ(著者)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第16話</t>
+          <t>第６０話　北西へ旅立つ器用貧乏（４）</t>
         </is>
       </c>
     </row>
@@ -46625,17 +47662,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+          <t>淫獄団地</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>板垣恵介 林たかあき</t>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第70話 不動の綱</t>
+          <t>第58話（前編）</t>
         </is>
       </c>
     </row>
@@ -46645,17 +47682,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>宇崎ちゃんは遊びたい！</t>
+          <t>剥かせて！竜ケ崎さん</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>丈(著者)</t>
+          <t>一智和智</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第136話</t>
+          <t>大学生編 第21話</t>
         </is>
       </c>
     </row>
@@ -46665,17 +47702,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>お前がヤったんだろ！</t>
+          <t>物語の黒幕に転生して</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>クシザキ</t>
+          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第11話	エンジョイランド</t>
+          <t>第41話</t>
         </is>
       </c>
     </row>
@@ -46685,17 +47722,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>聖者無双</t>
+          <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+          <t>安田剛助(著者)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第98話　脅威の黒幕②</t>
+          <t>第57話</t>
         </is>
       </c>
     </row>
@@ -46705,17 +47742,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第４８話　勇者、弟のために作った剣が、凄すぎて自我を持つ（１）</t>
+          <t>第6話 誓婚の光輪</t>
         </is>
       </c>
     </row>
@@ -46725,17 +47762,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>アザミヤコを好きになる</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>番外編④</t>
+          <t>第4話⑤</t>
         </is>
       </c>
     </row>
@@ -46745,17 +47782,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>拷問184</t>
+          <t>第２９食　聖女様の魔法、ステキですわ！（３）</t>
         </is>
       </c>
     </row>
@@ -46765,17 +47802,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第153話 よくわからないけれどデュマってるみたいです（２）</t>
+          <t>第39話 独身貴族は写真展を開く（1）</t>
         </is>
       </c>
     </row>
@@ -46785,17 +47822,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>第67話①　少しだけ日常を変えてみた</t>
         </is>
       </c>
     </row>
@@ -46805,17 +47842,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第98話</t>
+          <t>第10話前編</t>
         </is>
       </c>
     </row>
@@ -46825,17 +47862,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>サーシャちゃんとクラスメイトオタクくん</t>
+          <t>異世界食堂　洋食のねこや</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>はぐはぐ(著者)</t>
+          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第99話</t>
+          <t>第46話(後半)</t>
         </is>
       </c>
     </row>
@@ -46845,17 +47882,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>KAKERU</t>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第76話「フカフカのだんじょん2」（後半）</t>
+          <t>第53話 友の兄とお茶会を①</t>
         </is>
       </c>
     </row>
@@ -46865,17 +47902,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>やさぐれ召喚者は動かない（コミック）</t>
+          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>漫画／そらモチ 原作／吉岡剛 キャラクター原案／くろぎり</t>
+          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第3話(2)</t>
+          <t>第45話-2</t>
         </is>
       </c>
     </row>
@@ -46885,17 +47922,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>転生剣豪ズバババァーン！！</t>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>富士田けやき(原作) 坂崎ふれでぃ(作画)</t>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第2話</t>
+          <t>第8話-2</t>
         </is>
       </c>
     </row>
@@ -46905,17 +47942,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>EP.26②</t>
+          <t>おもしろい休載まんが</t>
         </is>
       </c>
     </row>
@@ -46925,17 +47962,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>最弱テイマーはゴミ拾いの旅を始めました。@COMIC</t>
+          <t>【目つき悪いシリーズ】ミタメトウラハラ</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>漫画：蕗野 冬 原作：ほのぼのる500 キャラクター原案：なま</t>
+          <t>ウラベスナヒト</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第30話 ②</t>
+          <t>#12息抜き</t>
         </is>
       </c>
     </row>
@@ -46945,17 +47982,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>漫画/すたひろ 原作/Y.A</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>chapter86【45話①】</t>
+          <t>第４８話　勇者、弟のために作った剣が、凄すぎて自我を持つ（２）</t>
         </is>
       </c>
     </row>
@@ -46965,17 +48002,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>岡沢六十四 るれくちぇ sage・ジョー</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第81話(前編) VS.ドロイエ</t>
+          <t>第154話 よくわからないけれどお使いを頼まれたようです（１）</t>
         </is>
       </c>
     </row>
@@ -46985,17 +48022,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第24話②</t>
+          <t>第88話その1</t>
         </is>
       </c>
     </row>
@@ -47005,17 +48042,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>おせっかい女子、恋をする</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>音竹 ひかる(著者)</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第17話</t>
+          <t>拷問185</t>
         </is>
       </c>
     </row>
@@ -47025,17 +48062,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ギャル神官はリザレがダルい</t>
+          <t>バーサス</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>秋★枝</t>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>幕間2</t>
+          <t>第33話 本物の勇者（後編-2）</t>
         </is>
       </c>
     </row>
@@ -47045,17 +48082,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>オタクに優しいギャルはいない!?</t>
+          <t>ギルドの雑用係が真の黒幕でした ～隠れた才能で暗躍無双～</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>のりしろちゃん 魚住さかな</t>
+          <t>漫画/パヤパヤ 原作/菱川さかく キャラクター原案/ゆーにっと</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>【#192】天音、大人になる？？</t>
+          <t>第3話（1）</t>
         </is>
       </c>
     </row>
@@ -47065,17 +48102,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>天獄で悪魔がボクを魅惑する</t>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>銀河味めてお(著者)</t>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第41話</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -47085,17 +48122,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
+          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
+          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第10話③「もう一度」</t>
+          <t>第4話</t>
         </is>
       </c>
     </row>
@@ -47105,17 +48142,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
+          <t>ライブダンジョン！</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第3話</t>
+          <t>第96話後半</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-06-08
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -57,6 +57,7 @@
     <sheet name="2026-05-18" sheetId="49" state="visible" r:id="rId49"/>
     <sheet name="2026-05-25" sheetId="50" state="visible" r:id="rId50"/>
     <sheet name="2026-06-01" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="2026-06-08" sheetId="52" state="visible" r:id="rId52"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -47157,22 +47158,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第137話</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>転生したらスライムだった件</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>原作：伏瀬 漫画：川上泰樹 キャラクター原案：みっつばー</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第133話　悪魔の囁き</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>ワンパンマン</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>228撃目</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>異種族レビュアーズ</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>天原(原作) masha(作画)</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第93話</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第48話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第23話-2「情報を引き出せ！」</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第７７話『天空神停止』④</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>いとこのこ</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>いぬちく(著者)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第52話</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第79話</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第10話 前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第41話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>帰ってください！ 阿久津さん</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>長岡太一(著者)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>番外編㉘</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>異世界居酒屋「のぶ」</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第132話</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第19話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第10話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第6話後編：リゼルアルテ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>ダンジョンの幼なじみ</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>久真やすひさ(著者)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第64話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第325話</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>ヨウハ(著者)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第91話</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>不純な彼女達は懺悔しない</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>ポロロッカ(著者)</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第39話</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第10話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>おまけ73</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>「おかえり、パパ」</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>蝉丸</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第36話　追跡</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第６０話　北西へ旅立つ器用貧乏（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>淫獄団地</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第58話（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>剥かせて！竜ケ崎さん</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>一智和智</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>大学生編 第21話</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>物語の黒幕に転生して</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第41話</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>安田剛助(著者)</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第57話</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第6話 誓婚の光輪</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第4話⑤</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第２９食　聖女様の魔法、ステキですわ！（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第39話 独身貴族は写真展を開く（1）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第67話①　少しだけ日常を変えてみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第10話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>異世界食堂　洋食のねこや</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第46話(後半)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第53話 友の兄とお茶会を①</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第45話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第8話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>おもしろい休載まんが</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>【目つき悪いシリーズ】ミタメトウラハラ</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>ウラベスナヒト</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>#12息抜き</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第４８話　勇者、弟のために作った剣が、凄すぎて自我を持つ（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第154話 よくわからないけれどお使いを頼まれたようです（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第88話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>拷問185</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>バーサス</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第33話 本物の勇者（後編-2）</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>ギルドの雑用係が真の黒幕でした ～隠れた才能で暗躍無双～</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>漫画/パヤパヤ 原作/菱川さかく キャラクター原案/ゆーにっと</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第3話（1）</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第4話</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>ライブダンジョン！</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第96話後半</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>宇崎ちゃんは遊びたい！</t>
+          <t>転生したらスライムだった件</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>丈(著者)</t>
+          <t>原作：伏瀬 漫画：川上泰樹 キャラクター原案：みっつばー</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第137話</t>
+          <t>第135話　黒色軍団</t>
         </is>
       </c>
     </row>
@@ -47182,17 +48219,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>転生したらスライムだった件</t>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>原作：伏瀬 漫画：川上泰樹 キャラクター原案：みっつばー</t>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第133話　悪魔の囁き</t>
+          <t>第79話 後編</t>
         </is>
       </c>
     </row>
@@ -47202,17 +48239,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ワンパンマン</t>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>原作/ＯＮＥ 作画/村田雄介</t>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>228撃目</t>
+          <t>第39話：天才と無能①</t>
         </is>
       </c>
     </row>
@@ -47222,17 +48259,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>異種族レビュアーズ</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>天原(原作) masha(作画)</t>
+          <t>むちまろ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第93話</t>
+          <t>第153話	Trick or KOMARO（中編）</t>
         </is>
       </c>
     </row>
@@ -47242,17 +48279,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>魔術師クノンは見えている</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第48話①</t>
+          <t>第７８話『寒天停止』①</t>
         </is>
       </c>
     </row>
@@ -47262,17 +48299,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+          <t>寿司ガキ</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+          <t>ichika(著者)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第23話-2「情報を引き出せ！」</t>
+          <t>第11話</t>
         </is>
       </c>
     </row>
@@ -47282,17 +48319,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第７７話『天空神停止』④</t>
+          <t>第87話その1</t>
         </is>
       </c>
     </row>
@@ -47302,17 +48339,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>いとこのこ</t>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>いぬちく(著者)</t>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第52話</t>
+          <t>第10話後半</t>
         </is>
       </c>
     </row>
@@ -47322,17 +48359,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第79話</t>
+          <t>第23話前半</t>
         </is>
       </c>
     </row>
@@ -47342,17 +48379,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+          <t>王子様の友達</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+          <t>すけろく(著者)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第10話 前編</t>
+          <t>番外編 くろすこ!!</t>
         </is>
       </c>
     </row>
@@ -47362,17 +48399,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+          <t>クセ強彼女は床にいざなう</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+          <t>須河篤志(著者)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第41話②</t>
+          <t>第22話後半</t>
         </is>
       </c>
     </row>
@@ -47382,17 +48419,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>帰ってください！ 阿久津さん</t>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>長岡太一(著者)</t>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>番外編㉘</t>
+          <t>第97話　螺旋(うず)</t>
         </is>
       </c>
     </row>
@@ -47402,17 +48439,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>異世界居酒屋「のぶ」</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第132話</t>
+          <t>第137話　ひさびさに本気出してみるⅡ（前編）</t>
         </is>
       </c>
     </row>
@@ -47422,17 +48459,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+          <t>まんきつしたい常連さん</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+          <t>しんみりん(著者)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第19話-2</t>
+          <t>第56話後編</t>
         </is>
       </c>
     </row>
@@ -47442,17 +48479,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+          <t>このヒーラー、めんどくさい</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+          <t>丹念に発酵(著者)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第10話前半</t>
+          <t>第98話：雨宿り</t>
         </is>
       </c>
     </row>
@@ -47462,17 +48499,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第6話後編：リゼルアルテ</t>
+          <t>第146話　国を守るぞ！・後編</t>
         </is>
       </c>
     </row>
@@ -47482,17 +48519,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ダンジョンの幼なじみ</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>久真やすひさ(著者)</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第64話後編</t>
+          <t>第137話</t>
         </is>
       </c>
     </row>
@@ -47502,17 +48539,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>異世界のんびり農家</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第325話</t>
+          <t>第81話④</t>
         </is>
       </c>
     </row>
@@ -47522,17 +48559,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ヨウハ(著者)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>第６０話　北西へ旅立つ器用貧乏（４）</t>
         </is>
       </c>
     </row>
@@ -47542,17 +48579,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ダークサモナーとデキている</t>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>車王(著者)</t>
+          <t>モリタ Ｕ４ nima</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第91話</t>
+          <t>第16話（３）　太っちょ貴族と摩訶不思議なる肉料理　（３）</t>
         </is>
       </c>
     </row>
@@ -47562,17 +48599,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>不純な彼女達は懺悔しない</t>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ポロロッカ(著者)</t>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第39話</t>
+          <t>第39話 独身貴族は写真展を開く（2）</t>
         </is>
       </c>
     </row>
@@ -47582,17 +48619,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>三部べべ(漫画) ねうしとら(原作)</t>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第10話-1</t>
+          <t>第２９食　聖女様の魔法、ステキですわ！（３）</t>
         </is>
       </c>
     </row>
@@ -47602,17 +48639,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>おまけ73</t>
+          <t>5巻発売告知漫画</t>
         </is>
       </c>
     </row>
@@ -47622,17 +48659,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>「おかえり、パパ」</t>
+          <t>美人女上司滝沢さん</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>蝉丸</t>
+          <t>やんBARU(著者)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第36話　追跡</t>
+          <t>第221話</t>
         </is>
       </c>
     </row>
@@ -47642,17 +48679,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第６０話　北西へ旅立つ器用貧乏（４）</t>
+          <t>第67話②　少しだけ日常を変えてみた</t>
         </is>
       </c>
     </row>
@@ -47662,17 +48699,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>淫獄団地</t>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第58話（前編）</t>
+          <t>第15話-1：一番弟子の卒業</t>
         </is>
       </c>
     </row>
@@ -47682,17 +48719,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>剥かせて！竜ケ崎さん</t>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>一智和智</t>
+          <t>板垣恵介 林たかあき</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>大学生編 第21話</t>
+          <t>第71話 這い上がり</t>
         </is>
       </c>
     </row>
@@ -47702,17 +48739,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>物語の黒幕に転生して</t>
+          <t>聖者無双</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第41話</t>
+          <t>第99話　リザリア①</t>
         </is>
       </c>
     </row>
@@ -47722,17 +48759,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>安田剛助(著者)</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第57話</t>
+          <t>第154話 よくわからないけれどお使いを頼まれたようです（２）</t>
         </is>
       </c>
     </row>
@@ -47742,17 +48779,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第6話 誓婚の光輪</t>
+          <t>拷問186</t>
         </is>
       </c>
     </row>
@@ -47762,17 +48799,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第4話⑤</t>
+          <t>第33話①</t>
         </is>
       </c>
     </row>
@@ -47782,17 +48819,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+          <t>雨森潤奈は湿度が高い</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>島知宏 音速炒飯 有都あらゆる</t>
+          <t>水城水城(原作) 稲鳴四季(作画) 潮崎しの(キャラクター原案)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第２９食　聖女様の魔法、ステキですわ！（３）</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -47802,17 +48839,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第39話 独身貴族は写真展を開く（1）</t>
+          <t>第４８話　勇者、弟のために作った剣が、凄すぎて自我を持つ（３）</t>
         </is>
       </c>
     </row>
@@ -47822,17 +48859,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第67話①　少しだけ日常を変えてみた</t>
+          <t>第46話-2</t>
         </is>
       </c>
     </row>
@@ -47842,17 +48879,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+          <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+          <t>クール教信者</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第10話前編</t>
+          <t>第167話</t>
         </is>
       </c>
     </row>
@@ -47862,17 +48899,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>異世界食堂　洋食のねこや</t>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第46話(後半)</t>
+          <t>第3話-②</t>
         </is>
       </c>
     </row>
@@ -47882,17 +48919,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第53話 友の兄とお茶会を①</t>
+          <t>第88話その2</t>
         </is>
       </c>
     </row>
@@ -47902,17 +48939,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
+          <t>原作:剃り残し 漫画:大窪太一</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第45話-2</t>
+          <t>第8話(後編)</t>
         </is>
       </c>
     </row>
@@ -47922,17 +48959,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第8話-2</t>
+          <t>第10話-1：初めてのお友達？</t>
         </is>
       </c>
     </row>
@@ -47942,17 +48979,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+          <t>ギャルの自転車を直したら懐かれた</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+          <t>タケチケイ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>おもしろい休載まんが</t>
+          <t>第1話　ギャルの自転車を直した</t>
         </is>
       </c>
     </row>
@@ -47962,17 +48999,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>【目つき悪いシリーズ】ミタメトウラハラ</t>
+          <t>田舎で恋は難しい!?</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ウラベスナヒト</t>
+          <t>ねこうめ(著者)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>#12息抜き</t>
+          <t>コミックス作業のためイラスト更新</t>
         </is>
       </c>
     </row>
@@ -47982,17 +49019,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第４８話　勇者、弟のために作った剣が、凄すぎて自我を持つ（２）</t>
+          <t>第64話　暗闇の中で、ひずみ（前編）</t>
         </is>
       </c>
     </row>
@@ -48002,17 +49039,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第154話 よくわからないけれどお使いを頼まれたようです（１）</t>
+          <t>第4話</t>
         </is>
       </c>
     </row>
@@ -48022,17 +49059,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>KAKERU</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第88話その1</t>
+          <t>第77話「最前線」（前半）</t>
         </is>
       </c>
     </row>
@@ -48042,17 +49079,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>拷問185</t>
+          <t>第87話 雨月リュウガ、加速す!!</t>
         </is>
       </c>
     </row>
@@ -48062,17 +49099,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>バーサス</t>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+          <t>セレビィ量産型(著者)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第33話 本物の勇者（後編-2）</t>
+          <t>第27.5話</t>
         </is>
       </c>
     </row>
@@ -48082,17 +49119,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ギルドの雑用係が真の黒幕でした ～隠れた才能で暗躍無双～</t>
+          <t>くらいあの子としたいこと</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>漫画/パヤパヤ 原作/菱川さかく キャラクター原案/ゆーにっと</t>
+          <t>碇マナツ(著者)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第3話（1）</t>
+          <t>特別編㉓</t>
         </is>
       </c>
     </row>
@@ -48102,17 +49139,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+          <t>おせっかい女子、恋をする</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+          <t>音竹 ひかる(著者)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>第19話</t>
         </is>
       </c>
     </row>
@@ -48122,17 +49159,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
+          <t>漫画/すたひろ 原作/Y.A</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第4話</t>
+          <t>chapter87【45話②】</t>
         </is>
       </c>
     </row>
@@ -48142,17 +49179,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ライブダンジョン！</t>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第96話後半</t>
+          <t>EP.27①</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-06-15
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -58,6 +58,7 @@
     <sheet name="2026-05-25" sheetId="50" state="visible" r:id="rId50"/>
     <sheet name="2026-06-01" sheetId="51" state="visible" r:id="rId51"/>
     <sheet name="2026-06-08" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="2026-06-15" sheetId="53" state="visible" r:id="rId53"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -48194,6 +48195,1042 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>転生したらスライムだった件</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>原作：伏瀬 漫画：川上泰樹 キャラクター原案：みっつばー</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第135話　黒色軍団</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第79話 後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第39話：天才と無能①</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第153話	Trick or KOMARO（中編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第７８話『寒天停止』①</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>寿司ガキ</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>ichika(著者)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第11話</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第87話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第10話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第23話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>王子様の友達</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>すけろく(著者)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>番外編 くろすこ!!</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第22話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第97話　螺旋(うず)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第137話　ひさびさに本気出してみるⅡ（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>まんきつしたい常連さん</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>しんみりん(著者)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第56話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>このヒーラー、めんどくさい</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>丹念に発酵(著者)</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第98話：雨宿り</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第146話　国を守るぞ！・後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第137話</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第81話④</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第６０話　北西へ旅立つ器用貧乏（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>モリタ Ｕ４ nima</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第16話（３）　太っちょ貴族と摩訶不思議なる肉料理　（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第39話 独身貴族は写真展を開く（2）</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第２９食　聖女様の魔法、ステキですわ！（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>5巻発売告知漫画</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>美人女上司滝沢さん</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>やんBARU(著者)</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第221話</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第67話②　少しだけ日常を変えてみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第15話-1：一番弟子の卒業</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 林たかあき</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第71話 這い上がり</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>聖者無双</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第99話　リザリア①</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第154話 よくわからないけれどお使いを頼まれたようです（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>拷問186</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第33話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>雨森潤奈は湿度が高い</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>水城水城(原作) 稲鳴四季(作画) 潮崎しの(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第４８話　勇者、弟のために作った剣が、凄すぎて自我を持つ（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第46話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>小林さんちのメイドラゴン</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>クール教信者</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第167話</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第3話-②</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第88話その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>原作:剃り残し 漫画:大窪太一</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第8話(後編)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第10話-1：初めてのお友達？</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>ギャルの自転車を直したら懐かれた</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>タケチケイ</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第1話　ギャルの自転車を直した</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>田舎で恋は難しい!?</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>ねこうめ(著者)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>コミックス作業のためイラスト更新</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第64話　暗闇の中で、ひずみ（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第4話</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>KAKERU</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第77話「最前線」（前半）</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第87話 雨月リュウガ、加速す!!</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第27.5話</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>特別編㉓</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第19話</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>漫画/すたひろ 原作/Y.A</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>chapter87【45話②】</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>EP.27①</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
@@ -48209,7 +49246,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第135話　黒色軍団</t>
+          <t>第136話　子供達の成長</t>
         </is>
       </c>
     </row>
@@ -48219,17 +49256,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第79話 後編</t>
+          <t>229撃目</t>
         </is>
       </c>
     </row>
@@ -48239,17 +49276,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+          <t>不徳のギルド</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>zunta(作画) はらわたさいぞう(原作)</t>
+          <t>河添太一</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第39話：天才と無能①</t>
+          <t>第１０７話：自壊の日</t>
         </is>
       </c>
     </row>
@@ -48259,17 +49296,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>魔術師クノンは見えている</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第153話	Trick or KOMARO（中編）</t>
+          <t>第48話➁</t>
         </is>
       </c>
     </row>
@@ -48279,17 +49316,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第７８話『寒天停止』①</t>
+          <t>第39話：天才と無能②</t>
         </is>
       </c>
     </row>
@@ -48299,17 +49336,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>寿司ガキ</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ichika(著者)</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第11話</t>
+          <t>第23話-3「情報を引き出せ！」</t>
         </is>
       </c>
     </row>
@@ -48319,17 +49356,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第87話その1</t>
+          <t>第７８話『寒天停止』②</t>
         </is>
       </c>
     </row>
@@ -48339,17 +49376,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+          <t>いとこのこ</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+          <t>いぬちく(著者)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第10話後半</t>
+          <t>第53話</t>
         </is>
       </c>
     </row>
@@ -48359,17 +49396,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+          <t>蜘蛛ですが、なにか？</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+          <t>かかし朝浩(著者) 馬場翁(原作) 輝竜司(キャラクター原案)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第23話前半</t>
+          <t>第79話その1</t>
         </is>
       </c>
     </row>
@@ -48379,17 +49416,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>王子様の友達</t>
+          <t>ダンジョンの幼なじみ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>すけろく(著者)</t>
+          <t>久真やすひさ(著者)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>番外編 くろすこ!!</t>
+          <t>第65話</t>
         </is>
       </c>
     </row>
@@ -48399,17 +49436,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第22話後半</t>
+          <t>第42話①</t>
         </is>
       </c>
     </row>
@@ -48419,17 +49456,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>板垣恵介 猪原賽 陸井栄史</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第97話　螺旋(うず)</t>
+          <t>第８０話　パルクールの戦いが始まった（１）</t>
         </is>
       </c>
     </row>
@@ -48439,17 +49476,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>久遠まこと(著者) 石のやっさん(原作)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第137話　ひさびさに本気出してみるⅡ（前編）</t>
+          <t>第37話</t>
         </is>
       </c>
     </row>
@@ -48459,17 +49496,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>まんきつしたい常連さん</t>
+          <t>帰ってください！ 阿久津さん</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>しんみりん(著者)</t>
+          <t>長岡太一(著者)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第56話後編</t>
+          <t>第207話</t>
         </is>
       </c>
     </row>
@@ -48479,17 +49516,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>このヒーラー、めんどくさい</t>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>丹念に発酵(著者)</t>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第98話：雨宿り</t>
+          <t>第20話-1</t>
         </is>
       </c>
     </row>
@@ -48499,17 +49536,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第146話　国を守るぞ！・後編</t>
+          <t>第7話前編：不穏な依頼</t>
         </is>
       </c>
     </row>
@@ -48519,17 +49556,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>宇崎ちゃんは遊びたい！</t>
+          <t>異世界のんびり農家</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>丈(著者)</t>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第137話</t>
+          <t>第326話</t>
         </is>
       </c>
     </row>
@@ -48539,17 +49576,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>ダークサモナーとデキている</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>車王(著者)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第81話④</t>
+          <t>テレビアニメ続報！</t>
         </is>
       </c>
     </row>
@@ -48559,17 +49596,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第６０話　北西へ旅立つ器用貧乏（４）</t>
+          <t>第16話-2</t>
         </is>
       </c>
     </row>
@@ -48579,17 +49616,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>モリタ Ｕ４ nima</t>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第16話（３）　太っちょ貴族と摩訶不思議なる肉料理　（３）</t>
+          <t>第10話-2</t>
         </is>
       </c>
     </row>
@@ -48599,17 +49636,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第39話 独身貴族は写真展を開く（2）</t>
+          <t>第147話　ユリヤの正体・前編</t>
         </is>
       </c>
     </row>
@@ -48619,17 +49656,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>島知宏 音速炒飯 有都あらゆる</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第２９食　聖女様の魔法、ステキですわ！（３）</t>
+          <t>第137話　ひさびさに本気出してみるⅡ（中編）</t>
         </is>
       </c>
     </row>
@@ -48639,17 +49676,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+          <t>ぽんドロイド！ はまさん</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+          <t>はれやまはれぞう(著者)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>5巻発売告知漫画</t>
+          <t>第21話</t>
         </is>
       </c>
     </row>
@@ -48659,17 +49696,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>美人女上司滝沢さん</t>
+          <t>お前がヤったんだろ！</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>やんBARU(著者)</t>
+          <t>クシザキ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第221話</t>
+          <t>第12話	リセイVSキョウフ</t>
         </is>
       </c>
     </row>
@@ -48679,17 +49716,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第67話②　少しだけ日常を変えてみた</t>
+          <t>第82話①</t>
         </is>
       </c>
     </row>
@@ -48699,17 +49736,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+          <t>魔のものたちは企てる</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+          <t>加藤拓弐(原作) ガしガし(作画)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第15話-1：一番弟子の卒業</t>
+          <t>第37話</t>
         </is>
       </c>
     </row>
@@ -48719,17 +49756,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>板垣恵介 林たかあき</t>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第71話 這い上がり</t>
+          <t>第2話-1</t>
         </is>
       </c>
     </row>
@@ -48739,17 +49776,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>聖者無双</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第99話　リザリア①</t>
+          <t>第5話①</t>
         </is>
       </c>
     </row>
@@ -48759,17 +49796,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>淫獄団地</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第154話 よくわからないけれどお使いを頼まれたようです（２）</t>
+          <t>第58話（後編）</t>
         </is>
       </c>
     </row>
@@ -48779,17 +49816,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>拷問186</t>
+          <t>第7話 ミステル家</t>
         </is>
       </c>
     </row>
@@ -48799,17 +49836,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>女友達は頼めば意外とヤらせてくれる</t>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ろくろ(漫画) 鏡遊(原作)</t>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第33話①</t>
+          <t>第39話 独身貴族は写真展を開く（3）</t>
         </is>
       </c>
     </row>
@@ -48819,17 +49856,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>雨森潤奈は湿度が高い</t>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>水城水城(原作) 稲鳴四季(作画) 潮崎しの(キャラクター原案)</t>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>第10話後編</t>
         </is>
       </c>
     </row>
@@ -48839,17 +49876,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>望まぬ不死の冒険者</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>中曽根ハイジ（漫画） 丘野 優（原作） じゃいあん（キャラクター原案）</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第４８話　勇者、弟のために作った剣が、凄すぎて自我を持つ（３）</t>
+          <t>第65話　必ず祓います</t>
         </is>
       </c>
     </row>
@@ -48859,17 +49896,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
+          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
+          <t>夜州 nini 藻</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第46話-2</t>
+          <t>第75話</t>
         </is>
       </c>
     </row>
@@ -48879,17 +49916,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>小林さんちのメイドラゴン</t>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>クール教信者</t>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第167話</t>
+          <t>第53話 友の兄とお茶会を②</t>
         </is>
       </c>
     </row>
@@ -48899,17 +49936,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+          <t>ヨウハ(著者)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第3話-②</t>
+          <t>第2話-1</t>
         </is>
       </c>
     </row>
@@ -48919,17 +49956,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>はぐはぐ(著者)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第88話その2</t>
+          <t>第100話</t>
         </is>
       </c>
     </row>
@@ -48939,17 +49976,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+          <t>描けないのでヤってみた</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>原作:剃り残し 漫画:大窪太一</t>
+          <t>逢上おかき(著者)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第8話(後編)</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -48959,17 +49996,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+          <t>お気楽領主の楽しい領地防衛 ～生産系魔術で名もなき村を最強の城塞都市に～</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+          <t>青色まろ（漫画） 赤池宗（原作） 転（原作イラスト）</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第10話-1：初めてのお友達？</t>
+          <t>第41話　誕生日</t>
         </is>
       </c>
     </row>
@@ -48979,17 +50016,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ギャルの自転車を直したら懐かれた</t>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>タケチケイ</t>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第1話　ギャルの自転車を直した</t>
+          <t>第48話　奴と新しい上司（後編）</t>
         </is>
       </c>
     </row>
@@ -48999,17 +50036,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>田舎で恋は難しい!?</t>
+          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ねこうめ(著者)</t>
+          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>コミックス作業のためイラスト更新</t>
+          <t>第3話</t>
         </is>
       </c>
     </row>
@@ -49019,17 +50056,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
+          <t>理想のヒモ生活</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
+          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第64話　暗闇の中で、ひずみ（前編）</t>
+          <t>第108話　その2</t>
         </is>
       </c>
     </row>
@@ -49039,17 +50076,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第4話</t>
+          <t>拷問187</t>
         </is>
       </c>
     </row>
@@ -49059,17 +50096,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>KAKERU</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第77話「最前線」（前半）</t>
+          <t>第155話 よくわからないけれどじぇじぇじぇな事態のようです（１）</t>
         </is>
       </c>
     </row>
@@ -49079,17 +50116,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第87話 雨月リュウガ、加速す!!</t>
+          <t>第４８話　勇者、弟のために作った剣が、凄すぎて自我を持つ（４）</t>
         </is>
       </c>
     </row>
@@ -49099,17 +50136,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>三枝さんはメガネ先輩と恋を描く</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>セレビィ量産型(著者)</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第27.5話</t>
+          <t>第88話その3</t>
         </is>
       </c>
     </row>
@@ -49119,17 +50156,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>特別編㉓</t>
+          <t>第9話-1</t>
         </is>
       </c>
     </row>
@@ -49139,17 +50176,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>おせっかい女子、恋をする</t>
+          <t>バーサス</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>音竹 ひかる(著者)</t>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第19話</t>
+          <t>第34話 思い知れ（1）</t>
         </is>
       </c>
     </row>
@@ -49159,17 +50196,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+          <t>義妹５人いる</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>漫画/すたひろ 原作/Y.A</t>
+          <t>じゃこ(漫画) 榛名丼(原作) むにんしき(キャラクター原案)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>chapter87【45話②】</t>
+          <t>第2話-1</t>
         </is>
       </c>
     </row>
@@ -49179,17 +50216,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+          <t>FUNA 東西 モトエ恵介</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>EP.27①</t>
+          <t>第130話 第2回異世界懇談会［その①］</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-06-22
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -59,6 +59,7 @@
     <sheet name="2026-06-01" sheetId="51" state="visible" r:id="rId51"/>
     <sheet name="2026-06-08" sheetId="52" state="visible" r:id="rId52"/>
     <sheet name="2026-06-15" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="2026-06-22" sheetId="54" state="visible" r:id="rId54"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -49231,22 +49232,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>転生したらスライムだった件</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>原作：伏瀬 漫画：川上泰樹 キャラクター原案：みっつばー</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第136話　子供達の成長</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>ワンパンマン</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>229撃目</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>不徳のギルド</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>河添太一</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第１０７話：自壊の日</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第48話➁</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第39話：天才と無能②</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第23話-3「情報を引き出せ！」</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第７８話『寒天停止』②</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>いとこのこ</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>いぬちく(著者)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第53話</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>蜘蛛ですが、なにか？</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>かかし朝浩(著者) 馬場翁(原作) 輝竜司(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第79話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>ダンジョンの幼なじみ</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>久真やすひさ(著者)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第65話</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第42話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第８０話　パルクールの戦いが始まった（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>久遠まこと(著者) 石のやっさん(原作)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第37話</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>帰ってください！ 阿久津さん</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>長岡太一(著者)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第207話</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第20話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第7話前編：不穏な依頼</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第326話</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>テレビアニメ続報！</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第16話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第10話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第147話　ユリヤの正体・前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第137話　ひさびさに本気出してみるⅡ（中編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>ぽんドロイド！ はまさん</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>はれやまはれぞう(著者)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第21話</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>クシザキ</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第12話	リセイVSキョウフ</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第82話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>魔のものたちは企てる</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>加藤拓弐(原作) ガしガし(作画)</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第37話</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第2話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第5話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>淫獄団地</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第58話（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第7話 ミステル家</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第39話 独身貴族は写真展を開く（3）</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第10話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>望まぬ不死の冒険者</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>中曽根ハイジ（漫画） 丘野 優（原作） じゃいあん（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第65話　必ず祓います</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>夜州 nini 藻</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第75話</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第53話 友の兄とお茶会を②</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>ヨウハ(著者)</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第2話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>はぐはぐ(著者)</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第100話</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>描けないのでヤってみた</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>逢上おかき(著者)</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>お気楽領主の楽しい領地防衛 ～生産系魔術で名もなき村を最強の城塞都市に～</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>青色まろ（漫画） 赤池宗（原作） 転（原作イラスト）</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第41話　誕生日</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第48話　奴と新しい上司（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第3話</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>理想のヒモ生活</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第108話　その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>拷問187</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第155話 よくわからないけれどじぇじぇじぇな事態のようです（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第４８話　勇者、弟のために作った剣が、凄すぎて自我を持つ（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第88話その3</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第9話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>バーサス</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第34話 思い知れ（1）</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>義妹５人いる</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>じゃこ(漫画) 榛名丼(原作) むにんしき(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第2話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>FUNA 東西 モトエ恵介</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第130話 第2回異世界懇談会［その①］</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>転生したらスライムだった件</t>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>原作：伏瀬 漫画：川上泰樹 キャラクター原案：みっつばー</t>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第136話　子供達の成長</t>
+          <t>第80話 前編</t>
         </is>
       </c>
     </row>
@@ -49256,17 +50293,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ワンパンマン</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>原作/ＯＮＥ 作画/村田雄介</t>
+          <t>むちまろ</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>229撃目</t>
+          <t>第154話	Trick or KOMARO（後編）</t>
         </is>
       </c>
     </row>
@@ -49276,17 +50313,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>不徳のギルド</t>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>河添太一</t>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第１０７話：自壊の日</t>
+          <t>第39話：天才と無能③</t>
         </is>
       </c>
     </row>
@@ -49296,17 +50333,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>魔術師クノンは見えている</t>
+          <t>蜘蛛ですが、なにか？</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+          <t>かかし朝浩(著者) 馬場翁(原作) 輝竜司(キャラクター原案)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第48話➁</t>
+          <t>第79話その2</t>
         </is>
       </c>
     </row>
@@ -49316,17 +50353,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>zunta(作画) はらわたさいぞう(原作)</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第39話：天才と無能②</t>
+          <t>第７８話『寒天停止』③</t>
         </is>
       </c>
     </row>
@@ -49336,17 +50373,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第23話-3「情報を引き出せ！」</t>
+          <t>第11話</t>
         </is>
       </c>
     </row>
@@ -49356,17 +50393,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第７８話『寒天停止』②</t>
+          <t>第８０話　パルクールの戦いが始まった（２）</t>
         </is>
       </c>
     </row>
@@ -49376,17 +50413,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>いとこのこ</t>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>いぬちく(著者)</t>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第53話</t>
+          <t>第87話その2</t>
         </is>
       </c>
     </row>
@@ -49396,17 +50433,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>蜘蛛ですが、なにか？</t>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>かかし朝浩(著者) 馬場翁(原作) 輝竜司(キャラクター原案)</t>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第79話その1</t>
+          <t>第10話 後編</t>
         </is>
       </c>
     </row>
@@ -49416,17 +50453,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ダンジョンの幼なじみ</t>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>久真やすひさ(著者)</t>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第65話</t>
+          <t>第23話後半</t>
         </is>
       </c>
     </row>
@@ -49436,17 +50473,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第42話①</t>
+          <t>第137話　ひさびさに本気出してみるⅡ（後編）</t>
         </is>
       </c>
     </row>
@@ -49456,17 +50493,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第８０話　パルクールの戦いが始まった（１）</t>
+          <t>第98話　経験値</t>
         </is>
       </c>
     </row>
@@ -49476,17 +50513,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
+          <t>異世界のんびり農家</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>久遠まこと(著者) 石のやっさん(原作)</t>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第37話</t>
+          <t>第327話</t>
         </is>
       </c>
     </row>
@@ -49496,17 +50533,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>帰ってください！ 阿久津さん</t>
+          <t>クセ強彼女は床にいざなう</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>長岡太一(著者)</t>
+          <t>須河篤志(著者)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第207話</t>
+          <t>第23話前半</t>
         </is>
       </c>
     </row>
@@ -49516,17 +50553,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第20話-1</t>
+          <t>第39話</t>
         </is>
       </c>
     </row>
@@ -49536,17 +50573,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第7話前編：不穏な依頼</t>
+          <t>第147話　ユリヤの正体・後編</t>
         </is>
       </c>
     </row>
@@ -49556,17 +50593,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>異世界のんびり農家</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第326話</t>
+          <t>第82話➁</t>
         </is>
       </c>
     </row>
@@ -49576,17 +50613,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ダークサモナーとデキている</t>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>車王(著者)</t>
+          <t>モリタ Ｕ４ nima</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>テレビアニメ続報！</t>
+          <t>第16話（４）　太っちょ貴族と摩訶不思議なる肉料理　（４）</t>
         </is>
       </c>
     </row>
@@ -49596,17 +50633,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+          <t>ヨウハ(著者)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第16話-2</t>
+          <t>第2話-1</t>
         </is>
       </c>
     </row>
@@ -49616,17 +50653,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+          <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>三部べべ(漫画) ねうしとら(原作)</t>
+          <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第10話-2</t>
+          <t>第13話</t>
         </is>
       </c>
     </row>
@@ -49636,17 +50673,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第147話　ユリヤの正体・前編</t>
+          <t>第39話 独身貴族は写真展を開く（4）</t>
         </is>
       </c>
     </row>
@@ -49656,17 +50693,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>濁る瞳で何を願う ハイセルク戦記</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>トルトネン 創-taro 斎藤八呑</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第137話　ひさびさに本気出してみるⅡ（中編）</t>
+          <t>第41話 統率者について</t>
         </is>
       </c>
     </row>
@@ -49676,17 +50713,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ぽんドロイド！ はまさん</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>はれやまはれぞう(著者)</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第21話</t>
+          <t>第68話①　休暇を満喫してみた</t>
         </is>
       </c>
     </row>
@@ -49696,17 +50733,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>お前がヤったんだろ！</t>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>クシザキ</t>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第12話	リセイVSキョウフ</t>
+          <t>第15話-2：一番弟子の卒業</t>
         </is>
       </c>
     </row>
@@ -49716,17 +50753,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>板垣恵介 林たかあき</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第82話①</t>
+          <t>第72話 ムサシ</t>
         </is>
       </c>
     </row>
@@ -49736,17 +50773,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>魔のものたちは企てる</t>
+          <t>骸骨騎士様、只今異世界へお出掛け中</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>加藤拓弐(原作) ガしガし(作画)</t>
+          <t>サワノアキラ（漫画） 秤猿鬼（原作） KeG（キャラクター原案）</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第37話</t>
+          <t>第68章　龍王の会談（前編）</t>
         </is>
       </c>
     </row>
@@ -49756,17 +50793,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第2話-1</t>
+          <t>第33話②</t>
         </is>
       </c>
     </row>
@@ -49776,17 +50813,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>聖者無双</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第5話①</t>
+          <t>第99話　リザリア②</t>
         </is>
       </c>
     </row>
@@ -49796,17 +50833,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>淫獄団地</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第58話（後編）</t>
+          <t>第155話 よくわからないけれどじぇじぇじぇな事態のようです（２）</t>
         </is>
       </c>
     </row>
@@ -49816,17 +50853,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+          <t>めちゃくちゃ追放される話</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+          <t>杉浦次郎 向浦宏和</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第7話 ミステル家</t>
+          <t>第４話（中編）</t>
         </is>
       </c>
     </row>
@@ -49836,17 +50873,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第39話 独身貴族は写真展を開く（3）</t>
+          <t>第４８話　勇者、弟のために作った剣が、凄すぎて自我を持つ（５）</t>
         </is>
       </c>
     </row>
@@ -49856,17 +50893,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第10話後編</t>
+          <t>拷問188</t>
         </is>
       </c>
     </row>
@@ -49876,17 +50913,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>望まぬ不死の冒険者</t>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>中曽根ハイジ（漫画） 丘野 優（原作） じゃいあん（キャラクター原案）</t>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第65話　必ず祓います</t>
+          <t>第10話-2：初めてのお友達？</t>
         </is>
       </c>
     </row>
@@ -49896,17 +50933,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>夜州 nini 藻</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第75話</t>
+          <t>第88話その4</t>
         </is>
       </c>
     </row>
@@ -49916,17 +50953,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+          <t>回復術士のやり直し</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第53話 友の兄とお茶会を②</t>
+          <t>第78話-2</t>
         </is>
       </c>
     </row>
@@ -49936,17 +50973,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+          <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ヨウハ(著者)</t>
+          <t>クール教信者</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第2話-1</t>
+          <t>第168話</t>
         </is>
       </c>
     </row>
@@ -49956,17 +50993,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>サーシャちゃんとクラスメイトオタクくん</t>
+          <t>インフィニット・デンドログラム</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>はぐはぐ(著者)</t>
+          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第100話</t>
+          <t>第79話</t>
         </is>
       </c>
     </row>
@@ -49976,17 +51013,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>描けないのでヤってみた</t>
+          <t>【目つき悪いシリーズ】ミタメトウラハラ</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>逢上おかき(著者)</t>
+          <t>ウラベスナヒト</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>#13誘惑</t>
         </is>
       </c>
     </row>
@@ -49996,17 +51033,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>お気楽領主の楽しい領地防衛 ～生産系魔術で名もなき村を最強の城塞都市に～</t>
+          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>青色まろ（漫画） 赤池宗（原作） 転（原作イラスト）</t>
+          <t>六志麻あさ 業務用餅 kisui</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第41話　誕生日</t>
+          <t>第８８話</t>
         </is>
       </c>
     </row>
@@ -50016,17 +51053,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+          <t>俺は星間国家の悪徳領主！</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第48話　奴と新しい上司（後編）</t>
+          <t>第48話　化け物共</t>
         </is>
       </c>
     </row>
@@ -50036,17 +51073,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第3話</t>
+          <t>第7話(2)</t>
         </is>
       </c>
     </row>
@@ -50056,17 +51093,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>理想のヒモ生活</t>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第108話　その2</t>
+          <t>第24話③</t>
         </is>
       </c>
     </row>
@@ -50076,17 +51113,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>拷問187</t>
+          <t>第88話 悩める原口監督！</t>
         </is>
       </c>
     </row>
@@ -50096,17 +51133,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>セレビィ量産型(著者)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第155話 よくわからないけれどじぇじぇじぇな事態のようです（１）</t>
+          <t>第28話前半</t>
         </is>
       </c>
     </row>
@@ -50116,17 +51153,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>KAKERU</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第４８話　勇者、弟のために作った剣が、凄すぎて自我を持つ（４）</t>
+          <t>第77話「最前線」（後半）</t>
         </is>
       </c>
     </row>
@@ -50136,17 +51173,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>くらいあの子としたいこと</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>碇マナツ(著者)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第88話その3</t>
+          <t>特別編㉔</t>
         </is>
       </c>
     </row>
@@ -50156,17 +51193,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+          <t>漫画/すたひろ 原作/Y.A</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第9話-1</t>
+          <t>chapter88【46話①】</t>
         </is>
       </c>
     </row>
@@ -50176,17 +51213,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>バーサス</t>
+          <t>男子高校生だけどギャルにTSしました</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+          <t>太陽まりい(著者)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第34話 思い知れ（1）</t>
+          <t>第27話前編</t>
         </is>
       </c>
     </row>
@@ -50196,17 +51233,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>義妹５人いる</t>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>じゃこ(漫画) 榛名丼(原作) むにんしき(キャラクター原案)</t>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第2話-1</t>
+          <t>EP.27②</t>
         </is>
       </c>
     </row>
@@ -50216,17 +51253,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
+          <t>ギャルの自転車を直したら懐かれた</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>FUNA 東西 モトエ恵介</t>
+          <t>タケチケイ（漫画） 生姜寧也（原作）</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第130話 第2回異世界懇談会［その①］</t>
+          <t>第2話　ギャルと弁当を食べた（後編）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-06-29
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -60,6 +60,7 @@
     <sheet name="2026-06-08" sheetId="52" state="visible" r:id="rId52"/>
     <sheet name="2026-06-15" sheetId="53" state="visible" r:id="rId53"/>
     <sheet name="2026-06-22" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="2026-06-29" sheetId="55" state="visible" r:id="rId55"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -50268,22 +50269,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第80話 前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第154話	Trick or KOMARO（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第39話：天才と無能③</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>蜘蛛ですが、なにか？</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>かかし朝浩(著者) 馬場翁(原作) 輝竜司(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第79話その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第７８話『寒天停止』③</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第11話</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第８０話　パルクールの戦いが始まった（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第87話その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第10話 後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第23話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第137話　ひさびさに本気出してみるⅡ（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第98話　経験値</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第327話</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第23話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第39話</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第147話　ユリヤの正体・後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第82話➁</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>モリタ Ｕ４ nima</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第16話（４）　太っちょ貴族と摩訶不思議なる肉料理　（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>ヨウハ(著者)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第2話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第13話</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第39話 独身貴族は写真展を開く（4）</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>濁る瞳で何を願う ハイセルク戦記</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>トルトネン 創-taro 斎藤八呑</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第41話 統率者について</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第68話①　休暇を満喫してみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第15話-2：一番弟子の卒業</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 林たかあき</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第72話 ムサシ</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>骸骨騎士様、只今異世界へお出掛け中</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>サワノアキラ（漫画） 秤猿鬼（原作） KeG（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第68章　龍王の会談（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第33話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>聖者無双</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第99話　リザリア②</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第155話 よくわからないけれどじぇじぇじぇな事態のようです（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>めちゃくちゃ追放される話</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>杉浦次郎 向浦宏和</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第４話（中編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第４８話　勇者、弟のために作った剣が、凄すぎて自我を持つ（５）</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>拷問188</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第10話-2：初めてのお友達？</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第88話その4</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>回復術士のやり直し</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第78話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>小林さんちのメイドラゴン</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>クール教信者</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第168話</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>インフィニット・デンドログラム</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第79話</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>【目つき悪いシリーズ】ミタメトウラハラ</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>ウラベスナヒト</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>#13誘惑</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>六志麻あさ 業務用餅 kisui</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第８８話</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>俺は星間国家の悪徳領主！</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第48話　化け物共</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第7話(2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第24話③</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第88話 悩める原口監督！</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第28話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>KAKERU</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第77話「最前線」（後半）</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>特別編㉔</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>漫画/すたひろ 原作/Y.A</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>chapter88【46話①】</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>男子高校生だけどギャルにTSしました</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>太陽まりい(著者)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第27話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>EP.27②</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>ギャルの自転車を直したら懐かれた</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>タケチケイ（漫画） 生姜寧也（原作）</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第2話　ギャルと弁当を食べた（後編）</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第80話 前編</t>
+          <t>第138話</t>
         </is>
       </c>
     </row>
@@ -50293,17 +51330,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>異世界おじさん</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>殆ど死んでいる(著者)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第154話	Trick or KOMARO（後編）</t>
+          <t>第78話</t>
         </is>
       </c>
     </row>
@@ -50313,17 +51350,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>zunta(作画) はらわたさいぞう(原作)</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第39話：天才と無能③</t>
+          <t>230撃目</t>
         </is>
       </c>
     </row>
@@ -50333,17 +51370,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>蜘蛛ですが、なにか？</t>
+          <t>魔術師クノンは見えている</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>かかし朝浩(著者) 馬場翁(原作) 輝竜司(キャラクター原案)</t>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第79話その2</t>
+          <t>第49話①</t>
         </is>
       </c>
     </row>
@@ -50353,17 +51390,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第７８話『寒天停止』③</t>
+          <t>第24話-1「父と子と」</t>
         </is>
       </c>
     </row>
@@ -50373,17 +51410,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第11話</t>
+          <t>※アライブクイーン投票用：7/31（金）まで投票受付中！</t>
         </is>
       </c>
     </row>
@@ -50393,17 +51430,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第８０話　パルクールの戦いが始まった（２）</t>
+          <t>第７８話『寒天停止』④</t>
         </is>
       </c>
     </row>
@@ -50413,17 +51450,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第87話その2</t>
+          <t>コミックス最新第4巻絶賛発売中!!</t>
         </is>
       </c>
     </row>
@@ -50433,17 +51470,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第10話 後編</t>
+          <t>第８１話　デカ盛りの戦いが始まった（１）</t>
         </is>
       </c>
     </row>
@@ -50453,17 +51490,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+          <t>いとこのこ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+          <t>いぬちく(著者)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第23話後半</t>
+          <t>第54話</t>
         </is>
       </c>
     </row>
@@ -50473,17 +51510,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第137話　ひさびさに本気出してみるⅡ（後編）</t>
+          <t>第7話後編：不穏な依頼</t>
         </is>
       </c>
     </row>
@@ -50493,17 +51530,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>板垣恵介 猪原賽 陸井栄史</t>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第98話　経験値</t>
+          <t>第11話-1</t>
         </is>
       </c>
     </row>
@@ -50513,17 +51550,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>異世界のんびり農家</t>
+          <t>描けないのでヤってみた</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+          <t>逢上おかき(著者)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第327話</t>
+          <t>第2話</t>
         </is>
       </c>
     </row>
@@ -50533,17 +51570,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第23話前半</t>
+          <t>おまけ74</t>
         </is>
       </c>
     </row>
@@ -50553,17 +51590,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+          <t>ダークサモナーとデキている</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+          <t>車王(著者)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第39話</t>
+          <t>第93話</t>
         </is>
       </c>
     </row>
@@ -50573,17 +51610,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第147話　ユリヤの正体・後編</t>
+          <t>第8話 邂逅</t>
         </is>
       </c>
     </row>
@@ -50593,17 +51630,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>異世界のんびり農家</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第82話➁</t>
+          <t>第328話</t>
         </is>
       </c>
     </row>
@@ -50613,17 +51650,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>モリタ Ｕ４ nima</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第16話（４）　太っちょ貴族と摩訶不思議なる肉料理　（４）</t>
+          <t>第5話②</t>
         </is>
       </c>
     </row>
@@ -50633,17 +51670,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+          <t>「おかえり、パパ」</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ヨウハ(著者)</t>
+          <t>蝉丸</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第2話-1</t>
+          <t>特別編「質問」</t>
         </is>
       </c>
     </row>
@@ -50653,17 +51690,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第13話</t>
+          <t>第６１話　他領へ向かう器用貧乏（１）</t>
         </is>
       </c>
     </row>
@@ -50673,17 +51710,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第39話 独身貴族は写真展を開く（4）</t>
+          <t>第82話③</t>
         </is>
       </c>
     </row>
@@ -50693,17 +51730,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>濁る瞳で何を願う ハイセルク戦記</t>
+          <t>淫獄団地</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>トルトネン 創-taro 斎藤八呑</t>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第41話 統率者について</t>
+          <t>第59話（前編）</t>
         </is>
       </c>
     </row>
@@ -50713,17 +51750,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>ヨウハ(著者)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第68話①　休暇を満喫してみた</t>
+          <t>第2話-2</t>
         </is>
       </c>
     </row>
@@ -50733,17 +51770,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+          <t>お前がヤったんだろ！</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+          <t>クシザキ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第15話-2：一番弟子の卒業</t>
+          <t>第13話	いまさら部活といわれても</t>
         </is>
       </c>
     </row>
@@ -50753,17 +51790,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>板垣恵介 林たかあき</t>
+          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第72話 ムサシ</t>
+          <t>第46話-2</t>
         </is>
       </c>
     </row>
@@ -50773,17 +51810,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>骸骨騎士様、只今異世界へお出掛け中</t>
+          <t>アザミヤコを好きになる</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>サワノアキラ（漫画） 秤猿鬼（原作） KeG（キャラクター原案）</t>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第68章　龍王の会談（前編）</t>
+          <t>第16話</t>
         </is>
       </c>
     </row>
@@ -50793,17 +51830,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>女友達は頼めば意外とヤらせてくれる</t>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ろくろ(漫画) 鏡遊(原作)</t>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第33話②</t>
+          <t>第53話 友の兄とお茶会を③</t>
         </is>
       </c>
     </row>
@@ -50813,17 +51850,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>聖者無双</t>
+          <t>衛宮さんちの今日のごはん</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+          <t>TAa(漫画) 只野まこと(料理監修) ＴＹＰＥ－ＭＯＯＮ(原作)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第99話　リザリア②</t>
+          <t>第79話</t>
         </is>
       </c>
     </row>
@@ -50833,17 +51870,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>ダンジョンの幼なじみ</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>久真やすひさ(著者)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第155話 よくわからないけれどじぇじぇじぇな事態のようです（２）</t>
+          <t>※アライブクイーン投票用：7/31（金）まで投票受付中！</t>
         </is>
       </c>
     </row>
@@ -50853,17 +51890,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>めちゃくちゃ追放される話</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>杉浦次郎 向浦宏和</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第４話（中編）</t>
+          <t>拷問189</t>
         </is>
       </c>
     </row>
@@ -50873,17 +51910,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第４８話　勇者、弟のために作った剣が、凄すぎて自我を持つ（５）</t>
+          <t>第156話 よくわからないけれどサバイバルするみたいです（１）</t>
         </is>
       </c>
     </row>
@@ -50893,17 +51930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>骸骨騎士様、只今異世界へお出掛け中</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>サワノアキラ（漫画） 秤猿鬼（原作） KeG（キャラクター原案）</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>拷問188</t>
+          <t>第68章　龍王の会談（後編）</t>
         </is>
       </c>
     </row>
@@ -50913,17 +51950,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+          <t>バーサス</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第10話-2：初めてのお友達？</t>
+          <t>第34話 思い知れ（2）</t>
         </is>
       </c>
     </row>
@@ -50943,7 +51980,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第88話その4</t>
+          <t>第89話その1</t>
         </is>
       </c>
     </row>
@@ -50953,17 +51990,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>回復術士のやり直し</t>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第78話-2</t>
+          <t>第2話-2</t>
         </is>
       </c>
     </row>
@@ -50973,17 +52010,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>小林さんちのメイドラゴン</t>
+          <t>幼女戦記</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>クール教信者</t>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第168話</t>
+          <t>第百十五章：ドードーバード航空戦Ⅹ</t>
         </is>
       </c>
     </row>
@@ -50993,17 +52030,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>インフィニット・デンドログラム</t>
+          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
+          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第79話</t>
+          <t>第31話</t>
         </is>
       </c>
     </row>
@@ -51013,17 +52050,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>【目つき悪いシリーズ】ミタメトウラハラ</t>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ウラベスナヒト</t>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>#13誘惑</t>
+          <t>第9話-2</t>
         </is>
       </c>
     </row>
@@ -51033,17 +52070,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
+          <t>ウォルテニア戦記</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>六志麻あさ 業務用餅 kisui</t>
+          <t>漫画：八木ゆかり 原作：保利亮太 キャラクター原案：bob</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第８８話</t>
+          <t>第61話</t>
         </is>
       </c>
     </row>
@@ -51053,17 +52090,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>俺は星間国家の悪徳領主！</t>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第48話　化け物共</t>
+          <t>冥府の休載まんが</t>
         </is>
       </c>
     </row>
@@ -51073,17 +52110,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第7話(2)</t>
+          <t>第10話-2</t>
         </is>
       </c>
     </row>
@@ -51093,17 +52130,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第24話③</t>
+          <t>第7話(2)</t>
         </is>
       </c>
     </row>
@@ -51113,17 +52150,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+          <t>転生剣豪ズバババァーン！！</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+          <t>富士田けやき(原作) 坂崎ふれでぃ(作画)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第88話 悩める原口監督！</t>
+          <t>第3話</t>
         </is>
       </c>
     </row>
@@ -51133,17 +52170,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>三枝さんはメガネ先輩と恋を描く</t>
+          <t>おせっかい女子、恋をする</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>セレビィ量産型(著者)</t>
+          <t>音竹 ひかる(著者)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第28話前半</t>
+          <t>第22話</t>
         </is>
       </c>
     </row>
@@ -51153,17 +52190,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+          <t>塔の管理をしてみよう</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>KAKERU</t>
+          <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第77話「最前線」（後半）</t>
+          <t>第102話</t>
         </is>
       </c>
     </row>
@@ -51173,17 +52210,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>追放僧侶の賢者タイム</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>原作・野原のはて 作画・鈴木シオン</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>特別編㉔</t>
+          <t>第6話　賢者に至る道</t>
         </is>
       </c>
     </row>
@@ -51193,17 +52230,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+          <t>ライブダンジョン！</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>漫画/すたひろ 原作/Y.A</t>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>chapter88【46話①】</t>
+          <t>第97話後半</t>
         </is>
       </c>
     </row>
@@ -51213,17 +52250,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>男子高校生だけどギャルにTSしました</t>
+          <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>太陽まりい(著者)</t>
+          <t>岡沢六十四 るれくちぇ sage・ジョー</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第27話前編</t>
+          <t>第82話(前編) インフェルノ襲来</t>
         </is>
       </c>
     </row>
@@ -51233,17 +52270,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+          <t>めっちゃ召喚された件 THE COMIC</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>EP.27②</t>
+          <t>第56話①</t>
         </is>
       </c>
     </row>
@@ -51253,17 +52290,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ギャルの自転車を直したら懐かれた</t>
+          <t>黄金の経験値</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>タケチケイ（漫画） 生姜寧也（原作）</t>
+          <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第2話　ギャルと弁当を食べた（後編）</t>
+          <t>第26話</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-07-06
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -61,6 +61,7 @@
     <sheet name="2026-06-15" sheetId="53" state="visible" r:id="rId53"/>
     <sheet name="2026-06-22" sheetId="54" state="visible" r:id="rId54"/>
     <sheet name="2026-06-29" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="2026-07-06" sheetId="56" state="visible" r:id="rId56"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -51305,22 +51306,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第138話</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>異世界おじさん</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>殆ど死んでいる(著者)</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第78話</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>ワンパンマン</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>230撃目</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第49話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第24話-1「父と子と」</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>※アライブクイーン投票用：7/31（金）まで投票受付中！</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第７８話『寒天停止』④</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>コミックス最新第4巻絶賛発売中!!</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第８１話　デカ盛りの戦いが始まった（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>いとこのこ</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>いぬちく(著者)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第54話</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第7話後編：不穏な依頼</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第11話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>描けないのでヤってみた</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>逢上おかき(著者)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第2話</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>おまけ74</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第93話</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第8話 邂逅</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第328話</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第5話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>「おかえり、パパ」</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>蝉丸</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>特別編「質問」</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第６１話　他領へ向かう器用貧乏（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第82話③</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>淫獄団地</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第59話（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>ヨウハ(著者)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第2話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>クシザキ</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第13話	いまさら部活といわれても</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第46話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>アザミヤコを好きになる</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第16話</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第53話 友の兄とお茶会を③</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>衛宮さんちの今日のごはん</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>TAa(漫画) 只野まこと(料理監修) ＴＹＰＥ－ＭＯＯＮ(原作)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第79話</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>ダンジョンの幼なじみ</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>久真やすひさ(著者)</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>※アライブクイーン投票用：7/31（金）まで投票受付中！</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>拷問189</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第156話 よくわからないけれどサバイバルするみたいです（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>骸骨騎士様、只今異世界へお出掛け中</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>サワノアキラ（漫画） 秤猿鬼（原作） KeG（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第68章　龍王の会談（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>バーサス</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第34話 思い知れ（2）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第89話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第2話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>幼女戦記</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第百十五章：ドードーバード航空戦Ⅹ</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第31話</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第9話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>ウォルテニア戦記</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>漫画：八木ゆかり 原作：保利亮太 キャラクター原案：bob</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第61話</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>冥府の休載まんが</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第10話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第7話(2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>転生剣豪ズバババァーン！！</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>富士田けやき(原作) 坂崎ふれでぃ(作画)</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第3話</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第22話</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>塔の管理をしてみよう</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第102話</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>追放僧侶の賢者タイム</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>原作・野原のはて 作画・鈴木シオン</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第6話　賢者に至る道</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>ライブダンジョン！</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第97話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>岡沢六十四 るれくちぇ sage・ジョー</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第82話(前編) インフェルノ襲来</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>めっちゃ召喚された件 THE COMIC</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第56話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>黄金の経験値</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第26話</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>宇崎ちゃんは遊びたい！</t>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>丈(著者)</t>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第138話</t>
+          <t>第80話 後編</t>
         </is>
       </c>
     </row>
@@ -51330,17 +52367,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>異世界おじさん</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>殆ど死んでいる(著者)</t>
+          <t>むちまろ</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第78話</t>
+          <t>第155話	こまろの世界Ⅲ</t>
         </is>
       </c>
     </row>
@@ -51350,17 +52387,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ワンパンマン</t>
+          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>原作/ＯＮＥ 作画/村田雄介</t>
+          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>230撃目</t>
+          <t>第80話</t>
         </is>
       </c>
     </row>
@@ -51370,17 +52407,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>魔術師クノンは見えている</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第49話①</t>
+          <t>第８１話　デカ盛りの戦いが始まった（２）</t>
         </is>
       </c>
     </row>
@@ -51390,17 +52427,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第24話-1「父と子と」</t>
+          <t>第88話その1</t>
         </is>
       </c>
     </row>
@@ -51410,17 +52447,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>※アライブクイーン投票用：7/31（金）まで投票受付中！</t>
+          <t>第12話</t>
         </is>
       </c>
     </row>
@@ -51430,17 +52467,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>王子様の友達</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>すけろく(著者)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第７８話『寒天停止』④</t>
+          <t>第38話</t>
         </is>
       </c>
     </row>
@@ -51450,17 +52487,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>コミックス最新第4巻絶賛発売中!!</t>
+          <t>第24話</t>
         </is>
       </c>
     </row>
@@ -51470,17 +52507,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>帰ってください！ 阿久津さん</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>長岡太一(著者)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第８１話　デカ盛りの戦いが始まった（１）</t>
+          <t>第208話</t>
         </is>
       </c>
     </row>
@@ -51490,17 +52527,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>いとこのこ</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>いぬちく(著者)</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第54話</t>
+          <t>第138話　ひさびさに本気出してみるⅢ（前編）</t>
         </is>
       </c>
     </row>
@@ -51510,17 +52547,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+          <t>不純な彼女達は懺悔しない</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+          <t>ポロロッカ(著者)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第7話後編：不穏な依頼</t>
+          <t>最終話</t>
         </is>
       </c>
     </row>
@@ -51530,17 +52567,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>三部べべ(漫画) ねうしとら(原作)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第11話-1</t>
+          <t>第148話　ヴィーイとの対決・前編</t>
         </is>
       </c>
     </row>
@@ -51550,17 +52587,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>描けないのでヤってみた</t>
+          <t>クセ強彼女は床にいざなう</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>逢上おかき(著者)</t>
+          <t>須河篤志(著者)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第2話</t>
+          <t>第23話後半</t>
         </is>
       </c>
     </row>
@@ -51570,17 +52607,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>おまけ74</t>
+          <t>第82話④</t>
         </is>
       </c>
     </row>
@@ -51590,17 +52627,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ダークサモナーとデキている</t>
+          <t>田舎で恋は難しい!?</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>車王(著者)</t>
+          <t>ねこうめ(著者)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第93話</t>
+          <t>第8話</t>
         </is>
       </c>
     </row>
@@ -51610,17 +52647,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+          <t>まんきつしたい常連さん</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+          <t>しんみりん(著者)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第8話 邂逅</t>
+          <t>第57話前編</t>
         </is>
       </c>
     </row>
@@ -51630,17 +52667,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>異世界のんびり農家</t>
+          <t>剥かせて！竜ケ崎さん</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+          <t>一智和智</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第328話</t>
+          <t>大学生編 第22話</t>
         </is>
       </c>
     </row>
@@ -51650,17 +52687,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第5話②</t>
+          <t>第６１話　他領へ向かう器用貧乏（２）</t>
         </is>
       </c>
     </row>
@@ -51670,17 +52707,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>「おかえり、パパ」</t>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>蝉丸</t>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>特別編「質問」</t>
+          <t>第３０食　シルバーホーンのステーキ、パクパクですわ！（その２）（２）</t>
         </is>
       </c>
     </row>
@@ -51690,17 +52727,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>このヒーラー、めんどくさい</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>丹念に発酵(著者)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第６１話　他領へ向かう器用貧乏（１）</t>
+          <t>第99話：石棺</t>
         </is>
       </c>
     </row>
@@ -51710,17 +52747,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第82話③</t>
+          <t>第40話 独身貴族は友人を実家に連れていく（1）</t>
         </is>
       </c>
     </row>
@@ -51730,17 +52767,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>淫獄団地</t>
+          <t>ぽんドロイド！ はまさん</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+          <t>はれやまはれぞう(著者)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第59話（前編）</t>
+          <t>第22話</t>
         </is>
       </c>
     </row>
@@ -51750,17 +52787,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ヨウハ(著者)</t>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第2話-2</t>
+          <t>第11話前編</t>
         </is>
       </c>
     </row>
@@ -51770,17 +52807,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>お前がヤったんだろ！</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>クシザキ</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第13話	いまさら部活といわれても</t>
+          <t>第68話②　休暇を満喫してみた</t>
         </is>
       </c>
     </row>
@@ -51790,17 +52827,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
+          <t>異世界食堂　洋食のねこや</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
+          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第46話-2</t>
+          <t>第47話➁</t>
         </is>
       </c>
     </row>
@@ -51810,17 +52847,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>アザミヤコを好きになる</t>
+          <t>魔のものたちは企てる</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+          <t>加藤拓弐(原作) ガしガし(作画)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第16話</t>
+          <t>単行本4巻告知＆休載イラスト</t>
         </is>
       </c>
     </row>
@@ -51830,17 +52867,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+          <t>セレビィ量産型(著者)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第53話 友の兄とお茶会を③</t>
+          <t>第28話後半</t>
         </is>
       </c>
     </row>
@@ -51850,17 +52887,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>衛宮さんちの今日のごはん</t>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>TAa(漫画) 只野まこと(料理監修) ＴＹＰＥ－ＭＯＯＮ(原作)</t>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第79話</t>
+          <t>第16話-1：落ちていく少女</t>
         </is>
       </c>
     </row>
@@ -51870,17 +52907,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ダンジョンの幼なじみ</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>久真やすひさ(著者)</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>※アライブクイーン投票用：7/31（金）まで投票受付中！</t>
+          <t>第156話 よくわからないけれどサバイバルするみたいです（２）</t>
         </is>
       </c>
     </row>
@@ -51890,17 +52927,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>聖者無双</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>拷問189</t>
+          <t>第100話　将来の夢と目標①</t>
         </is>
       </c>
     </row>
@@ -51910,17 +52947,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>原作:剃り残し 漫画:大窪太一</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第156話 よくわからないけれどサバイバルするみたいです（１）</t>
+          <t>第9話</t>
         </is>
       </c>
     </row>
@@ -51930,17 +52967,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>骸骨騎士様、只今異世界へお出掛け中</t>
+          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>サワノアキラ（漫画） 秤猿鬼（原作） KeG（キャラクター原案）</t>
+          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第68章　龍王の会談（後編）</t>
+          <t>第47話-2</t>
         </is>
       </c>
     </row>
@@ -51950,17 +52987,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>バーサス</t>
+          <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+          <t>クール教信者</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第34話 思い知れ（2）</t>
+          <t>第169話</t>
         </is>
       </c>
     </row>
@@ -51970,17 +53007,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>幼女戦記</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第89話その1</t>
+          <t>第百十六章：邂逅Ⅰ</t>
         </is>
       </c>
     </row>
@@ -51990,17 +53027,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+          <t>「お相手は一般の方です」</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+          <t>嵯峨祐介(著者)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第2話-2</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -52010,17 +53047,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>幼女戦記</t>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第百十五章：ドードーバード航空戦Ⅹ</t>
+          <t>第11話-1：仲良くしましょう！</t>
         </is>
       </c>
     </row>
@@ -52030,17 +53067,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
+          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
+          <t>六志麻あさ 業務用餅 kisui</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第31話</t>
+          <t>第８９話</t>
         </is>
       </c>
     </row>
@@ -52050,17 +53087,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第9話-2</t>
+          <t>第89話 雨月の隠された秘密！</t>
         </is>
       </c>
     </row>
@@ -52070,17 +53107,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ウォルテニア戦記</t>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>漫画：八木ゆかり 原作：保利亮太 キャラクター原案：bob</t>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第61話</t>
+          <t>特別イラスト</t>
         </is>
       </c>
     </row>
@@ -52090,17 +53127,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>冥府の休載まんが</t>
+          <t>拷問190</t>
         </is>
       </c>
     </row>
@@ -52110,17 +53147,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+          <t>くらいあの子としたいこと</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+          <t>碇マナツ(著者)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第10話-2</t>
+          <t>特別編㉕</t>
         </is>
       </c>
     </row>
@@ -52130,17 +53167,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+          <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第7話(2)</t>
+          <t>第22話　最弱貴族、伯爵を撃退する(１)</t>
         </is>
       </c>
     </row>
@@ -52150,17 +53187,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>転生剣豪ズバババァーン！！</t>
+          <t>役目を果たした日陰の勇者は、辺境で自由に生きていきます</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>富士田けやき(原作) 坂崎ふれでぃ(作画)</t>
+          <t>船野真帆(作画) 丘野優(原作) 布施龍太(キャラクター原案)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第3話</t>
+          <t>第16話後半</t>
         </is>
       </c>
     </row>
@@ -52170,17 +53207,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>おせっかい女子、恋をする</t>
+          <t>ギャル神官はリザレがダルい</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>音竹 ひかる(著者)</t>
+          <t>秋★枝</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第22話</t>
+          <t>第7話</t>
         </is>
       </c>
     </row>
@@ -52190,17 +53227,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>塔の管理をしてみよう</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第102話</t>
+          <t>第138話</t>
         </is>
       </c>
     </row>
@@ -52210,17 +53247,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>追放僧侶の賢者タイム</t>
+          <t>めちゃくちゃ追放される話</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>原作・野原のはて 作画・鈴木シオン</t>
+          <t>杉浦次郎 向浦宏和</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第6話　賢者に至る道</t>
+          <t>第４話（後編）</t>
         </is>
       </c>
     </row>
@@ -52230,17 +53267,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ライブダンジョン！</t>
+          <t>美容スキルでクラスの女の子を可愛くしたい</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+          <t>藤白ぺるか(原作) 紺野あずれ(漫画) 水野早桜(キャラクター原案)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第97話後半</t>
+          <t>第7話</t>
         </is>
       </c>
     </row>
@@ -52250,17 +53287,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
+          <t>おせっかい女子、恋をする</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>岡沢六十四 るれくちぇ sage・ジョー</t>
+          <t>音竹 ひかる(著者)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第82話(前編) インフェルノ襲来</t>
+          <t>第23話</t>
         </is>
       </c>
     </row>
@@ -52270,17 +53307,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>めっちゃ召喚された件 THE COMIC</t>
+          <t>魔法少女リリカルなのは EXCEEDS</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
+          <t>都築真紀 川上修一</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第56話①</t>
+          <t>第１３話②</t>
         </is>
       </c>
     </row>
@@ -52290,17 +53327,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>黄金の経験値</t>
+          <t>異世界おじさん</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
+          <t>殆ど死んでいる(著者)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第26話</t>
+          <t>第78話</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-07-13
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -62,6 +62,7 @@
     <sheet name="2026-06-22" sheetId="54" state="visible" r:id="rId54"/>
     <sheet name="2026-06-29" sheetId="55" state="visible" r:id="rId55"/>
     <sheet name="2026-07-06" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="2026-07-13" sheetId="57" state="visible" r:id="rId57"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -52342,22 +52343,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第80話 後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第155話	こまろの世界Ⅲ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第80話</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第８１話　デカ盛りの戦いが始まった（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第88話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第12話</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>王子様の友達</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>すけろく(著者)</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第38話</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第24話</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>帰ってください！ 阿久津さん</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>長岡太一(著者)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第208話</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第138話　ひさびさに本気出してみるⅢ（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>不純な彼女達は懺悔しない</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>ポロロッカ(著者)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>最終話</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第148話　ヴィーイとの対決・前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第23話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第82話④</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>田舎で恋は難しい!?</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>ねこうめ(著者)</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第8話</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>まんきつしたい常連さん</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>しんみりん(著者)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第57話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>剥かせて！竜ケ崎さん</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>一智和智</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>大学生編 第22話</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第６１話　他領へ向かう器用貧乏（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第３０食　シルバーホーンのステーキ、パクパクですわ！（その２）（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>このヒーラー、めんどくさい</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>丹念に発酵(著者)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第99話：石棺</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第40話 独身貴族は友人を実家に連れていく（1）</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>ぽんドロイド！ はまさん</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>はれやまはれぞう(著者)</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第22話</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第11話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第68話②　休暇を満喫してみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>異世界食堂　洋食のねこや</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第47話➁</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>魔のものたちは企てる</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>加藤拓弐(原作) ガしガし(作画)</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>単行本4巻告知＆休載イラスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第28話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第16話-1：落ちていく少女</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第156話 よくわからないけれどサバイバルするみたいです（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>聖者無双</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第100話　将来の夢と目標①</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>原作:剃り残し 漫画:大窪太一</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第9話</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第47話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>小林さんちのメイドラゴン</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>クール教信者</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第169話</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>幼女戦記</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第百十六章：邂逅Ⅰ</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>「お相手は一般の方です」</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>嵯峨祐介(著者)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第11話-1：仲良くしましょう！</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>六志麻あさ 業務用餅 kisui</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第８９話</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第89話 雨月の隠された秘密！</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>特別イラスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>拷問190</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>特別編㉕</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>空野進 sorani ファルまろ</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第22話　最弱貴族、伯爵を撃退する(１)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>役目を果たした日陰の勇者は、辺境で自由に生きていきます</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>船野真帆(作画) 丘野優(原作) 布施龍太(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第16話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>ギャル神官はリザレがダルい</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>秋★枝</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第7話</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第138話</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>めちゃくちゃ追放される話</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>杉浦次郎 向浦宏和</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第４話（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>美容スキルでクラスの女の子を可愛くしたい</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>藤白ぺるか(原作) 紺野あずれ(漫画) 水野早桜(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第7話</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第23話</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>魔法少女リリカルなのは EXCEEDS</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>都築真紀 川上修一</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第１３話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>異世界おじさん</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>殆ど死んでいる(著者)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第78話</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第80話 後編</t>
+          <t>231撃目</t>
         </is>
       </c>
     </row>
@@ -52367,17 +53404,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>不徳のギルド</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>河添太一</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第155話	こまろの世界Ⅲ</t>
+          <t>第１０８話：煩悩ガール</t>
         </is>
       </c>
     </row>
@@ -52387,17 +53424,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
+          <t>魔術師クノンは見えている</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第80話</t>
+          <t>第49話②</t>
         </is>
       </c>
     </row>
@@ -52407,17 +53444,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第８１話　デカ盛りの戦いが始まった（２）</t>
+          <t>第40話：親友だから①</t>
         </is>
       </c>
     </row>
@@ -52427,17 +53464,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第88話その1</t>
+          <t>第24話-2「父と子と」</t>
         </is>
       </c>
     </row>
@@ -52447,17 +53484,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+          <t>いとこのこ</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+          <t>いぬちく(著者)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第12話</t>
+          <t>第55話</t>
         </is>
       </c>
     </row>
@@ -52467,17 +53504,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>王子様の友達</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>すけろく(著者)</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第38話</t>
+          <t>第７９話『呉越停止』①</t>
         </is>
       </c>
     </row>
@@ -52487,17 +53524,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第24話</t>
+          <t>第８２話　恋愛相談の戦いが始まった</t>
         </is>
       </c>
     </row>
@@ -52507,17 +53544,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>帰ってください！ 阿久津さん</t>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>長岡太一(著者)</t>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第208話</t>
+          <t>第21話-1</t>
         </is>
       </c>
     </row>
@@ -52527,17 +53564,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第138話　ひさびさに本気出してみるⅢ（前編）</t>
+          <t>第8話前編：アトリ</t>
         </is>
       </c>
     </row>
@@ -52547,17 +53584,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>不純な彼女達は懺悔しない</t>
+          <t>ダンジョンの幼なじみ</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ポロロッカ(著者)</t>
+          <t>久真やすひさ(著者)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>最終話</t>
+          <t>第66話</t>
         </is>
       </c>
     </row>
@@ -52567,17 +53604,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第148話　ヴィーイとの対決・前編</t>
+          <t>第138話　ひさびさに本気出してみるⅢ（中編）</t>
         </is>
       </c>
     </row>
@@ -52587,17 +53624,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>久遠まこと(著者) 石のやっさん(原作)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第23話後半</t>
+          <t>第38話</t>
         </is>
       </c>
     </row>
@@ -52607,17 +53644,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>金属スライムを倒しまくった俺が【黒鋼の王】と呼ばれるまで</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>藤屋いずこ(著者) 温泉カピバラ(原作) 山椒魚(キャラクター原案)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第82話④</t>
+          <t>第20章</t>
         </is>
       </c>
     </row>
@@ -52627,17 +53664,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>田舎で恋は難しい!?</t>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ねこうめ(著者)</t>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第8話</t>
+          <t>第99話　進化(スキルアップ)</t>
         </is>
       </c>
     </row>
@@ -52647,17 +53684,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>まんきつしたい常連さん</t>
+          <t>ダークサモナーとデキている</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>しんみりん(著者)</t>
+          <t>車王(著者)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第57話前編</t>
+          <t>第94話</t>
         </is>
       </c>
     </row>
@@ -52667,17 +53704,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>剥かせて！竜ケ崎さん</t>
+          <t>まんきつしたい常連さん</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>一智和智</t>
+          <t>しんみりん(著者)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>大学生編 第22話</t>
+          <t>第57話中編</t>
         </is>
       </c>
     </row>
@@ -52687,17 +53724,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第６１話　他領へ向かう器用貧乏（２）</t>
+          <t>第148話　ヴィーイとの対決・後編</t>
         </is>
       </c>
     </row>
@@ -52707,17 +53744,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>島知宏 音速炒飯 有都あらゆる</t>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第３０食　シルバーホーンのステーキ、パクパクですわ！（その２）（２）</t>
+          <t>第9話 師匠</t>
         </is>
       </c>
     </row>
@@ -52727,17 +53764,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>このヒーラー、めんどくさい</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>丹念に発酵(著者)</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第99話：石棺</t>
+          <t>第83話①</t>
         </is>
       </c>
     </row>
@@ -52747,17 +53784,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+          <t>淫獄団地</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第40話 独身貴族は友人を実家に連れていく（1）</t>
+          <t>第59話（後編）</t>
         </is>
       </c>
     </row>
@@ -52767,17 +53804,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ぽんドロイド！ はまさん</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>はれやまはれぞう(著者)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第22話</t>
+          <t>第６１話　他領へ向かう器用貧乏（３）</t>
         </is>
       </c>
     </row>
@@ -52787,17 +53824,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+          <t>お前がヤったんだろ！</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+          <t>クシザキ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第11話前編</t>
+          <t>第14話	童貞遊戯</t>
         </is>
       </c>
     </row>
@@ -52807,17 +53844,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第68話②　休暇を満喫してみた</t>
+          <t>第３０食　シルバーホーンのステーキ、パクパクですわ！（その２）（３）</t>
         </is>
       </c>
     </row>
@@ -52827,17 +53864,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>異世界食堂　洋食のねこや</t>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
+          <t>ヨウハ(著者)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第47話➁</t>
+          <t>第3話-1</t>
         </is>
       </c>
     </row>
@@ -52847,17 +53884,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>魔のものたちは企てる</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>加藤拓弐(原作) ガしガし(作画)</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>単行本4巻告知＆休載イラスト</t>
+          <t>第5話③</t>
         </is>
       </c>
     </row>
@@ -52867,17 +53904,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>三枝さんはメガネ先輩と恋を描く</t>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>セレビィ量産型(著者)</t>
+          <t>モリタ Ｕ４ nima</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第28話後半</t>
+          <t>第17話（１）　クリスティーナお姉さまの結婚（１）</t>
         </is>
       </c>
     </row>
@@ -52887,17 +53924,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第16話-1：落ちていく少女</t>
+          <t>第40話 独身貴族は友人を実家に連れていく（2）</t>
         </is>
       </c>
     </row>
@@ -52907,17 +53944,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>幼女戦記</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第156話 よくわからないけれどサバイバルするみたいです（２）</t>
+          <t>第百十七章：邂逅Ⅱ</t>
         </is>
       </c>
     </row>
@@ -52927,17 +53964,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>聖者無双</t>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+          <t>板垣恵介 林たかあき</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第100話　将来の夢と目標①</t>
+          <t>第73話 慈愛</t>
         </is>
       </c>
     </row>
@@ -52947,17 +53984,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>原作:剃り残し 漫画:大窪太一</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第9話</t>
+          <t>第69話①　あにめを見てみた</t>
         </is>
       </c>
     </row>
@@ -52967,17 +54004,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第47話-2</t>
+          <t>第89話その2</t>
         </is>
       </c>
     </row>
@@ -52987,17 +54024,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>小林さんちのメイドラゴン</t>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>クール教信者</t>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第169話</t>
+          <t>第49話　奴の罪（前編）</t>
         </is>
       </c>
     </row>
@@ -53007,17 +54044,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>幼女戦記</t>
+          <t>「おかえり、パパ」</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
+          <t>蝉丸</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第百十六章：邂逅Ⅰ</t>
+          <t>単行本6巻限定描きおろし「都子の一日」試し読み</t>
         </is>
       </c>
     </row>
@@ -53027,17 +54064,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>「お相手は一般の方です」</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>嵯峨祐介(著者)</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>第４９話　ガイアスと剣神、激戦を繰り広げる。勇者は、オカモトさんに不吉な占いをされてしまう（１）</t>
         </is>
       </c>
     </row>
@@ -53047,17 +54084,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+          <t>如意自在(著者)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第11話-1：仲良くしましょう！</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -53067,17 +54104,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>六志麻あさ 業務用餅 kisui</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第８９話</t>
+          <t>第157話 よくわからないけれど清算してもらうみたいです（１）</t>
         </is>
       </c>
     </row>
@@ -53087,17 +54124,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+          <t>英雄王、武を極めるため転生す ～そして、世界最強の見習い騎士♀～</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+          <t>漫画‥くろむら基人 原作‥ハヤケン キャラクター原案‥Nagu</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第89話 雨月の隠された秘密！</t>
+          <t>第34話 前編</t>
         </is>
       </c>
     </row>
@@ -53107,17 +54144,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>女友達は頼めば意外とヤらせてくれる</t>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ろくろ(漫画) 鏡遊(原作)</t>
+          <t>はぐはぐ(著者)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>特別イラスト</t>
+          <t>第101話前編</t>
         </is>
       </c>
     </row>
@@ -53127,17 +54164,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>拷問190</t>
+          <t>第3話-1</t>
         </is>
       </c>
     </row>
@@ -53147,17 +54184,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>特別編㉕</t>
+          <t>第4話-①</t>
         </is>
       </c>
     </row>
@@ -53167,17 +54204,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>空野進 sorani ファルまろ</t>
+          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第22話　最弱貴族、伯爵を撃退する(１)</t>
+          <t>第5話</t>
         </is>
       </c>
     </row>
@@ -53187,17 +54224,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>役目を果たした日陰の勇者は、辺境で自由に生きていきます</t>
+          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>船野真帆(作画) 丘野優(原作) 布施龍太(キャラクター原案)</t>
+          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第16話後半</t>
+          <t>第66話　扉の先へ</t>
         </is>
       </c>
     </row>
@@ -53207,17 +54244,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ギャル神官はリザレがダルい</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>秋★枝</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第7話</t>
+          <t>拷問191</t>
         </is>
       </c>
     </row>
@@ -53227,17 +54264,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>宇崎ちゃんは遊びたい！</t>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>丈(著者)</t>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第138話</t>
+          <t>第10話-1</t>
         </is>
       </c>
     </row>
@@ -53247,17 +54284,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>めちゃくちゃ追放される話</t>
+          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>杉浦次郎 向浦宏和</t>
+          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第４話（後編）</t>
+          <t>第4話</t>
         </is>
       </c>
     </row>
@@ -53267,17 +54304,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>美容スキルでクラスの女の子を可愛くしたい</t>
+          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>藤白ぺるか(原作) 紺野あずれ(漫画) 水野早桜(キャラクター原案)</t>
+          <t>FUNA 東西 モトエ恵介</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第7話</t>
+          <t>第131話 第2回異世界懇談会［その②］</t>
         </is>
       </c>
     </row>
@@ -53287,17 +54324,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>おせっかい女子、恋をする</t>
+          <t>描けないのでヤってみた</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>音竹 ひかる(著者)</t>
+          <t>逢上おかき(著者)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第23話</t>
+          <t>第3話</t>
         </is>
       </c>
     </row>
@@ -53307,17 +54344,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS</t>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>都築真紀 川上修一</t>
+          <t>KAKERU</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第１３話②</t>
+          <t>第78話「ケンタウロス」（前半）</t>
         </is>
       </c>
     </row>
@@ -53327,17 +54364,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>異世界おじさん</t>
+          <t>バーサス</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>殆ど死んでいる(著者)</t>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第78話</t>
+          <t>休載イラスト「退場魔王」</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-07-20
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -63,6 +63,7 @@
     <sheet name="2026-06-29" sheetId="55" state="visible" r:id="rId55"/>
     <sheet name="2026-07-06" sheetId="56" state="visible" r:id="rId56"/>
     <sheet name="2026-07-13" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="2026-07-20" sheetId="58" state="visible" r:id="rId58"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -53379,22 +53380,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>ワンパンマン</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>231撃目</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>不徳のギルド</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>河添太一</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第１０８話：煩悩ガール</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第49話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第40話：親友だから①</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第24話-2「父と子と」</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>いとこのこ</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>いぬちく(著者)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第55話</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第７９話『呉越停止』①</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第８２話　恋愛相談の戦いが始まった</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第21話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第8話前編：アトリ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>ダンジョンの幼なじみ</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>久真やすひさ(著者)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第66話</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第138話　ひさびさに本気出してみるⅢ（中編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>久遠まこと(著者) 石のやっさん(原作)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第38話</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>金属スライムを倒しまくった俺が【黒鋼の王】と呼ばれるまで</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>藤屋いずこ(著者) 温泉カピバラ(原作) 山椒魚(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第20章</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第99話　進化(スキルアップ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第94話</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>まんきつしたい常連さん</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>しんみりん(著者)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第57話中編</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第148話　ヴィーイとの対決・後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第9話 師匠</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第83話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>淫獄団地</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第59話（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第６１話　他領へ向かう器用貧乏（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>クシザキ</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第14話	童貞遊戯</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第３０食　シルバーホーンのステーキ、パクパクですわ！（その２）（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>ヨウハ(著者)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第3話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第5話③</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>モリタ Ｕ４ nima</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第17話（１）　クリスティーナお姉さまの結婚（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第40話 独身貴族は友人を実家に連れていく（2）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>幼女戦記</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第百十七章：邂逅Ⅱ</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 林たかあき</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第73話 慈愛</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第69話①　あにめを見てみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第89話その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第49話　奴の罪（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>「おかえり、パパ」</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>蝉丸</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>単行本6巻限定描きおろし「都子の一日」試し読み</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第４９話　ガイアスと剣神、激戦を繰り広げる。勇者は、オカモトさんに不吉な占いをされてしまう（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>如意自在(著者)</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第157話 よくわからないけれど清算してもらうみたいです（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>英雄王、武を極めるため転生す ～そして、世界最強の見習い騎士♀～</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>漫画‥くろむら基人 原作‥ハヤケン キャラクター原案‥Nagu</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第34話 前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>はぐはぐ(著者)</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第101話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第3話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第4話-①</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第5話</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第66話　扉の先へ</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>拷問191</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第10話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第4話</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>FUNA 東西 モトエ恵介</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第131話 第2回異世界懇談会［その②］</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>描けないのでヤってみた</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>逢上おかき(著者)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第3話</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>KAKERU</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第78話「ケンタウロス」（前半）</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>バーサス</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>休載イラスト「退場魔王」</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ワンパンマン</t>
+          <t>異種族レビュアーズ</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>原作/ＯＮＥ 作画/村田雄介</t>
+          <t>天原(原作) masha(作画)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>231撃目</t>
+          <t>第94話</t>
         </is>
       </c>
     </row>
@@ -53404,17 +54441,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>不徳のギルド</t>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>河添太一</t>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第１０８話：煩悩ガール</t>
+          <t>第81話 前編</t>
         </is>
       </c>
     </row>
@@ -53424,17 +54461,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>魔術師クノンは見えている</t>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第49話②</t>
+          <t>第40話：親友だから②</t>
         </is>
       </c>
     </row>
@@ -53444,17 +54481,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>zunta(作画) はらわたさいぞう(原作)</t>
+          <t>むちまろ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第40話：親友だから①</t>
+          <t>第156話	触覚フィードバックを主因とした外部非依存型報酬回路活性化メカニズムの予備的考察</t>
         </is>
       </c>
     </row>
@@ -53464,17 +54501,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第24話-2「父と子と」</t>
+          <t>第７９話『呉越停止』②</t>
         </is>
       </c>
     </row>
@@ -53484,17 +54521,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>いとこのこ</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>いぬちく(著者)</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第55話</t>
+          <t>第８３話　ラッキースケベの戦いが始まった（１）</t>
         </is>
       </c>
     </row>
@@ -53504,17 +54541,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第７９話『呉越停止』①</t>
+          <t>第12話後半</t>
         </is>
       </c>
     </row>
@@ -53524,17 +54561,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第８２話　恋愛相談の戦いが始まった</t>
+          <t>第88話その2</t>
         </is>
       </c>
     </row>
@@ -53544,17 +54581,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+          <t>帰ってください！ 阿久津さん</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+          <t>長岡太一(著者)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第21話-1</t>
+          <t>第209話</t>
         </is>
       </c>
     </row>
@@ -53564,17 +54601,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第8話前編：アトリ</t>
+          <t>第138話　ひさびさに本気出してみるⅢ（後編）</t>
         </is>
       </c>
     </row>
@@ -53584,17 +54621,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ダンジョンの幼なじみ</t>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>久真やすひさ(著者)</t>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第66話</t>
+          <t>第11話-2</t>
         </is>
       </c>
     </row>
@@ -53604,17 +54641,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第138話　ひさびさに本気出してみるⅢ（中編）</t>
+          <t>第17話-2</t>
         </is>
       </c>
     </row>
@@ -53624,17 +54661,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
+          <t>まんきつしたい常連さん</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>久遠まこと(著者) 石のやっさん(原作)</t>
+          <t>しんみりん(著者)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第38話</t>
+          <t>第57話後編</t>
         </is>
       </c>
     </row>
@@ -53644,17 +54681,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>金属スライムを倒しまくった俺が【黒鋼の王】と呼ばれるまで</t>
+          <t>クセ強彼女は床にいざなう</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>藤屋いずこ(著者) 温泉カピバラ(原作) 山椒魚(キャラクター原案)</t>
+          <t>須河篤志(著者)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第20章</t>
+          <t>第24話前半</t>
         </is>
       </c>
     </row>
@@ -53664,17 +54701,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>板垣恵介 猪原賽 陸井栄史</t>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第99話　進化(スキルアップ)</t>
+          <t>第40話</t>
         </is>
       </c>
     </row>
@@ -53684,17 +54721,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ダークサモナーとデキている</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>車王(著者)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第94話</t>
+          <t>第149話　復活！</t>
         </is>
       </c>
     </row>
@@ -53704,17 +54741,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>まんきつしたい常連さん</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>しんみりん(著者)</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第57話中編</t>
+          <t>第83話➁</t>
         </is>
       </c>
     </row>
@@ -53724,17 +54761,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>ぽんドロイド！ はまさん</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>はれやまはれぞう(著者)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第148話　ヴィーイとの対決・後編</t>
+          <t>第23話</t>
         </is>
       </c>
     </row>
@@ -53744,17 +54781,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+          <t>アザミヤコを好きになる</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第9話 師匠</t>
+          <t>第17話前編</t>
         </is>
       </c>
     </row>
@@ -53764,17 +54801,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第83話①</t>
+          <t>コミックス2巻発売告知記事</t>
         </is>
       </c>
     </row>
@@ -53784,17 +54821,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>淫獄団地</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第59話（後編）</t>
+          <t>第６２話　単独調査する器用貧乏（１）</t>
         </is>
       </c>
     </row>
@@ -53804,17 +54841,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第６１話　他領へ向かう器用貧乏（３）</t>
+          <t>第40話 独身貴族は友人を実家に連れていく（3）</t>
         </is>
       </c>
     </row>
@@ -53824,17 +54861,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>お前がヤったんだろ！</t>
+          <t>俺の担当は怪物</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>クシザキ</t>
+          <t>ぴざし(著者)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第14話	童貞遊戯</t>
+          <t>第3話前半</t>
         </is>
       </c>
     </row>
@@ -53864,17 +54901,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ヨウハ(著者)</t>
+          <t>夜州 nini 藻</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第3話-1</t>
+          <t>第76話（前編）</t>
         </is>
       </c>
     </row>
@@ -53884,17 +54921,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第5話③</t>
+          <t>第11話後編</t>
         </is>
       </c>
     </row>
@@ -53904,17 +54941,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>モリタ Ｕ４ nima</t>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第17話（１）　クリスティーナお姉さまの結婚（１）</t>
+          <t>第53話 友の兄とお茶会を④</t>
         </is>
       </c>
     </row>
@@ -53924,17 +54961,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第40話 独身貴族は友人を実家に連れていく（2）</t>
+          <t>拷問192</t>
         </is>
       </c>
     </row>
@@ -53944,17 +54981,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>幼女戦記</t>
+          <t>寿司ガキ</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
+          <t>ichika(著者)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第百十七章：邂逅Ⅱ</t>
+          <t>【マンガ総選挙出馬中】清き一票をお願いします！</t>
         </is>
       </c>
     </row>
@@ -53964,17 +55001,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>板垣恵介 林たかあき</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第73話 慈愛</t>
+          <t>【マンガ総選挙出馬中】清き一票をお願いします！</t>
         </is>
       </c>
     </row>
@@ -53984,17 +55021,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第69話①　あにめを見てみた</t>
+          <t>第16話-2：落ちていく少女</t>
         </is>
       </c>
     </row>
@@ -54004,17 +55041,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第89話その2</t>
+          <t>第157話 よくわからないけれど清算してもらうみたいです（２）</t>
         </is>
       </c>
     </row>
@@ -54024,17 +55061,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第49話　奴の罪（前編）</t>
+          <t>第４９話　ガイアスと剣神、激戦を繰り広げる。勇者は、オカモトさんに不吉な占いをされてしまう（２）</t>
         </is>
       </c>
     </row>
@@ -54044,17 +55081,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>「おかえり、パパ」</t>
+          <t>聖者無双</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>蝉丸</t>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>単行本6巻限定描きおろし「都子の一日」試し読み</t>
+          <t>第100話　将来の夢と目標②</t>
         </is>
       </c>
     </row>
@@ -54064,17 +55101,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第４９話　ガイアスと剣神、激戦を繰り広げる。勇者は、オカモトさんに不吉な占いをされてしまう（１）</t>
+          <t>第11話-2：仲良くしましょう！</t>
         </is>
       </c>
     </row>
@@ -54084,17 +55121,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+          <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>如意自在(著者)</t>
+          <t>クール教信者</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>第170話</t>
         </is>
       </c>
     </row>
@@ -54104,17 +55141,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>幼女戦記</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第157話 よくわからないけれど清算してもらうみたいです（１）</t>
+          <t>第百十八章-2：邂逅Ⅲ</t>
         </is>
       </c>
     </row>
@@ -54124,17 +55161,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>英雄王、武を極めるため転生す ～そして、世界最強の見習い騎士♀～</t>
+          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>漫画‥くろむら基人 原作‥ハヤケン キャラクター原案‥Nagu</t>
+          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第34話 前編</t>
+          <t>第65話　復讐からは、何も生まれない</t>
         </is>
       </c>
     </row>
@@ -54144,17 +55181,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>サーシャちゃんとクラスメイトオタクくん</t>
+          <t>くらいあの子としたいこと</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>はぐはぐ(著者)</t>
+          <t>碇マナツ(著者)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第101話前編</t>
+          <t>第99話</t>
         </is>
       </c>
     </row>
@@ -54164,17 +55201,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第3話-1</t>
+          <t>第11話-1</t>
         </is>
       </c>
     </row>
@@ -54184,17 +55221,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+          <t>ギャルの自転車を直したら懐かれた</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+          <t>タケチケイ（漫画） 生姜寧也（原作）</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第4話-①</t>
+          <t>第3話　ギャルと約束した（前編）</t>
         </is>
       </c>
     </row>
@@ -54204,17 +55241,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
+          <t>魔法少女リリカルなのは EXCEEDS</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
+          <t>都築真紀 川上修一</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第5話</t>
+          <t>第１４話①</t>
         </is>
       </c>
     </row>
@@ -54224,17 +55261,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
+          <t>俺は星間国家の悪徳領主！</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
+          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第66話　扉の先へ</t>
+          <t>第49話　最高に無駄だろう!?</t>
         </is>
       </c>
     </row>
@@ -54244,17 +55281,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>拷問191</t>
+          <t>第90話 竜牙、漆黒を駆ける!!</t>
         </is>
       </c>
     </row>
@@ -54264,17 +55301,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+          <t>六志麻あさ 業務用餅 kisui</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第10話-1</t>
+          <t>第９０話</t>
         </is>
       </c>
     </row>
@@ -54284,17 +55321,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
+          <t>セレビィ量産型(著者)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第4話</t>
+          <t>第28.5話</t>
         </is>
       </c>
     </row>
@@ -54304,17 +55341,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>FUNA 東西 モトエ恵介</t>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第131話 第2回異世界懇談会［その②］</t>
+          <t>第24話④</t>
         </is>
       </c>
     </row>
@@ -54324,17 +55361,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>描けないのでヤってみた</t>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>逢上おかき(著者)</t>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第3話</t>
+          <t>EP.28①</t>
         </is>
       </c>
     </row>
@@ -54344,17 +55381,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>KAKERU</t>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第78話「ケンタウロス」（前半）</t>
+          <t>第8話(1)</t>
         </is>
       </c>
     </row>
@@ -54364,17 +55401,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>バーサス</t>
+          <t>ライブダンジョン！</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>休載イラスト「退場魔王」</t>
+          <t>第98話前半</t>
         </is>
       </c>
     </row>

</xml_diff>